<commit_message>
Next good build is still in progress, for now, this is a update for people to observe and work off
</commit_message>
<xml_diff>
--- a/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
+++ b/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damon\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02761766-1310-4838-8056-26512F17A207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EA7AD5-9B41-4283-BCB9-B6339B638926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="150">
   <si>
     <t>Dialogue Enter</t>
   </si>
@@ -484,6 +484,12 @@
   </si>
   <si>
     <t>Hmm, well we have some Bleeding Grapes back at the Space Station you can have some of those.</t>
+  </si>
+  <si>
+    <t>Restart</t>
+  </si>
+  <si>
+    <t>Exit</t>
   </si>
 </sst>
 </file>
@@ -4811,9 +4817,7 @@
       <c r="H63" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="I63" s="1" t="s">
-        <v>70</v>
-      </c>
+      <c r="I63" s="1"/>
       <c r="J63" s="1" t="s">
         <v>13</v>
       </c>
@@ -4823,17 +4827,25 @@
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
       <c r="N63" s="1"/>
-      <c r="O63" s="7"/>
+      <c r="O63" s="7" t="s">
+        <v>148</v>
+      </c>
       <c r="P63" s="7"/>
       <c r="Q63" s="7"/>
-      <c r="R63" s="7"/>
+      <c r="R63" s="7" t="s">
+        <v>70</v>
+      </c>
       <c r="S63" s="7"/>
       <c r="T63" s="7"/>
       <c r="U63" s="7"/>
-      <c r="V63" s="7"/>
+      <c r="V63" s="7" t="s">
+        <v>149</v>
+      </c>
       <c r="W63" s="7"/>
       <c r="X63" s="7"/>
-      <c r="Y63" s="7"/>
+      <c r="Y63" s="7" t="s">
+        <v>149</v>
+      </c>
       <c r="Z63" s="7"/>
       <c r="AA63" s="7"/>
       <c r="AB63" s="7"/>

</xml_diff>

<commit_message>
Telelmetry data is now setup, the Tutorial Script is also added to the spreadsheet
</commit_message>
<xml_diff>
--- a/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
+++ b/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damon\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\papadoal\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EA7AD5-9B41-4283-BCB9-B6339B638926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB375D9-647B-4BB0-9F58-31BE6DB42B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="201">
   <si>
     <t>Dialogue Enter</t>
   </si>
@@ -490,13 +490,166 @@
   </si>
   <si>
     <t>Exit</t>
+  </si>
+  <si>
+    <t>Tutorial</t>
+  </si>
+  <si>
+    <t>Your eyes have not had a chance to rest since you’ve boarded the ship. Even as you stir from your sleep, a cacophony of bright oranges assault your vision, only interrupted by an errant shock of white or earthy brown.</t>
+  </si>
+  <si>
+    <t>Your feet hover over the floating edge of your bed, the quiet whishing of your R00mbotTM vacuuming softly under your bed threatening to lull you back to sleep.</t>
+  </si>
+  <si>
+    <t>The soft carpeted flooring as you stand and stare at the stars growing ever distant out from your large circular window and sigh.</t>
+  </si>
+  <si>
+    <t>The carpet continues into the hallway, though lines lead those less experienced with the ship to its various sections and amenities.</t>
+  </si>
+  <si>
+    <t>The Diplomatic Liner-A1LYU80V-8469 has been your home of choice for years now.  You have grown so close to her that the two of you share a call-sign, Amore.</t>
+  </si>
+  <si>
+    <t>As you head to your destination you are stopped by a group of large hulking masses of misshapen clay as they cross your path.</t>
+  </si>
+  <si>
+    <t>Ignoring you, they stomp off in a hurry, one of the ship's many robots follows them, cleaning off the dust and chipping in its path.</t>
+  </si>
+  <si>
+    <t>The softly blinking lights of the bridge copy the shining stars out the massive bow-facing windows. A number of figures are waiting for you in the command center, your new crew if you had to hazard a guess.</t>
+  </si>
+  <si>
+    <t>To your left a woman is rapping her knuckles against one of the consoles, swaying nervously to the knocks.</t>
+  </si>
+  <si>
+    <t>Next to her another woman is staring at a tablet, leaning against the same console, a series of yellow holographic rings emanating from one of her eyes.</t>
+  </si>
+  <si>
+    <t>Down further into the bridge you see a person asleep in an egg-shaped chair, one of those clay beasts hunkered over them.</t>
+  </si>
+  <si>
+    <t>In fact a number of these creatures are found all through the lower levels of the bridge, attending to odd tasks and shuffling about with purpose.</t>
+  </si>
+  <si>
+    <t>Lastly to your left you find a strange Lepidopteran creature, clipboard in hand, looking at you attentively.</t>
+  </si>
+  <si>
+    <t>Before you have a chance to greet them, the lights flash briefly to signal an incoming message.</t>
+  </si>
+  <si>
+    <t>From the center of the room a hologram of your commanding officer is displayed, their blue-light form flickering periodically.</t>
+  </si>
+  <si>
+    <t>Ah, I see you’re all here.</t>
+  </si>
+  <si>
+    <t>Their voice crackles with the instability of ultra-long range transmission</t>
+  </si>
+  <si>
+    <t>Captain, the fight against the heathen steLLarITM corporation is set to open on a new frontier.</t>
+  </si>
+  <si>
+    <t>We must join forces to win in the free market of ideas and also violence.</t>
+  </si>
+  <si>
+    <t>We AstranautsTM must quickly shore up some support in this star system to ensure the local populace is receptive to our products and our values of freedom and commerce.</t>
+  </si>
+  <si>
+    <t>The commander salutes with pride, but only you and the winged creature actually join him.</t>
+  </si>
+  <si>
+    <t>I am familiar with your, uhm-</t>
+  </si>
+  <si>
+    <t>If someone's face could turn red over the blue-tinged display of a hologram, you would swear your captain was blushing vigorously.</t>
+  </si>
+  <si>
+    <t>You are cleared to use any and all methods to enter these xenoform societies and bring them into the welcoming bosom of AstratechTM corporation and the wider sacred AstraTM conglomerate.</t>
+  </si>
+  <si>
+    <t>-specialized maneuvers, Captain Amore of the Amore.</t>
+  </si>
+  <si>
+    <t>In their infinite generosity, our corporate sponsors granted the use of a small crew to help you help out on your mission</t>
+  </si>
+  <si>
+    <t>(Because they aren’t eligible for union membership)</t>
+  </si>
+  <si>
+    <t>The first of which is Pu Ai, an excellent explorer and xenobiologist.</t>
+  </si>
+  <si>
+    <t>(as a recipient of a scholarship program she is an indentured citemployee until she pays of her student loan debt)</t>
+  </si>
+  <si>
+    <t>The anxious woman at your left looks up to you and smiles, though you wouldn’t call it reassuring.</t>
+  </si>
+  <si>
+    <t>Joining her is her longtime companion, Shira Rahman. A brilliant transfer from our competitally, AstraSystemsTM, her cyborg enhancements make her a brilliant mind to have on any expedition.</t>
+  </si>
+  <si>
+    <t>(and fortunately technically not fully an organic or inorganic mind and therefore not eligible for coverage by either guild)</t>
+  </si>
+  <si>
+    <t>The other woman does not look up from her tablet.</t>
+  </si>
+  <si>
+    <t>We also have Judah Ben Loew and his group of glamim to meet any labour or mystical needs you may have.</t>
+  </si>
+  <si>
+    <t> (His ability to provide great quantities of unpaid labour has earned the ire of workers with rights everywhere)</t>
+  </si>
+  <si>
+    <t>The golem watching over their creator’s sleeping form waves at you.</t>
+  </si>
+  <si>
+    <t>Lastly, Marie Posa, a LepidJanussian, is here to serve you as your ship's communications officer.</t>
+  </si>
+  <si>
+    <t>(Do not let her get tired or you will meet her worse half and learn why her species is considered too volatile for solidarity with other citemployees)</t>
+  </si>
+  <si>
+    <t>The one non-human in the room nods at you, a sign of deference you believe, as her face is otherwise inscrutable.</t>
+  </si>
+  <si>
+    <t>Now I’ve been ordered to test your ability to command your crew members after your last mut-, incident kerfuffle. Please select Judah and Shira to assist you in this training exercise.</t>
+  </si>
+  <si>
+    <t>Exercise</t>
+  </si>
+  <si>
+    <t>Wonderful!</t>
+  </si>
+  <si>
+    <t>The captain’s tone is overly saccharine and rigid as though reading from a script.</t>
+  </si>
+  <si>
+    <t>Now use their combined brain power to solve this simple logic puzzle</t>
+  </si>
+  <si>
+    <t>You're amazing. Now use Shira’s Science knowledge to help defeat the negative thoughts in this mental exercise.</t>
+  </si>
+  <si>
+    <t>Now remember even though your crew members are third class citemployees and are therefore exempt from traditional labour laws, overuse of your employees can lead to a depreciation of value for your human resources.</t>
+  </si>
+  <si>
+    <t>Wow, great job, me and other surrogate parental figures are proud of you.</t>
+  </si>
+  <si>
+    <t>With the completion of this module you are now recertified to undertake missions for the glorious AstraTM conglomerate. Good luck Captain!</t>
+  </si>
+  <si>
+    <t>You see the commander fiddle with something on his desk. Quietly you can make out. “Astra’sTM Excellent Value, that’s over. How do I turn this off?”</t>
+  </si>
+  <si>
+    <t>Your commander’s face disappears from the bridge and your crew members wait on your word. You have your orders.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,7 +728,41 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="47">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1063,50 +1250,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM87" totalsRowShown="0" dataDxfId="42">
-  <autoFilter ref="B5:AM87" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM132" totalsRowShown="0" dataDxfId="46">
+  <autoFilter ref="B5:AM132" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:AM20">
     <sortCondition ref="B5:B20"/>
   </sortState>
   <tableColumns count="38">
-    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="41"/>
-    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="39"/>
-    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="38"/>
-    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="32"/>
-    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="31"/>
-    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="30"/>
-    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="28"/>
-    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="27"/>
-    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="26"/>
-    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="25"/>
-    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="24"/>
-    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="23"/>
-    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="22"/>
-    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="21"/>
-    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="20"/>
-    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="19"/>
-    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="18"/>
-    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="17"/>
-    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="16"/>
-    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="15"/>
-    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="14"/>
-    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="13"/>
-    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="12"/>
-    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="11"/>
-    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="10"/>
-    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="9"/>
-    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="8"/>
-    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="7"/>
-    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="6"/>
-    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="5"/>
-    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="4"/>
+    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="45"/>
+    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="43"/>
+    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="42"/>
+    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="36"/>
+    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="35"/>
+    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="34"/>
+    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="32"/>
+    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="31"/>
+    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="30"/>
+    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="29"/>
+    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="28"/>
+    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="27"/>
+    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="26"/>
+    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="25"/>
+    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="24"/>
+    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="23"/>
+    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="22"/>
+    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="21"/>
+    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="20"/>
+    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="19"/>
+    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="18"/>
+    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="17"/>
+    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="16"/>
+    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="15"/>
+    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="14"/>
+    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="13"/>
+    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="12"/>
+    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="11"/>
+    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="10"/>
+    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="9"/>
+    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1462,39 +1649,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AD6004-D6D5-49E8-98E5-3900A70D687C}">
-  <dimension ref="B4:AM87"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B4:AM132"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" customWidth="1"/>
-    <col min="4" max="7" width="14.77734375" customWidth="1"/>
-    <col min="8" max="8" width="60.77734375" customWidth="1"/>
-    <col min="9" max="10" width="14.77734375" customWidth="1"/>
-    <col min="11" max="14" width="15.77734375" customWidth="1"/>
-    <col min="15" max="15" width="20.77734375" customWidth="1"/>
-    <col min="16" max="16" width="18.77734375" customWidth="1"/>
-    <col min="17" max="17" width="15.77734375" customWidth="1"/>
-    <col min="18" max="18" width="14.77734375" customWidth="1"/>
-    <col min="19" max="21" width="15.77734375" customWidth="1"/>
-    <col min="22" max="22" width="20.77734375" customWidth="1"/>
-    <col min="23" max="23" width="18.77734375" customWidth="1"/>
-    <col min="24" max="24" width="15.77734375" customWidth="1"/>
-    <col min="25" max="25" width="14.77734375" customWidth="1"/>
-    <col min="26" max="28" width="15.77734375" customWidth="1"/>
-    <col min="29" max="29" width="20.77734375" customWidth="1"/>
-    <col min="30" max="30" width="18.77734375" customWidth="1"/>
-    <col min="31" max="31" width="15.77734375" customWidth="1"/>
-    <col min="32" max="32" width="14.77734375" customWidth="1"/>
-    <col min="33" max="35" width="15.77734375" customWidth="1"/>
-    <col min="36" max="36" width="20.77734375" customWidth="1"/>
-    <col min="37" max="37" width="18.77734375" customWidth="1"/>
-    <col min="38" max="38" width="15.77734375" customWidth="1"/>
-    <col min="39" max="39" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="8.875" customWidth="1"/>
+    <col min="2" max="2" width="8.625" customWidth="1"/>
+    <col min="3" max="3" width="15.75" customWidth="1"/>
+    <col min="4" max="7" width="14.75" customWidth="1"/>
+    <col min="8" max="8" width="60.75" customWidth="1"/>
+    <col min="9" max="10" width="14.75" customWidth="1"/>
+    <col min="11" max="14" width="15.75" customWidth="1"/>
+    <col min="15" max="15" width="20.75" customWidth="1"/>
+    <col min="16" max="16" width="18.75" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.75" customWidth="1"/>
+    <col min="19" max="21" width="15.75" customWidth="1"/>
+    <col min="22" max="22" width="20.75" customWidth="1"/>
+    <col min="23" max="23" width="18.75" customWidth="1"/>
+    <col min="24" max="24" width="15.75" customWidth="1"/>
+    <col min="25" max="25" width="14.75" customWidth="1"/>
+    <col min="26" max="28" width="15.75" customWidth="1"/>
+    <col min="29" max="29" width="20.75" customWidth="1"/>
+    <col min="30" max="30" width="18.75" customWidth="1"/>
+    <col min="31" max="31" width="15.75" customWidth="1"/>
+    <col min="32" max="32" width="14.75" customWidth="1"/>
+    <col min="33" max="35" width="15.75" customWidth="1"/>
+    <col min="36" max="36" width="20.75" customWidth="1"/>
+    <col min="37" max="37" width="18.75" customWidth="1"/>
+    <col min="38" max="38" width="15.75" customWidth="1"/>
+    <col min="39" max="39" width="14.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:39" ht="88.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:39" ht="88.9" customHeight="1"/>
+    <row r="5" spans="2:39">
       <c r="B5" t="s">
         <v>22</v>
       </c>
@@ -1610,7 +1797,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:39" ht="28.5">
       <c r="B6" s="1">
         <v>0</v>
       </c>
@@ -1664,7 +1851,7 @@
       <c r="AL6" s="7"/>
       <c r="AM6" s="7"/>
     </row>
-    <row r="7" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:39" ht="28.5">
       <c r="B7" s="1">
         <f t="shared" ref="B7:B70" si="0">1+B6</f>
         <v>1</v>
@@ -1719,7 +1906,7 @@
       <c r="AL7" s="7"/>
       <c r="AM7" s="7"/>
     </row>
-    <row r="8" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:39" ht="28.5">
       <c r="B8" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1772,7 +1959,7 @@
       <c r="AL8" s="7"/>
       <c r="AM8" s="7"/>
     </row>
-    <row r="9" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:39" ht="42.75">
       <c r="B9" s="1">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1827,7 +2014,7 @@
       <c r="AL9" s="7"/>
       <c r="AM9" s="7"/>
     </row>
-    <row r="10" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:39" ht="28.5">
       <c r="B10" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1886,7 +2073,7 @@
       <c r="AL10" s="7"/>
       <c r="AM10" s="7"/>
     </row>
-    <row r="11" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:39">
       <c r="B11" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1943,7 +2130,7 @@
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
     </row>
-    <row r="12" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:39" ht="42.75">
       <c r="B12" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1996,7 +2183,7 @@
       <c r="AL12" s="7"/>
       <c r="AM12" s="7"/>
     </row>
-    <row r="13" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:39" ht="28.5">
       <c r="B13" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2049,7 +2236,7 @@
       <c r="AL13" s="7"/>
       <c r="AM13" s="7"/>
     </row>
-    <row r="14" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:39">
       <c r="B14" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2104,7 +2291,7 @@
       <c r="AL14" s="7"/>
       <c r="AM14" s="7"/>
     </row>
-    <row r="15" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:39" ht="28.5">
       <c r="B15" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2169,7 +2356,7 @@
       <c r="AL15" s="7"/>
       <c r="AM15" s="7"/>
     </row>
-    <row r="16" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:39">
       <c r="B16" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2226,7 +2413,7 @@
       <c r="AL16" s="7"/>
       <c r="AM16" s="7"/>
     </row>
-    <row r="17" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:39" ht="28.5">
       <c r="B17" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2281,7 +2468,7 @@
       <c r="AL17" s="7"/>
       <c r="AM17" s="7"/>
     </row>
-    <row r="18" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:39">
       <c r="B18" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2338,7 +2525,7 @@
       <c r="AL18" s="7"/>
       <c r="AM18" s="7"/>
     </row>
-    <row r="19" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:39" ht="28.5">
       <c r="B19" s="1">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2395,7 +2582,7 @@
       <c r="AL19" s="7"/>
       <c r="AM19" s="7"/>
     </row>
-    <row r="20" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:39">
       <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2450,7 +2637,7 @@
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
     </row>
-    <row r="21" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:39">
       <c r="B21" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2503,7 +2690,7 @@
       <c r="AL21" s="7"/>
       <c r="AM21" s="7"/>
     </row>
-    <row r="22" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:39" ht="42.75">
       <c r="B22" s="1">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2556,7 +2743,7 @@
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
     </row>
-    <row r="23" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:39" ht="28.5">
       <c r="B23" s="1">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2609,7 +2796,7 @@
       <c r="AL23" s="7"/>
       <c r="AM23" s="7"/>
     </row>
-    <row r="24" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:39">
       <c r="B24" s="1">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2662,7 +2849,7 @@
       <c r="AL24" s="7"/>
       <c r="AM24" s="7"/>
     </row>
-    <row r="25" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:39" ht="28.5">
       <c r="B25" s="1">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2739,7 +2926,7 @@
       <c r="AL25" s="7"/>
       <c r="AM25" s="7"/>
     </row>
-    <row r="26" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:39">
       <c r="B26" s="1">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2796,7 +2983,7 @@
       <c r="AL26" s="7"/>
       <c r="AM26" s="7"/>
     </row>
-    <row r="27" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:39" ht="28.5">
       <c r="B27" s="1">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2849,7 +3036,7 @@
       <c r="AL27" s="7"/>
       <c r="AM27" s="7"/>
     </row>
-    <row r="28" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:39">
       <c r="B28" s="1">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -2904,7 +3091,7 @@
       <c r="AL28" s="7"/>
       <c r="AM28" s="7"/>
     </row>
-    <row r="29" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:39">
       <c r="B29" s="1">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -2959,7 +3146,7 @@
       <c r="AL29" s="7"/>
       <c r="AM29" s="7"/>
     </row>
-    <row r="30" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:39">
       <c r="B30" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3014,7 +3201,7 @@
       <c r="AL30" s="7"/>
       <c r="AM30" s="7"/>
     </row>
-    <row r="31" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:39">
       <c r="B31" s="1">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3069,7 +3256,7 @@
       <c r="AL31" s="7"/>
       <c r="AM31" s="7"/>
     </row>
-    <row r="32" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:39">
       <c r="B32" s="1">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3122,7 +3309,7 @@
       <c r="AL32" s="7"/>
       <c r="AM32" s="7"/>
     </row>
-    <row r="33" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:39">
       <c r="B33" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3177,7 +3364,7 @@
       <c r="AL33" s="7"/>
       <c r="AM33" s="7"/>
     </row>
-    <row r="34" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:39">
       <c r="B34" s="1">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3232,7 +3419,7 @@
       <c r="AL34" s="7"/>
       <c r="AM34" s="7"/>
     </row>
-    <row r="35" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:39" ht="28.5">
       <c r="B35" s="1">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3287,7 +3474,7 @@
       <c r="AL35" s="7"/>
       <c r="AM35" s="7"/>
     </row>
-    <row r="36" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:39">
       <c r="B36" s="1">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3340,7 +3527,7 @@
       <c r="AL36" s="7"/>
       <c r="AM36" s="7"/>
     </row>
-    <row r="37" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:39">
       <c r="B37" s="1">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3395,7 +3582,7 @@
       <c r="AL37" s="7"/>
       <c r="AM37" s="7"/>
     </row>
-    <row r="38" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:39">
       <c r="B38" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3448,7 +3635,7 @@
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
     </row>
-    <row r="39" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:39">
       <c r="B39" s="1">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3503,7 +3690,7 @@
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
     </row>
-    <row r="40" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:39" ht="28.5">
       <c r="B40" s="1">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3556,7 +3743,7 @@
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
     </row>
-    <row r="41" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:39" ht="28.5">
       <c r="B41" s="1">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3609,7 +3796,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
     </row>
-    <row r="42" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:39" ht="28.5">
       <c r="B42" s="1">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3664,7 +3851,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
     </row>
-    <row r="43" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:39">
       <c r="B43" s="1">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3717,7 +3904,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
     </row>
-    <row r="44" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:39">
       <c r="B44" s="1">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3786,7 +3973,7 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
     </row>
-    <row r="45" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:39">
       <c r="B45" s="1">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3843,7 +4030,7 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
     </row>
-    <row r="46" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:39" ht="28.5">
       <c r="B46" s="1">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -3898,7 +4085,7 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
     </row>
-    <row r="47" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:39" ht="42.75">
       <c r="B47" s="1">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -3953,7 +4140,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
     </row>
-    <row r="48" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:39">
       <c r="B48" s="1">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -4008,7 +4195,7 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
     </row>
-    <row r="49" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:39" ht="28.5">
       <c r="B49" s="1">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -4063,7 +4250,7 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
     </row>
-    <row r="50" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:39" ht="42.75">
       <c r="B50" s="1">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -4118,7 +4305,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
     </row>
-    <row r="51" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:39" ht="28.5">
       <c r="B51" s="1">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -4171,7 +4358,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
     </row>
-    <row r="52" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:39">
       <c r="B52" s="1">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -4226,7 +4413,7 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
     </row>
-    <row r="53" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:39" ht="28.5">
       <c r="B53" s="1">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -4279,7 +4466,7 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
     </row>
-    <row r="54" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:39" ht="28.5">
       <c r="B54" s="1">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -4334,7 +4521,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
     </row>
-    <row r="55" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:39" ht="42.75">
       <c r="B55" s="1">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -4387,7 +4574,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
     </row>
-    <row r="56" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:39" ht="28.5">
       <c r="B56" s="1">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -4464,7 +4651,7 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
     </row>
-    <row r="57" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:39" ht="28.5">
       <c r="B57" s="1">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -4519,7 +4706,7 @@
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
     </row>
-    <row r="58" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:39">
       <c r="B58" s="1">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -4574,7 +4761,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
     </row>
-    <row r="59" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:39">
       <c r="B59" s="1">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -4629,7 +4816,7 @@
       <c r="AL59" s="7"/>
       <c r="AM59" s="7"/>
     </row>
-    <row r="60" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:39">
       <c r="B60" s="1">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -4684,7 +4871,7 @@
       <c r="AL60" s="7"/>
       <c r="AM60" s="7"/>
     </row>
-    <row r="61" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:39">
       <c r="B61" s="1">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -4741,7 +4928,7 @@
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
     </row>
-    <row r="62" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:39">
       <c r="B62" s="1">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -4798,7 +4985,7 @@
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
     </row>
-    <row r="63" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:39">
       <c r="B63" s="1">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -4861,7 +5048,7 @@
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
     </row>
-    <row r="64" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:39">
       <c r="B64" s="1">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -4912,7 +5099,7 @@
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
     </row>
-    <row r="65" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:39" ht="42.75">
       <c r="B65" s="1">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -4925,8 +5112,12 @@
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
-      <c r="G65" s="1"/>
-      <c r="H65" s="8"/>
+      <c r="G65" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H65" s="8" t="s">
+        <v>151</v>
+      </c>
       <c r="I65" s="1"/>
       <c r="J65" s="1" t="s">
         <v>13</v>
@@ -4963,7 +5154,7 @@
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
     </row>
-    <row r="66" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:39" ht="42.75">
       <c r="B66" s="1">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -4977,7 +5168,9 @@
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
-      <c r="H66" s="8"/>
+      <c r="H66" s="8" t="s">
+        <v>152</v>
+      </c>
       <c r="I66" s="1"/>
       <c r="J66" s="1" t="s">
         <v>13</v>
@@ -5014,7 +5207,7 @@
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
     </row>
-    <row r="67" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:39" ht="28.5">
       <c r="B67" s="1">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -5028,7 +5221,9 @@
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
-      <c r="H67" s="8"/>
+      <c r="H67" s="8" t="s">
+        <v>153</v>
+      </c>
       <c r="I67" s="1"/>
       <c r="J67" s="1" t="s">
         <v>13</v>
@@ -5065,7 +5260,7 @@
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
     </row>
-    <row r="68" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:39" ht="28.5">
       <c r="B68" s="1">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -5079,7 +5274,9 @@
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
-      <c r="H68" s="8"/>
+      <c r="H68" s="8" t="s">
+        <v>154</v>
+      </c>
       <c r="I68" s="1"/>
       <c r="J68" s="1" t="s">
         <v>13</v>
@@ -5116,7 +5313,7 @@
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
     </row>
-    <row r="69" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:39" ht="42.75">
       <c r="B69" s="1">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -5130,7 +5327,9 @@
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
-      <c r="H69" s="8"/>
+      <c r="H69" s="8" t="s">
+        <v>155</v>
+      </c>
       <c r="I69" s="1"/>
       <c r="J69" s="1" t="s">
         <v>13</v>
@@ -5167,7 +5366,7 @@
       <c r="AL69" s="7"/>
       <c r="AM69" s="7"/>
     </row>
-    <row r="70" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:39" ht="28.5">
       <c r="B70" s="1">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -5181,7 +5380,9 @@
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
-      <c r="H70" s="8"/>
+      <c r="H70" s="8" t="s">
+        <v>156</v>
+      </c>
       <c r="I70" s="1"/>
       <c r="J70" s="1" t="s">
         <v>13</v>
@@ -5218,9 +5419,9 @@
       <c r="AL70" s="7"/>
       <c r="AM70" s="7"/>
     </row>
-    <row r="71" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:39" ht="28.5">
       <c r="B71" s="1">
-        <f t="shared" ref="B71:B87" si="1">1+B70</f>
+        <f t="shared" ref="B71:B132" si="1">1+B70</f>
         <v>65</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -5232,7 +5433,9 @@
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
-      <c r="H71" s="8"/>
+      <c r="H71" s="8" t="s">
+        <v>157</v>
+      </c>
       <c r="I71" s="1"/>
       <c r="J71" s="1" t="s">
         <v>13</v>
@@ -5269,7 +5472,7 @@
       <c r="AL71" s="7"/>
       <c r="AM71" s="7"/>
     </row>
-    <row r="72" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:39" ht="42.75">
       <c r="B72" s="1">
         <f t="shared" si="1"/>
         <v>66</v>
@@ -5283,7 +5486,9 @@
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
-      <c r="H72" s="8"/>
+      <c r="H72" s="8" t="s">
+        <v>158</v>
+      </c>
       <c r="I72" s="1"/>
       <c r="J72" s="1" t="s">
         <v>13</v>
@@ -5320,7 +5525,7 @@
       <c r="AL72" s="7"/>
       <c r="AM72" s="7"/>
     </row>
-    <row r="73" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:39" ht="28.5">
       <c r="B73" s="1">
         <f t="shared" si="1"/>
         <v>67</v>
@@ -5334,7 +5539,9 @@
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
-      <c r="H73" s="8"/>
+      <c r="H73" s="8" t="s">
+        <v>159</v>
+      </c>
       <c r="I73" s="1"/>
       <c r="J73" s="1" t="s">
         <v>13</v>
@@ -5371,7 +5578,7 @@
       <c r="AL73" s="7"/>
       <c r="AM73" s="7"/>
     </row>
-    <row r="74" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:39" ht="42.75">
       <c r="B74" s="1">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -5385,7 +5592,9 @@
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
-      <c r="H74" s="8"/>
+      <c r="H74" s="8" t="s">
+        <v>160</v>
+      </c>
       <c r="I74" s="1"/>
       <c r="J74" s="1" t="s">
         <v>13</v>
@@ -5422,7 +5631,7 @@
       <c r="AL74" s="7"/>
       <c r="AM74" s="7"/>
     </row>
-    <row r="75" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:39" ht="28.5">
       <c r="B75" s="1">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -5436,7 +5645,9 @@
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
-      <c r="H75" s="8"/>
+      <c r="H75" s="8" t="s">
+        <v>161</v>
+      </c>
       <c r="I75" s="1"/>
       <c r="J75" s="1" t="s">
         <v>13</v>
@@ -5473,7 +5684,7 @@
       <c r="AL75" s="7"/>
       <c r="AM75" s="7"/>
     </row>
-    <row r="76" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:39" ht="28.5">
       <c r="B76" s="1">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -5487,7 +5698,9 @@
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
-      <c r="H76" s="8"/>
+      <c r="H76" s="8" t="s">
+        <v>162</v>
+      </c>
       <c r="I76" s="1"/>
       <c r="J76" s="1" t="s">
         <v>13</v>
@@ -5524,7 +5737,7 @@
       <c r="AL76" s="7"/>
       <c r="AM76" s="7"/>
     </row>
-    <row r="77" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:39" ht="28.5">
       <c r="B77" s="1">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -5538,7 +5751,9 @@
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
-      <c r="H77" s="8"/>
+      <c r="H77" s="8" t="s">
+        <v>163</v>
+      </c>
       <c r="I77" s="1"/>
       <c r="J77" s="1" t="s">
         <v>13</v>
@@ -5575,7 +5790,7 @@
       <c r="AL77" s="7"/>
       <c r="AM77" s="7"/>
     </row>
-    <row r="78" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:39" ht="28.5">
       <c r="B78" s="1">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -5589,7 +5804,9 @@
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
-      <c r="H78" s="8"/>
+      <c r="H78" s="8" t="s">
+        <v>164</v>
+      </c>
       <c r="I78" s="1"/>
       <c r="J78" s="1" t="s">
         <v>13</v>
@@ -5626,7 +5843,7 @@
       <c r="AL78" s="7"/>
       <c r="AM78" s="7"/>
     </row>
-    <row r="79" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:39" ht="28.5">
       <c r="B79" s="1">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -5640,7 +5857,9 @@
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
-      <c r="H79" s="8"/>
+      <c r="H79" s="8" t="s">
+        <v>165</v>
+      </c>
       <c r="I79" s="1"/>
       <c r="J79" s="1" t="s">
         <v>13</v>
@@ -5677,7 +5896,7 @@
       <c r="AL79" s="7"/>
       <c r="AM79" s="7"/>
     </row>
-    <row r="80" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:39">
       <c r="B80" s="1">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -5691,7 +5910,9 @@
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
-      <c r="H80" s="8"/>
+      <c r="H80" s="8" t="s">
+        <v>166</v>
+      </c>
       <c r="I80" s="1"/>
       <c r="J80" s="1" t="s">
         <v>13</v>
@@ -5728,7 +5949,7 @@
       <c r="AL80" s="7"/>
       <c r="AM80" s="7"/>
     </row>
-    <row r="81" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:39">
       <c r="B81" s="1">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -5742,7 +5963,9 @@
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
-      <c r="H81" s="8"/>
+      <c r="H81" s="8" t="s">
+        <v>167</v>
+      </c>
       <c r="I81" s="1"/>
       <c r="J81" s="1" t="s">
         <v>13</v>
@@ -5779,7 +6002,7 @@
       <c r="AL81" s="7"/>
       <c r="AM81" s="7"/>
     </row>
-    <row r="82" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:39" ht="28.5">
       <c r="B82" s="1">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -5793,7 +6016,9 @@
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
-      <c r="H82" s="8"/>
+      <c r="H82" s="8" t="s">
+        <v>168</v>
+      </c>
       <c r="I82" s="1"/>
       <c r="J82" s="1" t="s">
         <v>13</v>
@@ -5830,7 +6055,7 @@
       <c r="AL82" s="7"/>
       <c r="AM82" s="7"/>
     </row>
-    <row r="83" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:39" ht="42.75">
       <c r="B83" s="1">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -5844,7 +6069,9 @@
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
-      <c r="H83" s="8"/>
+      <c r="H83" s="8" t="s">
+        <v>170</v>
+      </c>
       <c r="I83" s="1"/>
       <c r="J83" s="1" t="s">
         <v>13</v>
@@ -5881,7 +6108,7 @@
       <c r="AL83" s="7"/>
       <c r="AM83" s="7"/>
     </row>
-    <row r="84" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:39">
       <c r="B84" s="1">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -5895,7 +6122,9 @@
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
-      <c r="H84" s="8"/>
+      <c r="H84" s="8" t="s">
+        <v>169</v>
+      </c>
       <c r="I84" s="1"/>
       <c r="J84" s="1" t="s">
         <v>13</v>
@@ -5932,7 +6161,7 @@
       <c r="AL84" s="7"/>
       <c r="AM84" s="7"/>
     </row>
-    <row r="85" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:39" ht="28.5">
       <c r="B85" s="1">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -5946,7 +6175,9 @@
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
-      <c r="H85" s="8"/>
+      <c r="H85" s="8" t="s">
+        <v>171</v>
+      </c>
       <c r="I85" s="1"/>
       <c r="J85" s="1" t="s">
         <v>13</v>
@@ -5983,7 +6214,7 @@
       <c r="AL85" s="7"/>
       <c r="AM85" s="7"/>
     </row>
-    <row r="86" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:39">
       <c r="B86" s="1">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -5997,7 +6228,9 @@
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
-      <c r="H86" s="8"/>
+      <c r="H86" s="8" t="s">
+        <v>172</v>
+      </c>
       <c r="I86" s="1"/>
       <c r="J86" s="1" t="s">
         <v>13</v>
@@ -6034,7 +6267,7 @@
       <c r="AL86" s="7"/>
       <c r="AM86" s="7"/>
     </row>
-    <row r="87" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:39" ht="28.5">
       <c r="B87" s="1">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -6048,7 +6281,9 @@
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
-      <c r="H87" s="8"/>
+      <c r="H87" s="8" t="s">
+        <v>173</v>
+      </c>
       <c r="I87" s="1"/>
       <c r="J87" s="1" t="s">
         <v>13</v>
@@ -6085,9 +6320,2004 @@
       <c r="AL87" s="7"/>
       <c r="AM87" s="7"/>
     </row>
+    <row r="88" spans="2:39">
+      <c r="B88" s="1">
+        <f t="shared" si="1"/>
+        <v>82</v>
+      </c>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="I88" s="1"/>
+      <c r="J88" s="1"/>
+      <c r="K88" s="1"/>
+      <c r="L88" s="1"/>
+      <c r="M88" s="1"/>
+      <c r="N88" s="1"/>
+      <c r="O88" s="7"/>
+      <c r="P88" s="7"/>
+      <c r="Q88" s="7"/>
+      <c r="R88" s="7"/>
+      <c r="S88" s="7"/>
+      <c r="T88" s="7"/>
+      <c r="U88" s="7"/>
+      <c r="V88" s="7"/>
+      <c r="W88" s="7"/>
+      <c r="X88" s="7"/>
+      <c r="Y88" s="7"/>
+      <c r="Z88" s="7"/>
+      <c r="AA88" s="7"/>
+      <c r="AB88" s="7"/>
+      <c r="AC88" s="7"/>
+      <c r="AD88" s="7"/>
+      <c r="AE88" s="7"/>
+      <c r="AF88" s="7"/>
+      <c r="AG88" s="7"/>
+      <c r="AH88" s="7"/>
+      <c r="AI88" s="7"/>
+      <c r="AJ88" s="7"/>
+      <c r="AK88" s="7"/>
+      <c r="AL88" s="7"/>
+      <c r="AM88" s="7"/>
+    </row>
+    <row r="89" spans="2:39" ht="42.75">
+      <c r="B89" s="1">
+        <f t="shared" si="1"/>
+        <v>83</v>
+      </c>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="I89" s="1"/>
+      <c r="J89" s="1"/>
+      <c r="K89" s="1"/>
+      <c r="L89" s="1"/>
+      <c r="M89" s="1"/>
+      <c r="N89" s="1"/>
+      <c r="O89" s="7"/>
+      <c r="P89" s="7"/>
+      <c r="Q89" s="7"/>
+      <c r="R89" s="7"/>
+      <c r="S89" s="7"/>
+      <c r="T89" s="7"/>
+      <c r="U89" s="7"/>
+      <c r="V89" s="7"/>
+      <c r="W89" s="7"/>
+      <c r="X89" s="7"/>
+      <c r="Y89" s="7"/>
+      <c r="Z89" s="7"/>
+      <c r="AA89" s="7"/>
+      <c r="AB89" s="7"/>
+      <c r="AC89" s="7"/>
+      <c r="AD89" s="7"/>
+      <c r="AE89" s="7"/>
+      <c r="AF89" s="7"/>
+      <c r="AG89" s="7"/>
+      <c r="AH89" s="7"/>
+      <c r="AI89" s="7"/>
+      <c r="AJ89" s="7"/>
+      <c r="AK89" s="7"/>
+      <c r="AL89" s="7"/>
+      <c r="AM89" s="7"/>
+    </row>
+    <row r="90" spans="2:39" ht="28.5">
+      <c r="B90" s="1">
+        <f t="shared" si="1"/>
+        <v>84</v>
+      </c>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="I90" s="1"/>
+      <c r="J90" s="1"/>
+      <c r="K90" s="1"/>
+      <c r="L90" s="1"/>
+      <c r="M90" s="1"/>
+      <c r="N90" s="1"/>
+      <c r="O90" s="7"/>
+      <c r="P90" s="7"/>
+      <c r="Q90" s="7"/>
+      <c r="R90" s="7"/>
+      <c r="S90" s="7"/>
+      <c r="T90" s="7"/>
+      <c r="U90" s="7"/>
+      <c r="V90" s="7"/>
+      <c r="W90" s="7"/>
+      <c r="X90" s="7"/>
+      <c r="Y90" s="7"/>
+      <c r="Z90" s="7"/>
+      <c r="AA90" s="7"/>
+      <c r="AB90" s="7"/>
+      <c r="AC90" s="7"/>
+      <c r="AD90" s="7"/>
+      <c r="AE90" s="7"/>
+      <c r="AF90" s="7"/>
+      <c r="AG90" s="7"/>
+      <c r="AH90" s="7"/>
+      <c r="AI90" s="7"/>
+      <c r="AJ90" s="7"/>
+      <c r="AK90" s="7"/>
+      <c r="AL90" s="7"/>
+      <c r="AM90" s="7"/>
+    </row>
+    <row r="91" spans="2:39">
+      <c r="B91" s="1">
+        <f t="shared" si="1"/>
+        <v>85</v>
+      </c>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="I91" s="1"/>
+      <c r="J91" s="1"/>
+      <c r="K91" s="1"/>
+      <c r="L91" s="1"/>
+      <c r="M91" s="1"/>
+      <c r="N91" s="1"/>
+      <c r="O91" s="7"/>
+      <c r="P91" s="7"/>
+      <c r="Q91" s="7"/>
+      <c r="R91" s="7"/>
+      <c r="S91" s="7"/>
+      <c r="T91" s="7"/>
+      <c r="U91" s="7"/>
+      <c r="V91" s="7"/>
+      <c r="W91" s="7"/>
+      <c r="X91" s="7"/>
+      <c r="Y91" s="7"/>
+      <c r="Z91" s="7"/>
+      <c r="AA91" s="7"/>
+      <c r="AB91" s="7"/>
+      <c r="AC91" s="7"/>
+      <c r="AD91" s="7"/>
+      <c r="AE91" s="7"/>
+      <c r="AF91" s="7"/>
+      <c r="AG91" s="7"/>
+      <c r="AH91" s="7"/>
+      <c r="AI91" s="7"/>
+      <c r="AJ91" s="7"/>
+      <c r="AK91" s="7"/>
+      <c r="AL91" s="7"/>
+      <c r="AM91" s="7"/>
+    </row>
+    <row r="92" spans="2:39">
+      <c r="B92" s="1">
+        <f t="shared" si="1"/>
+        <v>86</v>
+      </c>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+      <c r="K92" s="1"/>
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
+      <c r="N92" s="1"/>
+      <c r="O92" s="7"/>
+      <c r="P92" s="7"/>
+      <c r="Q92" s="7"/>
+      <c r="R92" s="7"/>
+      <c r="S92" s="7"/>
+      <c r="T92" s="7"/>
+      <c r="U92" s="7"/>
+      <c r="V92" s="7"/>
+      <c r="W92" s="7"/>
+      <c r="X92" s="7"/>
+      <c r="Y92" s="7"/>
+      <c r="Z92" s="7"/>
+      <c r="AA92" s="7"/>
+      <c r="AB92" s="7"/>
+      <c r="AC92" s="7"/>
+      <c r="AD92" s="7"/>
+      <c r="AE92" s="7"/>
+      <c r="AF92" s="7"/>
+      <c r="AG92" s="7"/>
+      <c r="AH92" s="7"/>
+      <c r="AI92" s="7"/>
+      <c r="AJ92" s="7"/>
+      <c r="AK92" s="7"/>
+      <c r="AL92" s="7"/>
+      <c r="AM92" s="7"/>
+    </row>
+    <row r="93" spans="2:39" ht="28.5">
+      <c r="B93" s="1">
+        <f t="shared" si="1"/>
+        <v>87</v>
+      </c>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="I93" s="1"/>
+      <c r="J93" s="1"/>
+      <c r="K93" s="1"/>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+      <c r="N93" s="1"/>
+      <c r="O93" s="7"/>
+      <c r="P93" s="7"/>
+      <c r="Q93" s="7"/>
+      <c r="R93" s="7"/>
+      <c r="S93" s="7"/>
+      <c r="T93" s="7"/>
+      <c r="U93" s="7"/>
+      <c r="V93" s="7"/>
+      <c r="W93" s="7"/>
+      <c r="X93" s="7"/>
+      <c r="Y93" s="7"/>
+      <c r="Z93" s="7"/>
+      <c r="AA93" s="7"/>
+      <c r="AB93" s="7"/>
+      <c r="AC93" s="7"/>
+      <c r="AD93" s="7"/>
+      <c r="AE93" s="7"/>
+      <c r="AF93" s="7"/>
+      <c r="AG93" s="7"/>
+      <c r="AH93" s="7"/>
+      <c r="AI93" s="7"/>
+      <c r="AJ93" s="7"/>
+      <c r="AK93" s="7"/>
+      <c r="AL93" s="7"/>
+      <c r="AM93" s="7"/>
+    </row>
+    <row r="94" spans="2:39" ht="28.5">
+      <c r="B94" s="1">
+        <f t="shared" si="1"/>
+        <v>88</v>
+      </c>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="I94" s="1"/>
+      <c r="J94" s="1"/>
+      <c r="K94" s="1"/>
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
+      <c r="N94" s="1"/>
+      <c r="O94" s="7"/>
+      <c r="P94" s="7"/>
+      <c r="Q94" s="7"/>
+      <c r="R94" s="7"/>
+      <c r="S94" s="7"/>
+      <c r="T94" s="7"/>
+      <c r="U94" s="7"/>
+      <c r="V94" s="7"/>
+      <c r="W94" s="7"/>
+      <c r="X94" s="7"/>
+      <c r="Y94" s="7"/>
+      <c r="Z94" s="7"/>
+      <c r="AA94" s="7"/>
+      <c r="AB94" s="7"/>
+      <c r="AC94" s="7"/>
+      <c r="AD94" s="7"/>
+      <c r="AE94" s="7"/>
+      <c r="AF94" s="7"/>
+      <c r="AG94" s="7"/>
+      <c r="AH94" s="7"/>
+      <c r="AI94" s="7"/>
+      <c r="AJ94" s="7"/>
+      <c r="AK94" s="7"/>
+      <c r="AL94" s="7"/>
+      <c r="AM94" s="7"/>
+    </row>
+    <row r="95" spans="2:39" ht="42.75">
+      <c r="B95" s="1">
+        <f t="shared" si="1"/>
+        <v>89</v>
+      </c>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="I95" s="1"/>
+      <c r="J95" s="1"/>
+      <c r="K95" s="1"/>
+      <c r="L95" s="1"/>
+      <c r="M95" s="1"/>
+      <c r="N95" s="1"/>
+      <c r="O95" s="7"/>
+      <c r="P95" s="7"/>
+      <c r="Q95" s="7"/>
+      <c r="R95" s="7"/>
+      <c r="S95" s="7"/>
+      <c r="T95" s="7"/>
+      <c r="U95" s="7"/>
+      <c r="V95" s="7"/>
+      <c r="W95" s="7"/>
+      <c r="X95" s="7"/>
+      <c r="Y95" s="7"/>
+      <c r="Z95" s="7"/>
+      <c r="AA95" s="7"/>
+      <c r="AB95" s="7"/>
+      <c r="AC95" s="7"/>
+      <c r="AD95" s="7"/>
+      <c r="AE95" s="7"/>
+      <c r="AF95" s="7"/>
+      <c r="AG95" s="7"/>
+      <c r="AH95" s="7"/>
+      <c r="AI95" s="7"/>
+      <c r="AJ95" s="7"/>
+      <c r="AK95" s="7"/>
+      <c r="AL95" s="7"/>
+      <c r="AM95" s="7"/>
+    </row>
+    <row r="96" spans="2:39" ht="28.5">
+      <c r="B96" s="1">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I96" s="1"/>
+      <c r="J96" s="1"/>
+      <c r="K96" s="1"/>
+      <c r="L96" s="1"/>
+      <c r="M96" s="1"/>
+      <c r="N96" s="1"/>
+      <c r="O96" s="7"/>
+      <c r="P96" s="7"/>
+      <c r="Q96" s="7"/>
+      <c r="R96" s="7"/>
+      <c r="S96" s="7"/>
+      <c r="T96" s="7"/>
+      <c r="U96" s="7"/>
+      <c r="V96" s="7"/>
+      <c r="W96" s="7"/>
+      <c r="X96" s="7"/>
+      <c r="Y96" s="7"/>
+      <c r="Z96" s="7"/>
+      <c r="AA96" s="7"/>
+      <c r="AB96" s="7"/>
+      <c r="AC96" s="7"/>
+      <c r="AD96" s="7"/>
+      <c r="AE96" s="7"/>
+      <c r="AF96" s="7"/>
+      <c r="AG96" s="7"/>
+      <c r="AH96" s="7"/>
+      <c r="AI96" s="7"/>
+      <c r="AJ96" s="7"/>
+      <c r="AK96" s="7"/>
+      <c r="AL96" s="7"/>
+      <c r="AM96" s="7"/>
+    </row>
+    <row r="97" spans="2:39">
+      <c r="B97" s="1">
+        <f t="shared" si="1"/>
+        <v>91</v>
+      </c>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1"/>
+      <c r="G97" s="1"/>
+      <c r="H97" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I97" s="1"/>
+      <c r="J97" s="1"/>
+      <c r="K97" s="1"/>
+      <c r="L97" s="1"/>
+      <c r="M97" s="1"/>
+      <c r="N97" s="1"/>
+      <c r="O97" s="7"/>
+      <c r="P97" s="7"/>
+      <c r="Q97" s="7"/>
+      <c r="R97" s="7"/>
+      <c r="S97" s="7"/>
+      <c r="T97" s="7"/>
+      <c r="U97" s="7"/>
+      <c r="V97" s="7"/>
+      <c r="W97" s="7"/>
+      <c r="X97" s="7"/>
+      <c r="Y97" s="7"/>
+      <c r="Z97" s="7"/>
+      <c r="AA97" s="7"/>
+      <c r="AB97" s="7"/>
+      <c r="AC97" s="7"/>
+      <c r="AD97" s="7"/>
+      <c r="AE97" s="7"/>
+      <c r="AF97" s="7"/>
+      <c r="AG97" s="7"/>
+      <c r="AH97" s="7"/>
+      <c r="AI97" s="7"/>
+      <c r="AJ97" s="7"/>
+      <c r="AK97" s="7"/>
+      <c r="AL97" s="7"/>
+      <c r="AM97" s="7"/>
+    </row>
+    <row r="98" spans="2:39" ht="28.5">
+      <c r="B98" s="1">
+        <f t="shared" si="1"/>
+        <v>92</v>
+      </c>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="I98" s="1"/>
+      <c r="J98" s="1"/>
+      <c r="K98" s="1"/>
+      <c r="L98" s="1"/>
+      <c r="M98" s="1"/>
+      <c r="N98" s="1"/>
+      <c r="O98" s="7"/>
+      <c r="P98" s="7"/>
+      <c r="Q98" s="7"/>
+      <c r="R98" s="7"/>
+      <c r="S98" s="7"/>
+      <c r="T98" s="7"/>
+      <c r="U98" s="7"/>
+      <c r="V98" s="7"/>
+      <c r="W98" s="7"/>
+      <c r="X98" s="7"/>
+      <c r="Y98" s="7"/>
+      <c r="Z98" s="7"/>
+      <c r="AA98" s="7"/>
+      <c r="AB98" s="7"/>
+      <c r="AC98" s="7"/>
+      <c r="AD98" s="7"/>
+      <c r="AE98" s="7"/>
+      <c r="AF98" s="7"/>
+      <c r="AG98" s="7"/>
+      <c r="AH98" s="7"/>
+      <c r="AI98" s="7"/>
+      <c r="AJ98" s="7"/>
+      <c r="AK98" s="7"/>
+      <c r="AL98" s="7"/>
+      <c r="AM98" s="7"/>
+    </row>
+    <row r="99" spans="2:39" ht="28.5">
+      <c r="B99" s="1">
+        <f t="shared" si="1"/>
+        <v>93</v>
+      </c>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I99" s="1"/>
+      <c r="J99" s="1"/>
+      <c r="K99" s="1"/>
+      <c r="L99" s="1"/>
+      <c r="M99" s="1"/>
+      <c r="N99" s="1"/>
+      <c r="O99" s="7"/>
+      <c r="P99" s="7"/>
+      <c r="Q99" s="7"/>
+      <c r="R99" s="7"/>
+      <c r="S99" s="7"/>
+      <c r="T99" s="7"/>
+      <c r="U99" s="7"/>
+      <c r="V99" s="7"/>
+      <c r="W99" s="7"/>
+      <c r="X99" s="7"/>
+      <c r="Y99" s="7"/>
+      <c r="Z99" s="7"/>
+      <c r="AA99" s="7"/>
+      <c r="AB99" s="7"/>
+      <c r="AC99" s="7"/>
+      <c r="AD99" s="7"/>
+      <c r="AE99" s="7"/>
+      <c r="AF99" s="7"/>
+      <c r="AG99" s="7"/>
+      <c r="AH99" s="7"/>
+      <c r="AI99" s="7"/>
+      <c r="AJ99" s="7"/>
+      <c r="AK99" s="7"/>
+      <c r="AL99" s="7"/>
+      <c r="AM99" s="7"/>
+    </row>
+    <row r="100" spans="2:39">
+      <c r="B100" s="1">
+        <f t="shared" si="1"/>
+        <v>94</v>
+      </c>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="I100" s="1"/>
+      <c r="J100" s="1"/>
+      <c r="K100" s="1"/>
+      <c r="L100" s="1"/>
+      <c r="M100" s="1"/>
+      <c r="N100" s="1"/>
+      <c r="O100" s="7"/>
+      <c r="P100" s="7"/>
+      <c r="Q100" s="7"/>
+      <c r="R100" s="7"/>
+      <c r="S100" s="7"/>
+      <c r="T100" s="7"/>
+      <c r="U100" s="7"/>
+      <c r="V100" s="7"/>
+      <c r="W100" s="7"/>
+      <c r="X100" s="7"/>
+      <c r="Y100" s="7"/>
+      <c r="Z100" s="7"/>
+      <c r="AA100" s="7"/>
+      <c r="AB100" s="7"/>
+      <c r="AC100" s="7"/>
+      <c r="AD100" s="7"/>
+      <c r="AE100" s="7"/>
+      <c r="AF100" s="7"/>
+      <c r="AG100" s="7"/>
+      <c r="AH100" s="7"/>
+      <c r="AI100" s="7"/>
+      <c r="AJ100" s="7"/>
+      <c r="AK100" s="7"/>
+      <c r="AL100" s="7"/>
+      <c r="AM100" s="7"/>
+    </row>
+    <row r="101" spans="2:39" ht="28.5">
+      <c r="B101" s="1">
+        <f t="shared" si="1"/>
+        <v>95</v>
+      </c>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="I101" s="1"/>
+      <c r="J101" s="1"/>
+      <c r="K101" s="1"/>
+      <c r="L101" s="1"/>
+      <c r="M101" s="1"/>
+      <c r="N101" s="1"/>
+      <c r="O101" s="7"/>
+      <c r="P101" s="7"/>
+      <c r="Q101" s="7"/>
+      <c r="R101" s="7"/>
+      <c r="S101" s="7"/>
+      <c r="T101" s="7"/>
+      <c r="U101" s="7"/>
+      <c r="V101" s="7"/>
+      <c r="W101" s="7"/>
+      <c r="X101" s="7"/>
+      <c r="Y101" s="7"/>
+      <c r="Z101" s="7"/>
+      <c r="AA101" s="7"/>
+      <c r="AB101" s="7"/>
+      <c r="AC101" s="7"/>
+      <c r="AD101" s="7"/>
+      <c r="AE101" s="7"/>
+      <c r="AF101" s="7"/>
+      <c r="AG101" s="7"/>
+      <c r="AH101" s="7"/>
+      <c r="AI101" s="7"/>
+      <c r="AJ101" s="7"/>
+      <c r="AK101" s="7"/>
+      <c r="AL101" s="7"/>
+      <c r="AM101" s="7"/>
+    </row>
+    <row r="102" spans="2:39" ht="42.75">
+      <c r="B102" s="1">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="I102" s="1"/>
+      <c r="J102" s="1"/>
+      <c r="K102" s="1"/>
+      <c r="L102" s="1"/>
+      <c r="M102" s="1"/>
+      <c r="N102" s="1"/>
+      <c r="O102" s="7"/>
+      <c r="P102" s="7"/>
+      <c r="Q102" s="7"/>
+      <c r="R102" s="7"/>
+      <c r="S102" s="7"/>
+      <c r="T102" s="7"/>
+      <c r="U102" s="7"/>
+      <c r="V102" s="7"/>
+      <c r="W102" s="7"/>
+      <c r="X102" s="7"/>
+      <c r="Y102" s="7"/>
+      <c r="Z102" s="7"/>
+      <c r="AA102" s="7"/>
+      <c r="AB102" s="7"/>
+      <c r="AC102" s="7"/>
+      <c r="AD102" s="7"/>
+      <c r="AE102" s="7"/>
+      <c r="AF102" s="7"/>
+      <c r="AG102" s="7"/>
+      <c r="AH102" s="7"/>
+      <c r="AI102" s="7"/>
+      <c r="AJ102" s="7"/>
+      <c r="AK102" s="7"/>
+      <c r="AL102" s="7"/>
+      <c r="AM102" s="7"/>
+    </row>
+    <row r="103" spans="2:39" ht="28.5">
+      <c r="B103" s="1">
+        <f t="shared" si="1"/>
+        <v>97</v>
+      </c>
+      <c r="C103" s="1"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="I103" s="1"/>
+      <c r="J103" s="1"/>
+      <c r="K103" s="1"/>
+      <c r="L103" s="1"/>
+      <c r="M103" s="1"/>
+      <c r="N103" s="1"/>
+      <c r="O103" s="7"/>
+      <c r="P103" s="7"/>
+      <c r="Q103" s="7"/>
+      <c r="R103" s="7"/>
+      <c r="S103" s="7"/>
+      <c r="T103" s="7"/>
+      <c r="U103" s="7"/>
+      <c r="V103" s="7"/>
+      <c r="W103" s="7"/>
+      <c r="X103" s="7"/>
+      <c r="Y103" s="7"/>
+      <c r="Z103" s="7"/>
+      <c r="AA103" s="7"/>
+      <c r="AB103" s="7"/>
+      <c r="AC103" s="7"/>
+      <c r="AD103" s="7"/>
+      <c r="AE103" s="7"/>
+      <c r="AF103" s="7"/>
+      <c r="AG103" s="7"/>
+      <c r="AH103" s="7"/>
+      <c r="AI103" s="7"/>
+      <c r="AJ103" s="7"/>
+      <c r="AK103" s="7"/>
+      <c r="AL103" s="7"/>
+      <c r="AM103" s="7"/>
+    </row>
+    <row r="104" spans="2:39" ht="42.75">
+      <c r="B104" s="1">
+        <f t="shared" si="1"/>
+        <v>98</v>
+      </c>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G104" s="1"/>
+      <c r="H104" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="I104" s="1"/>
+      <c r="J104" s="1"/>
+      <c r="K104" s="1"/>
+      <c r="L104" s="1"/>
+      <c r="M104" s="1"/>
+      <c r="N104" s="1"/>
+      <c r="O104" s="7"/>
+      <c r="P104" s="7"/>
+      <c r="Q104" s="7"/>
+      <c r="R104" s="7"/>
+      <c r="S104" s="7"/>
+      <c r="T104" s="7"/>
+      <c r="U104" s="7"/>
+      <c r="V104" s="7"/>
+      <c r="W104" s="7"/>
+      <c r="X104" s="7"/>
+      <c r="Y104" s="7"/>
+      <c r="Z104" s="7"/>
+      <c r="AA104" s="7"/>
+      <c r="AB104" s="7"/>
+      <c r="AC104" s="7"/>
+      <c r="AD104" s="7"/>
+      <c r="AE104" s="7"/>
+      <c r="AF104" s="7"/>
+      <c r="AG104" s="7"/>
+      <c r="AH104" s="7"/>
+      <c r="AI104" s="7"/>
+      <c r="AJ104" s="7"/>
+      <c r="AK104" s="7"/>
+      <c r="AL104" s="7"/>
+      <c r="AM104" s="7"/>
+    </row>
+    <row r="105" spans="2:39">
+      <c r="B105" s="1">
+        <f t="shared" si="1"/>
+        <v>99</v>
+      </c>
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1"/>
+      <c r="F105" s="1"/>
+      <c r="G105" s="1"/>
+      <c r="H105" s="8"/>
+      <c r="I105" s="1"/>
+      <c r="J105" s="1"/>
+      <c r="K105" s="1"/>
+      <c r="L105" s="1"/>
+      <c r="M105" s="1"/>
+      <c r="N105" s="1"/>
+      <c r="O105" s="7"/>
+      <c r="P105" s="7"/>
+      <c r="Q105" s="7"/>
+      <c r="R105" s="7"/>
+      <c r="S105" s="7"/>
+      <c r="T105" s="7"/>
+      <c r="U105" s="7"/>
+      <c r="V105" s="7"/>
+      <c r="W105" s="7"/>
+      <c r="X105" s="7"/>
+      <c r="Y105" s="7"/>
+      <c r="Z105" s="7"/>
+      <c r="AA105" s="7"/>
+      <c r="AB105" s="7"/>
+      <c r="AC105" s="7"/>
+      <c r="AD105" s="7"/>
+      <c r="AE105" s="7"/>
+      <c r="AF105" s="7"/>
+      <c r="AG105" s="7"/>
+      <c r="AH105" s="7"/>
+      <c r="AI105" s="7"/>
+      <c r="AJ105" s="7"/>
+      <c r="AK105" s="7"/>
+      <c r="AL105" s="7"/>
+      <c r="AM105" s="7"/>
+    </row>
+    <row r="106" spans="2:39">
+      <c r="B106" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="1"/>
+      <c r="G106" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H106" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I106" s="1"/>
+      <c r="J106" s="1"/>
+      <c r="K106" s="1"/>
+      <c r="L106" s="1"/>
+      <c r="M106" s="1"/>
+      <c r="N106" s="1"/>
+      <c r="O106" s="7"/>
+      <c r="P106" s="7"/>
+      <c r="Q106" s="7"/>
+      <c r="R106" s="7"/>
+      <c r="S106" s="7"/>
+      <c r="T106" s="7"/>
+      <c r="U106" s="7"/>
+      <c r="V106" s="7"/>
+      <c r="W106" s="7"/>
+      <c r="X106" s="7"/>
+      <c r="Y106" s="7"/>
+      <c r="Z106" s="7"/>
+      <c r="AA106" s="7"/>
+      <c r="AB106" s="7"/>
+      <c r="AC106" s="7"/>
+      <c r="AD106" s="7"/>
+      <c r="AE106" s="7"/>
+      <c r="AF106" s="7"/>
+      <c r="AG106" s="7"/>
+      <c r="AH106" s="7"/>
+      <c r="AI106" s="7"/>
+      <c r="AJ106" s="7"/>
+      <c r="AK106" s="7"/>
+      <c r="AL106" s="7"/>
+      <c r="AM106" s="7"/>
+    </row>
+    <row r="107" spans="2:39" ht="28.5">
+      <c r="B107" s="1">
+        <f t="shared" si="1"/>
+        <v>101</v>
+      </c>
+      <c r="C107" s="1"/>
+      <c r="D107" s="1"/>
+      <c r="E107" s="1"/>
+      <c r="F107" s="1"/>
+      <c r="G107" s="1"/>
+      <c r="H107" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="I107" s="1"/>
+      <c r="J107" s="1"/>
+      <c r="K107" s="1"/>
+      <c r="L107" s="1"/>
+      <c r="M107" s="1"/>
+      <c r="N107" s="1"/>
+      <c r="O107" s="7"/>
+      <c r="P107" s="7"/>
+      <c r="Q107" s="7"/>
+      <c r="R107" s="7"/>
+      <c r="S107" s="7"/>
+      <c r="T107" s="7"/>
+      <c r="U107" s="7"/>
+      <c r="V107" s="7"/>
+      <c r="W107" s="7"/>
+      <c r="X107" s="7"/>
+      <c r="Y107" s="7"/>
+      <c r="Z107" s="7"/>
+      <c r="AA107" s="7"/>
+      <c r="AB107" s="7"/>
+      <c r="AC107" s="7"/>
+      <c r="AD107" s="7"/>
+      <c r="AE107" s="7"/>
+      <c r="AF107" s="7"/>
+      <c r="AG107" s="7"/>
+      <c r="AH107" s="7"/>
+      <c r="AI107" s="7"/>
+      <c r="AJ107" s="7"/>
+      <c r="AK107" s="7"/>
+      <c r="AL107" s="7"/>
+      <c r="AM107" s="7"/>
+    </row>
+    <row r="108" spans="2:39">
+      <c r="B108" s="1">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+      <c r="C108" s="1"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+      <c r="F108" s="1"/>
+      <c r="G108" s="1"/>
+      <c r="H108" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="I108" s="1"/>
+      <c r="J108" s="1"/>
+      <c r="K108" s="1"/>
+      <c r="L108" s="1"/>
+      <c r="M108" s="1"/>
+      <c r="N108" s="1"/>
+      <c r="O108" s="7"/>
+      <c r="P108" s="7"/>
+      <c r="Q108" s="7"/>
+      <c r="R108" s="7"/>
+      <c r="S108" s="7"/>
+      <c r="T108" s="7"/>
+      <c r="U108" s="7"/>
+      <c r="V108" s="7"/>
+      <c r="W108" s="7"/>
+      <c r="X108" s="7"/>
+      <c r="Y108" s="7"/>
+      <c r="Z108" s="7"/>
+      <c r="AA108" s="7"/>
+      <c r="AB108" s="7"/>
+      <c r="AC108" s="7"/>
+      <c r="AD108" s="7"/>
+      <c r="AE108" s="7"/>
+      <c r="AF108" s="7"/>
+      <c r="AG108" s="7"/>
+      <c r="AH108" s="7"/>
+      <c r="AI108" s="7"/>
+      <c r="AJ108" s="7"/>
+      <c r="AK108" s="7"/>
+      <c r="AL108" s="7"/>
+      <c r="AM108" s="7"/>
+    </row>
+    <row r="109" spans="2:39" ht="28.5">
+      <c r="B109" s="1">
+        <f t="shared" si="1"/>
+        <v>103</v>
+      </c>
+      <c r="C109" s="1"/>
+      <c r="D109" s="1"/>
+      <c r="E109" s="1"/>
+      <c r="F109" s="1"/>
+      <c r="G109" s="1"/>
+      <c r="H109" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="I109" s="1"/>
+      <c r="J109" s="1"/>
+      <c r="K109" s="1"/>
+      <c r="L109" s="1"/>
+      <c r="M109" s="1"/>
+      <c r="N109" s="1"/>
+      <c r="O109" s="7"/>
+      <c r="P109" s="7"/>
+      <c r="Q109" s="7"/>
+      <c r="R109" s="7"/>
+      <c r="S109" s="7"/>
+      <c r="T109" s="7"/>
+      <c r="U109" s="7"/>
+      <c r="V109" s="7"/>
+      <c r="W109" s="7"/>
+      <c r="X109" s="7"/>
+      <c r="Y109" s="7"/>
+      <c r="Z109" s="7"/>
+      <c r="AA109" s="7"/>
+      <c r="AB109" s="7"/>
+      <c r="AC109" s="7"/>
+      <c r="AD109" s="7"/>
+      <c r="AE109" s="7"/>
+      <c r="AF109" s="7"/>
+      <c r="AG109" s="7"/>
+      <c r="AH109" s="7"/>
+      <c r="AI109" s="7"/>
+      <c r="AJ109" s="7"/>
+      <c r="AK109" s="7"/>
+      <c r="AL109" s="7"/>
+      <c r="AM109" s="7"/>
+    </row>
+    <row r="110" spans="2:39" ht="28.5">
+      <c r="B110" s="1">
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="1"/>
+      <c r="H110" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="I110" s="1"/>
+      <c r="J110" s="1"/>
+      <c r="K110" s="1"/>
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+      <c r="N110" s="1"/>
+      <c r="O110" s="7"/>
+      <c r="P110" s="7"/>
+      <c r="Q110" s="7"/>
+      <c r="R110" s="7"/>
+      <c r="S110" s="7"/>
+      <c r="T110" s="7"/>
+      <c r="U110" s="7"/>
+      <c r="V110" s="7"/>
+      <c r="W110" s="7"/>
+      <c r="X110" s="7"/>
+      <c r="Y110" s="7"/>
+      <c r="Z110" s="7"/>
+      <c r="AA110" s="7"/>
+      <c r="AB110" s="7"/>
+      <c r="AC110" s="7"/>
+      <c r="AD110" s="7"/>
+      <c r="AE110" s="7"/>
+      <c r="AF110" s="7"/>
+      <c r="AG110" s="7"/>
+      <c r="AH110" s="7"/>
+      <c r="AI110" s="7"/>
+      <c r="AJ110" s="7"/>
+      <c r="AK110" s="7"/>
+      <c r="AL110" s="7"/>
+      <c r="AM110" s="7"/>
+    </row>
+    <row r="111" spans="2:39">
+      <c r="B111" s="1">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+      <c r="C111" s="1"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="1"/>
+      <c r="H111" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="I111" s="1"/>
+      <c r="J111" s="1"/>
+      <c r="K111" s="1"/>
+      <c r="L111" s="1"/>
+      <c r="M111" s="1"/>
+      <c r="N111" s="1"/>
+      <c r="O111" s="7"/>
+      <c r="P111" s="7"/>
+      <c r="Q111" s="7"/>
+      <c r="R111" s="7"/>
+      <c r="S111" s="7"/>
+      <c r="T111" s="7"/>
+      <c r="U111" s="7"/>
+      <c r="V111" s="7"/>
+      <c r="W111" s="7"/>
+      <c r="X111" s="7"/>
+      <c r="Y111" s="7"/>
+      <c r="Z111" s="7"/>
+      <c r="AA111" s="7"/>
+      <c r="AB111" s="7"/>
+      <c r="AC111" s="7"/>
+      <c r="AD111" s="7"/>
+      <c r="AE111" s="7"/>
+      <c r="AF111" s="7"/>
+      <c r="AG111" s="7"/>
+      <c r="AH111" s="7"/>
+      <c r="AI111" s="7"/>
+      <c r="AJ111" s="7"/>
+      <c r="AK111" s="7"/>
+      <c r="AL111" s="7"/>
+      <c r="AM111" s="7"/>
+    </row>
+    <row r="112" spans="2:39" ht="57">
+      <c r="B112" s="1">
+        <f t="shared" si="1"/>
+        <v>106</v>
+      </c>
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="1"/>
+      <c r="G112" s="1"/>
+      <c r="H112" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="I112" s="1"/>
+      <c r="J112" s="1"/>
+      <c r="K112" s="1"/>
+      <c r="L112" s="1"/>
+      <c r="M112" s="1"/>
+      <c r="N112" s="1"/>
+      <c r="O112" s="7"/>
+      <c r="P112" s="7"/>
+      <c r="Q112" s="7"/>
+      <c r="R112" s="7"/>
+      <c r="S112" s="7"/>
+      <c r="T112" s="7"/>
+      <c r="U112" s="7"/>
+      <c r="V112" s="7"/>
+      <c r="W112" s="7"/>
+      <c r="X112" s="7"/>
+      <c r="Y112" s="7"/>
+      <c r="Z112" s="7"/>
+      <c r="AA112" s="7"/>
+      <c r="AB112" s="7"/>
+      <c r="AC112" s="7"/>
+      <c r="AD112" s="7"/>
+      <c r="AE112" s="7"/>
+      <c r="AF112" s="7"/>
+      <c r="AG112" s="7"/>
+      <c r="AH112" s="7"/>
+      <c r="AI112" s="7"/>
+      <c r="AJ112" s="7"/>
+      <c r="AK112" s="7"/>
+      <c r="AL112" s="7"/>
+      <c r="AM112" s="7"/>
+    </row>
+    <row r="113" spans="2:39" ht="28.5">
+      <c r="B113" s="1">
+        <f t="shared" si="1"/>
+        <v>107</v>
+      </c>
+      <c r="C113" s="1"/>
+      <c r="D113" s="1"/>
+      <c r="E113" s="1"/>
+      <c r="F113" s="1"/>
+      <c r="G113" s="1"/>
+      <c r="H113" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="I113" s="1"/>
+      <c r="J113" s="1"/>
+      <c r="K113" s="1"/>
+      <c r="L113" s="1"/>
+      <c r="M113" s="1"/>
+      <c r="N113" s="1"/>
+      <c r="O113" s="7"/>
+      <c r="P113" s="7"/>
+      <c r="Q113" s="7"/>
+      <c r="R113" s="7"/>
+      <c r="S113" s="7"/>
+      <c r="T113" s="7"/>
+      <c r="U113" s="7"/>
+      <c r="V113" s="7"/>
+      <c r="W113" s="7"/>
+      <c r="X113" s="7"/>
+      <c r="Y113" s="7"/>
+      <c r="Z113" s="7"/>
+      <c r="AA113" s="7"/>
+      <c r="AB113" s="7"/>
+      <c r="AC113" s="7"/>
+      <c r="AD113" s="7"/>
+      <c r="AE113" s="7"/>
+      <c r="AF113" s="7"/>
+      <c r="AG113" s="7"/>
+      <c r="AH113" s="7"/>
+      <c r="AI113" s="7"/>
+      <c r="AJ113" s="7"/>
+      <c r="AK113" s="7"/>
+      <c r="AL113" s="7"/>
+      <c r="AM113" s="7"/>
+    </row>
+    <row r="114" spans="2:39" ht="42.75">
+      <c r="B114" s="1">
+        <f t="shared" si="1"/>
+        <v>108</v>
+      </c>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+      <c r="F114" s="1"/>
+      <c r="G114" s="1"/>
+      <c r="H114" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="I114" s="1"/>
+      <c r="J114" s="1"/>
+      <c r="K114" s="1"/>
+      <c r="L114" s="1"/>
+      <c r="M114" s="1"/>
+      <c r="N114" s="1"/>
+      <c r="O114" s="7"/>
+      <c r="P114" s="7"/>
+      <c r="Q114" s="7"/>
+      <c r="R114" s="7"/>
+      <c r="S114" s="7"/>
+      <c r="T114" s="7"/>
+      <c r="U114" s="7"/>
+      <c r="V114" s="7"/>
+      <c r="W114" s="7"/>
+      <c r="X114" s="7"/>
+      <c r="Y114" s="7"/>
+      <c r="Z114" s="7"/>
+      <c r="AA114" s="7"/>
+      <c r="AB114" s="7"/>
+      <c r="AC114" s="7"/>
+      <c r="AD114" s="7"/>
+      <c r="AE114" s="7"/>
+      <c r="AF114" s="7"/>
+      <c r="AG114" s="7"/>
+      <c r="AH114" s="7"/>
+      <c r="AI114" s="7"/>
+      <c r="AJ114" s="7"/>
+      <c r="AK114" s="7"/>
+      <c r="AL114" s="7"/>
+      <c r="AM114" s="7"/>
+    </row>
+    <row r="115" spans="2:39" ht="28.5">
+      <c r="B115" s="1">
+        <f t="shared" si="1"/>
+        <v>109</v>
+      </c>
+      <c r="C115" s="1"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="1"/>
+      <c r="F115" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G115" s="1"/>
+      <c r="H115" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="I115" s="1"/>
+      <c r="J115" s="1"/>
+      <c r="K115" s="1"/>
+      <c r="L115" s="1"/>
+      <c r="M115" s="1"/>
+      <c r="N115" s="1"/>
+      <c r="O115" s="7"/>
+      <c r="P115" s="7"/>
+      <c r="Q115" s="7"/>
+      <c r="R115" s="7"/>
+      <c r="S115" s="7"/>
+      <c r="T115" s="7"/>
+      <c r="U115" s="7"/>
+      <c r="V115" s="7"/>
+      <c r="W115" s="7"/>
+      <c r="X115" s="7"/>
+      <c r="Y115" s="7"/>
+      <c r="Z115" s="7"/>
+      <c r="AA115" s="7"/>
+      <c r="AB115" s="7"/>
+      <c r="AC115" s="7"/>
+      <c r="AD115" s="7"/>
+      <c r="AE115" s="7"/>
+      <c r="AF115" s="7"/>
+      <c r="AG115" s="7"/>
+      <c r="AH115" s="7"/>
+      <c r="AI115" s="7"/>
+      <c r="AJ115" s="7"/>
+      <c r="AK115" s="7"/>
+      <c r="AL115" s="7"/>
+      <c r="AM115" s="7"/>
+    </row>
+    <row r="116" spans="2:39">
+      <c r="B116" s="1">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+      <c r="C116" s="1"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+      <c r="F116" s="1"/>
+      <c r="G116" s="1"/>
+      <c r="H116" s="8"/>
+      <c r="I116" s="1"/>
+      <c r="J116" s="1"/>
+      <c r="K116" s="1"/>
+      <c r="L116" s="1"/>
+      <c r="M116" s="1"/>
+      <c r="N116" s="1"/>
+      <c r="O116" s="7"/>
+      <c r="P116" s="7"/>
+      <c r="Q116" s="7"/>
+      <c r="R116" s="7"/>
+      <c r="S116" s="7"/>
+      <c r="T116" s="7"/>
+      <c r="U116" s="7"/>
+      <c r="V116" s="7"/>
+      <c r="W116" s="7"/>
+      <c r="X116" s="7"/>
+      <c r="Y116" s="7"/>
+      <c r="Z116" s="7"/>
+      <c r="AA116" s="7"/>
+      <c r="AB116" s="7"/>
+      <c r="AC116" s="7"/>
+      <c r="AD116" s="7"/>
+      <c r="AE116" s="7"/>
+      <c r="AF116" s="7"/>
+      <c r="AG116" s="7"/>
+      <c r="AH116" s="7"/>
+      <c r="AI116" s="7"/>
+      <c r="AJ116" s="7"/>
+      <c r="AK116" s="7"/>
+      <c r="AL116" s="7"/>
+      <c r="AM116" s="7"/>
+    </row>
+    <row r="117" spans="2:39">
+      <c r="B117" s="1">
+        <f t="shared" si="1"/>
+        <v>111</v>
+      </c>
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+      <c r="F117" s="1"/>
+      <c r="G117" s="1"/>
+      <c r="H117" s="8"/>
+      <c r="I117" s="1"/>
+      <c r="J117" s="1"/>
+      <c r="K117" s="1"/>
+      <c r="L117" s="1"/>
+      <c r="M117" s="1"/>
+      <c r="N117" s="1"/>
+      <c r="O117" s="7"/>
+      <c r="P117" s="7"/>
+      <c r="Q117" s="7"/>
+      <c r="R117" s="7"/>
+      <c r="S117" s="7"/>
+      <c r="T117" s="7"/>
+      <c r="U117" s="7"/>
+      <c r="V117" s="7"/>
+      <c r="W117" s="7"/>
+      <c r="X117" s="7"/>
+      <c r="Y117" s="7"/>
+      <c r="Z117" s="7"/>
+      <c r="AA117" s="7"/>
+      <c r="AB117" s="7"/>
+      <c r="AC117" s="7"/>
+      <c r="AD117" s="7"/>
+      <c r="AE117" s="7"/>
+      <c r="AF117" s="7"/>
+      <c r="AG117" s="7"/>
+      <c r="AH117" s="7"/>
+      <c r="AI117" s="7"/>
+      <c r="AJ117" s="7"/>
+      <c r="AK117" s="7"/>
+      <c r="AL117" s="7"/>
+      <c r="AM117" s="7"/>
+    </row>
+    <row r="118" spans="2:39">
+      <c r="B118" s="1">
+        <f t="shared" si="1"/>
+        <v>112</v>
+      </c>
+      <c r="C118" s="1"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+      <c r="F118" s="1"/>
+      <c r="G118" s="1"/>
+      <c r="H118" s="8"/>
+      <c r="I118" s="1"/>
+      <c r="J118" s="1"/>
+      <c r="K118" s="1"/>
+      <c r="L118" s="1"/>
+      <c r="M118" s="1"/>
+      <c r="N118" s="1"/>
+      <c r="O118" s="7"/>
+      <c r="P118" s="7"/>
+      <c r="Q118" s="7"/>
+      <c r="R118" s="7"/>
+      <c r="S118" s="7"/>
+      <c r="T118" s="7"/>
+      <c r="U118" s="7"/>
+      <c r="V118" s="7"/>
+      <c r="W118" s="7"/>
+      <c r="X118" s="7"/>
+      <c r="Y118" s="7"/>
+      <c r="Z118" s="7"/>
+      <c r="AA118" s="7"/>
+      <c r="AB118" s="7"/>
+      <c r="AC118" s="7"/>
+      <c r="AD118" s="7"/>
+      <c r="AE118" s="7"/>
+      <c r="AF118" s="7"/>
+      <c r="AG118" s="7"/>
+      <c r="AH118" s="7"/>
+      <c r="AI118" s="7"/>
+      <c r="AJ118" s="7"/>
+      <c r="AK118" s="7"/>
+      <c r="AL118" s="7"/>
+      <c r="AM118" s="7"/>
+    </row>
+    <row r="119" spans="2:39">
+      <c r="B119" s="1">
+        <f t="shared" si="1"/>
+        <v>113</v>
+      </c>
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1"/>
+      <c r="F119" s="1"/>
+      <c r="G119" s="1"/>
+      <c r="H119" s="8"/>
+      <c r="I119" s="1"/>
+      <c r="J119" s="1"/>
+      <c r="K119" s="1"/>
+      <c r="L119" s="1"/>
+      <c r="M119" s="1"/>
+      <c r="N119" s="1"/>
+      <c r="O119" s="7"/>
+      <c r="P119" s="7"/>
+      <c r="Q119" s="7"/>
+      <c r="R119" s="7"/>
+      <c r="S119" s="7"/>
+      <c r="T119" s="7"/>
+      <c r="U119" s="7"/>
+      <c r="V119" s="7"/>
+      <c r="W119" s="7"/>
+      <c r="X119" s="7"/>
+      <c r="Y119" s="7"/>
+      <c r="Z119" s="7"/>
+      <c r="AA119" s="7"/>
+      <c r="AB119" s="7"/>
+      <c r="AC119" s="7"/>
+      <c r="AD119" s="7"/>
+      <c r="AE119" s="7"/>
+      <c r="AF119" s="7"/>
+      <c r="AG119" s="7"/>
+      <c r="AH119" s="7"/>
+      <c r="AI119" s="7"/>
+      <c r="AJ119" s="7"/>
+      <c r="AK119" s="7"/>
+      <c r="AL119" s="7"/>
+      <c r="AM119" s="7"/>
+    </row>
+    <row r="120" spans="2:39">
+      <c r="B120" s="1">
+        <f t="shared" si="1"/>
+        <v>114</v>
+      </c>
+      <c r="C120" s="1"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="1"/>
+      <c r="F120" s="1"/>
+      <c r="G120" s="1"/>
+      <c r="H120" s="8"/>
+      <c r="I120" s="1"/>
+      <c r="J120" s="1"/>
+      <c r="K120" s="1"/>
+      <c r="L120" s="1"/>
+      <c r="M120" s="1"/>
+      <c r="N120" s="1"/>
+      <c r="O120" s="7"/>
+      <c r="P120" s="7"/>
+      <c r="Q120" s="7"/>
+      <c r="R120" s="7"/>
+      <c r="S120" s="7"/>
+      <c r="T120" s="7"/>
+      <c r="U120" s="7"/>
+      <c r="V120" s="7"/>
+      <c r="W120" s="7"/>
+      <c r="X120" s="7"/>
+      <c r="Y120" s="7"/>
+      <c r="Z120" s="7"/>
+      <c r="AA120" s="7"/>
+      <c r="AB120" s="7"/>
+      <c r="AC120" s="7"/>
+      <c r="AD120" s="7"/>
+      <c r="AE120" s="7"/>
+      <c r="AF120" s="7"/>
+      <c r="AG120" s="7"/>
+      <c r="AH120" s="7"/>
+      <c r="AI120" s="7"/>
+      <c r="AJ120" s="7"/>
+      <c r="AK120" s="7"/>
+      <c r="AL120" s="7"/>
+      <c r="AM120" s="7"/>
+    </row>
+    <row r="121" spans="2:39">
+      <c r="B121" s="1">
+        <f t="shared" si="1"/>
+        <v>115</v>
+      </c>
+      <c r="C121" s="1"/>
+      <c r="D121" s="1"/>
+      <c r="E121" s="1"/>
+      <c r="F121" s="1"/>
+      <c r="G121" s="1"/>
+      <c r="H121" s="8"/>
+      <c r="I121" s="1"/>
+      <c r="J121" s="1"/>
+      <c r="K121" s="1"/>
+      <c r="L121" s="1"/>
+      <c r="M121" s="1"/>
+      <c r="N121" s="1"/>
+      <c r="O121" s="7"/>
+      <c r="P121" s="7"/>
+      <c r="Q121" s="7"/>
+      <c r="R121" s="7"/>
+      <c r="S121" s="7"/>
+      <c r="T121" s="7"/>
+      <c r="U121" s="7"/>
+      <c r="V121" s="7"/>
+      <c r="W121" s="7"/>
+      <c r="X121" s="7"/>
+      <c r="Y121" s="7"/>
+      <c r="Z121" s="7"/>
+      <c r="AA121" s="7"/>
+      <c r="AB121" s="7"/>
+      <c r="AC121" s="7"/>
+      <c r="AD121" s="7"/>
+      <c r="AE121" s="7"/>
+      <c r="AF121" s="7"/>
+      <c r="AG121" s="7"/>
+      <c r="AH121" s="7"/>
+      <c r="AI121" s="7"/>
+      <c r="AJ121" s="7"/>
+      <c r="AK121" s="7"/>
+      <c r="AL121" s="7"/>
+      <c r="AM121" s="7"/>
+    </row>
+    <row r="122" spans="2:39">
+      <c r="B122" s="1">
+        <f t="shared" si="1"/>
+        <v>116</v>
+      </c>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+      <c r="F122" s="1"/>
+      <c r="G122" s="1"/>
+      <c r="H122" s="8"/>
+      <c r="I122" s="1"/>
+      <c r="J122" s="1"/>
+      <c r="K122" s="1"/>
+      <c r="L122" s="1"/>
+      <c r="M122" s="1"/>
+      <c r="N122" s="1"/>
+      <c r="O122" s="7"/>
+      <c r="P122" s="7"/>
+      <c r="Q122" s="7"/>
+      <c r="R122" s="7"/>
+      <c r="S122" s="7"/>
+      <c r="T122" s="7"/>
+      <c r="U122" s="7"/>
+      <c r="V122" s="7"/>
+      <c r="W122" s="7"/>
+      <c r="X122" s="7"/>
+      <c r="Y122" s="7"/>
+      <c r="Z122" s="7"/>
+      <c r="AA122" s="7"/>
+      <c r="AB122" s="7"/>
+      <c r="AC122" s="7"/>
+      <c r="AD122" s="7"/>
+      <c r="AE122" s="7"/>
+      <c r="AF122" s="7"/>
+      <c r="AG122" s="7"/>
+      <c r="AH122" s="7"/>
+      <c r="AI122" s="7"/>
+      <c r="AJ122" s="7"/>
+      <c r="AK122" s="7"/>
+      <c r="AL122" s="7"/>
+      <c r="AM122" s="7"/>
+    </row>
+    <row r="123" spans="2:39">
+      <c r="B123" s="1">
+        <f t="shared" si="1"/>
+        <v>117</v>
+      </c>
+      <c r="C123" s="1"/>
+      <c r="D123" s="1"/>
+      <c r="E123" s="1"/>
+      <c r="F123" s="1"/>
+      <c r="G123" s="1"/>
+      <c r="H123" s="8"/>
+      <c r="I123" s="1"/>
+      <c r="J123" s="1"/>
+      <c r="K123" s="1"/>
+      <c r="L123" s="1"/>
+      <c r="M123" s="1"/>
+      <c r="N123" s="1"/>
+      <c r="O123" s="7"/>
+      <c r="P123" s="7"/>
+      <c r="Q123" s="7"/>
+      <c r="R123" s="7"/>
+      <c r="S123" s="7"/>
+      <c r="T123" s="7"/>
+      <c r="U123" s="7"/>
+      <c r="V123" s="7"/>
+      <c r="W123" s="7"/>
+      <c r="X123" s="7"/>
+      <c r="Y123" s="7"/>
+      <c r="Z123" s="7"/>
+      <c r="AA123" s="7"/>
+      <c r="AB123" s="7"/>
+      <c r="AC123" s="7"/>
+      <c r="AD123" s="7"/>
+      <c r="AE123" s="7"/>
+      <c r="AF123" s="7"/>
+      <c r="AG123" s="7"/>
+      <c r="AH123" s="7"/>
+      <c r="AI123" s="7"/>
+      <c r="AJ123" s="7"/>
+      <c r="AK123" s="7"/>
+      <c r="AL123" s="7"/>
+      <c r="AM123" s="7"/>
+    </row>
+    <row r="124" spans="2:39">
+      <c r="B124" s="1">
+        <f t="shared" si="1"/>
+        <v>118</v>
+      </c>
+      <c r="C124" s="1"/>
+      <c r="D124" s="1"/>
+      <c r="E124" s="1"/>
+      <c r="F124" s="1"/>
+      <c r="G124" s="1"/>
+      <c r="H124" s="8"/>
+      <c r="I124" s="1"/>
+      <c r="J124" s="1"/>
+      <c r="K124" s="1"/>
+      <c r="L124" s="1"/>
+      <c r="M124" s="1"/>
+      <c r="N124" s="1"/>
+      <c r="O124" s="7"/>
+      <c r="P124" s="7"/>
+      <c r="Q124" s="7"/>
+      <c r="R124" s="7"/>
+      <c r="S124" s="7"/>
+      <c r="T124" s="7"/>
+      <c r="U124" s="7"/>
+      <c r="V124" s="7"/>
+      <c r="W124" s="7"/>
+      <c r="X124" s="7"/>
+      <c r="Y124" s="7"/>
+      <c r="Z124" s="7"/>
+      <c r="AA124" s="7"/>
+      <c r="AB124" s="7"/>
+      <c r="AC124" s="7"/>
+      <c r="AD124" s="7"/>
+      <c r="AE124" s="7"/>
+      <c r="AF124" s="7"/>
+      <c r="AG124" s="7"/>
+      <c r="AH124" s="7"/>
+      <c r="AI124" s="7"/>
+      <c r="AJ124" s="7"/>
+      <c r="AK124" s="7"/>
+      <c r="AL124" s="7"/>
+      <c r="AM124" s="7"/>
+    </row>
+    <row r="125" spans="2:39">
+      <c r="B125" s="1">
+        <f t="shared" si="1"/>
+        <v>119</v>
+      </c>
+      <c r="C125" s="1"/>
+      <c r="D125" s="1"/>
+      <c r="E125" s="1"/>
+      <c r="F125" s="1"/>
+      <c r="G125" s="1"/>
+      <c r="H125" s="8"/>
+      <c r="I125" s="1"/>
+      <c r="J125" s="1"/>
+      <c r="K125" s="1"/>
+      <c r="L125" s="1"/>
+      <c r="M125" s="1"/>
+      <c r="N125" s="1"/>
+      <c r="O125" s="7"/>
+      <c r="P125" s="7"/>
+      <c r="Q125" s="7"/>
+      <c r="R125" s="7"/>
+      <c r="S125" s="7"/>
+      <c r="T125" s="7"/>
+      <c r="U125" s="7"/>
+      <c r="V125" s="7"/>
+      <c r="W125" s="7"/>
+      <c r="X125" s="7"/>
+      <c r="Y125" s="7"/>
+      <c r="Z125" s="7"/>
+      <c r="AA125" s="7"/>
+      <c r="AB125" s="7"/>
+      <c r="AC125" s="7"/>
+      <c r="AD125" s="7"/>
+      <c r="AE125" s="7"/>
+      <c r="AF125" s="7"/>
+      <c r="AG125" s="7"/>
+      <c r="AH125" s="7"/>
+      <c r="AI125" s="7"/>
+      <c r="AJ125" s="7"/>
+      <c r="AK125" s="7"/>
+      <c r="AL125" s="7"/>
+      <c r="AM125" s="7"/>
+    </row>
+    <row r="126" spans="2:39">
+      <c r="B126" s="1">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="1"/>
+      <c r="F126" s="1"/>
+      <c r="G126" s="1"/>
+      <c r="H126" s="8"/>
+      <c r="I126" s="1"/>
+      <c r="J126" s="1"/>
+      <c r="K126" s="1"/>
+      <c r="L126" s="1"/>
+      <c r="M126" s="1"/>
+      <c r="N126" s="1"/>
+      <c r="O126" s="7"/>
+      <c r="P126" s="7"/>
+      <c r="Q126" s="7"/>
+      <c r="R126" s="7"/>
+      <c r="S126" s="7"/>
+      <c r="T126" s="7"/>
+      <c r="U126" s="7"/>
+      <c r="V126" s="7"/>
+      <c r="W126" s="7"/>
+      <c r="X126" s="7"/>
+      <c r="Y126" s="7"/>
+      <c r="Z126" s="7"/>
+      <c r="AA126" s="7"/>
+      <c r="AB126" s="7"/>
+      <c r="AC126" s="7"/>
+      <c r="AD126" s="7"/>
+      <c r="AE126" s="7"/>
+      <c r="AF126" s="7"/>
+      <c r="AG126" s="7"/>
+      <c r="AH126" s="7"/>
+      <c r="AI126" s="7"/>
+      <c r="AJ126" s="7"/>
+      <c r="AK126" s="7"/>
+      <c r="AL126" s="7"/>
+      <c r="AM126" s="7"/>
+    </row>
+    <row r="127" spans="2:39">
+      <c r="B127" s="1">
+        <f t="shared" si="1"/>
+        <v>121</v>
+      </c>
+      <c r="C127" s="1"/>
+      <c r="D127" s="1"/>
+      <c r="E127" s="1"/>
+      <c r="F127" s="1"/>
+      <c r="G127" s="1"/>
+      <c r="H127" s="8"/>
+      <c r="I127" s="1"/>
+      <c r="J127" s="1"/>
+      <c r="K127" s="1"/>
+      <c r="L127" s="1"/>
+      <c r="M127" s="1"/>
+      <c r="N127" s="1"/>
+      <c r="O127" s="7"/>
+      <c r="P127" s="7"/>
+      <c r="Q127" s="7"/>
+      <c r="R127" s="7"/>
+      <c r="S127" s="7"/>
+      <c r="T127" s="7"/>
+      <c r="U127" s="7"/>
+      <c r="V127" s="7"/>
+      <c r="W127" s="7"/>
+      <c r="X127" s="7"/>
+      <c r="Y127" s="7"/>
+      <c r="Z127" s="7"/>
+      <c r="AA127" s="7"/>
+      <c r="AB127" s="7"/>
+      <c r="AC127" s="7"/>
+      <c r="AD127" s="7"/>
+      <c r="AE127" s="7"/>
+      <c r="AF127" s="7"/>
+      <c r="AG127" s="7"/>
+      <c r="AH127" s="7"/>
+      <c r="AI127" s="7"/>
+      <c r="AJ127" s="7"/>
+      <c r="AK127" s="7"/>
+      <c r="AL127" s="7"/>
+      <c r="AM127" s="7"/>
+    </row>
+    <row r="128" spans="2:39">
+      <c r="B128" s="1">
+        <f t="shared" si="1"/>
+        <v>122</v>
+      </c>
+      <c r="C128" s="1"/>
+      <c r="D128" s="1"/>
+      <c r="E128" s="1"/>
+      <c r="F128" s="1"/>
+      <c r="G128" s="1"/>
+      <c r="H128" s="8"/>
+      <c r="I128" s="1"/>
+      <c r="J128" s="1"/>
+      <c r="K128" s="1"/>
+      <c r="L128" s="1"/>
+      <c r="M128" s="1"/>
+      <c r="N128" s="1"/>
+      <c r="O128" s="7"/>
+      <c r="P128" s="7"/>
+      <c r="Q128" s="7"/>
+      <c r="R128" s="7"/>
+      <c r="S128" s="7"/>
+      <c r="T128" s="7"/>
+      <c r="U128" s="7"/>
+      <c r="V128" s="7"/>
+      <c r="W128" s="7"/>
+      <c r="X128" s="7"/>
+      <c r="Y128" s="7"/>
+      <c r="Z128" s="7"/>
+      <c r="AA128" s="7"/>
+      <c r="AB128" s="7"/>
+      <c r="AC128" s="7"/>
+      <c r="AD128" s="7"/>
+      <c r="AE128" s="7"/>
+      <c r="AF128" s="7"/>
+      <c r="AG128" s="7"/>
+      <c r="AH128" s="7"/>
+      <c r="AI128" s="7"/>
+      <c r="AJ128" s="7"/>
+      <c r="AK128" s="7"/>
+      <c r="AL128" s="7"/>
+      <c r="AM128" s="7"/>
+    </row>
+    <row r="129" spans="2:39">
+      <c r="B129" s="1">
+        <f t="shared" si="1"/>
+        <v>123</v>
+      </c>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="1"/>
+      <c r="F129" s="1"/>
+      <c r="G129" s="1"/>
+      <c r="H129" s="8"/>
+      <c r="I129" s="1"/>
+      <c r="J129" s="1"/>
+      <c r="K129" s="1"/>
+      <c r="L129" s="1"/>
+      <c r="M129" s="1"/>
+      <c r="N129" s="1"/>
+      <c r="O129" s="7"/>
+      <c r="P129" s="7"/>
+      <c r="Q129" s="7"/>
+      <c r="R129" s="7"/>
+      <c r="S129" s="7"/>
+      <c r="T129" s="7"/>
+      <c r="U129" s="7"/>
+      <c r="V129" s="7"/>
+      <c r="W129" s="7"/>
+      <c r="X129" s="7"/>
+      <c r="Y129" s="7"/>
+      <c r="Z129" s="7"/>
+      <c r="AA129" s="7"/>
+      <c r="AB129" s="7"/>
+      <c r="AC129" s="7"/>
+      <c r="AD129" s="7"/>
+      <c r="AE129" s="7"/>
+      <c r="AF129" s="7"/>
+      <c r="AG129" s="7"/>
+      <c r="AH129" s="7"/>
+      <c r="AI129" s="7"/>
+      <c r="AJ129" s="7"/>
+      <c r="AK129" s="7"/>
+      <c r="AL129" s="7"/>
+      <c r="AM129" s="7"/>
+    </row>
+    <row r="130" spans="2:39">
+      <c r="B130" s="1">
+        <f t="shared" si="1"/>
+        <v>124</v>
+      </c>
+      <c r="C130" s="1"/>
+      <c r="D130" s="1"/>
+      <c r="E130" s="1"/>
+      <c r="F130" s="1"/>
+      <c r="G130" s="1"/>
+      <c r="H130" s="8"/>
+      <c r="I130" s="1"/>
+      <c r="J130" s="1"/>
+      <c r="K130" s="1"/>
+      <c r="L130" s="1"/>
+      <c r="M130" s="1"/>
+      <c r="N130" s="1"/>
+      <c r="O130" s="7"/>
+      <c r="P130" s="7"/>
+      <c r="Q130" s="7"/>
+      <c r="R130" s="7"/>
+      <c r="S130" s="7"/>
+      <c r="T130" s="7"/>
+      <c r="U130" s="7"/>
+      <c r="V130" s="7"/>
+      <c r="W130" s="7"/>
+      <c r="X130" s="7"/>
+      <c r="Y130" s="7"/>
+      <c r="Z130" s="7"/>
+      <c r="AA130" s="7"/>
+      <c r="AB130" s="7"/>
+      <c r="AC130" s="7"/>
+      <c r="AD130" s="7"/>
+      <c r="AE130" s="7"/>
+      <c r="AF130" s="7"/>
+      <c r="AG130" s="7"/>
+      <c r="AH130" s="7"/>
+      <c r="AI130" s="7"/>
+      <c r="AJ130" s="7"/>
+      <c r="AK130" s="7"/>
+      <c r="AL130" s="7"/>
+      <c r="AM130" s="7"/>
+    </row>
+    <row r="131" spans="2:39">
+      <c r="B131" s="1">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+      <c r="C131" s="1"/>
+      <c r="D131" s="1"/>
+      <c r="E131" s="1"/>
+      <c r="F131" s="1"/>
+      <c r="G131" s="1"/>
+      <c r="H131" s="8"/>
+      <c r="I131" s="1"/>
+      <c r="J131" s="1"/>
+      <c r="K131" s="1"/>
+      <c r="L131" s="1"/>
+      <c r="M131" s="1"/>
+      <c r="N131" s="1"/>
+      <c r="O131" s="7"/>
+      <c r="P131" s="7"/>
+      <c r="Q131" s="7"/>
+      <c r="R131" s="7"/>
+      <c r="S131" s="7"/>
+      <c r="T131" s="7"/>
+      <c r="U131" s="7"/>
+      <c r="V131" s="7"/>
+      <c r="W131" s="7"/>
+      <c r="X131" s="7"/>
+      <c r="Y131" s="7"/>
+      <c r="Z131" s="7"/>
+      <c r="AA131" s="7"/>
+      <c r="AB131" s="7"/>
+      <c r="AC131" s="7"/>
+      <c r="AD131" s="7"/>
+      <c r="AE131" s="7"/>
+      <c r="AF131" s="7"/>
+      <c r="AG131" s="7"/>
+      <c r="AH131" s="7"/>
+      <c r="AI131" s="7"/>
+      <c r="AJ131" s="7"/>
+      <c r="AK131" s="7"/>
+      <c r="AL131" s="7"/>
+      <c r="AM131" s="7"/>
+    </row>
+    <row r="132" spans="2:39">
+      <c r="B132" s="1">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="C132" s="1"/>
+      <c r="D132" s="1"/>
+      <c r="E132" s="1"/>
+      <c r="F132" s="1"/>
+      <c r="G132" s="1"/>
+      <c r="H132" s="8"/>
+      <c r="I132" s="1"/>
+      <c r="J132" s="1"/>
+      <c r="K132" s="1"/>
+      <c r="L132" s="1"/>
+      <c r="M132" s="1"/>
+      <c r="N132" s="1"/>
+      <c r="O132" s="7"/>
+      <c r="P132" s="7"/>
+      <c r="Q132" s="7"/>
+      <c r="R132" s="7"/>
+      <c r="S132" s="7"/>
+      <c r="T132" s="7"/>
+      <c r="U132" s="7"/>
+      <c r="V132" s="7"/>
+      <c r="W132" s="7"/>
+      <c r="X132" s="7"/>
+      <c r="Y132" s="7"/>
+      <c r="Z132" s="7"/>
+      <c r="AA132" s="7"/>
+      <c r="AB132" s="7"/>
+      <c r="AC132" s="7"/>
+      <c r="AD132" s="7"/>
+      <c r="AE132" s="7"/>
+      <c r="AF132" s="7"/>
+      <c r="AG132" s="7"/>
+      <c r="AH132" s="7"/>
+      <c r="AI132" s="7"/>
+      <c r="AJ132" s="7"/>
+      <c r="AK132" s="7"/>
+      <c r="AL132" s="7"/>
+      <c r="AM132" s="7"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="E6:E87">
+  <conditionalFormatting sqref="E6:E132">
     <cfRule type="containsBlanks" dxfId="3" priority="1">
       <formula>LEN(TRIM(E6))=0</formula>
     </cfRule>
@@ -6095,7 +8325,7 @@
       <formula>NOT(ISERROR(SEARCH("x",E6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F87">
+  <conditionalFormatting sqref="F6:F132">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
@@ -6104,20 +8334,21 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D87 J6:J87" xr:uid="{CD5956F3-4E0A-44DB-A8DC-925168F89EE9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D132 J6:J132" xr:uid="{CD5956F3-4E0A-44DB-A8DC-925168F89EE9}">
       <formula1>INDIRECT("ExpressionsList[Expressions]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T87 AA6:AA87 AH6:AH87 M6 M8:M20" xr:uid="{F01B3C1A-78E2-4F4D-B484-DA9ABA464973}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T132 AA6:AA132 AH6:AH132 M6 M8:M20" xr:uid="{F01B3C1A-78E2-4F4D-B484-DA9ABA464973}">
       <formula1>INDIRECT("ConditionalsList[Conditionals]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C87 K6:K87" xr:uid="{3FFEAF7F-218C-4ED0-9224-5256A4750AA6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C132 K6:K132" xr:uid="{3FFEAF7F-218C-4ED0-9224-5256A4750AA6}">
       <formula1>INDIRECT("CharactersList[Characters]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6125,14 +8356,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EDBD295-5C93-44DD-9985-3C1BB495EB4B}">
   <dimension ref="B2:F11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.25" customWidth="1"/>
+    <col min="4" max="4" width="14.125" customWidth="1"/>
+    <col min="6" max="6" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -6143,7 +8374,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6">
       <c r="B3" t="s">
         <v>16</v>
       </c>
@@ -6154,7 +8385,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -6165,7 +8396,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6">
       <c r="B5" t="s">
         <v>41</v>
       </c>
@@ -6176,7 +8407,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6">
       <c r="B6" t="s">
         <v>20</v>
       </c>
@@ -6184,7 +8415,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6">
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -6192,7 +8423,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6">
       <c r="B8" t="s">
         <v>18</v>
       </c>
@@ -6200,7 +8431,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6">
       <c r="B9" t="s">
         <v>19</v>
       </c>
@@ -6208,12 +8439,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6">
       <c r="B10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6">
       <c r="B11" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
switching over to another computer to finish up
</commit_message>
<xml_diff>
--- a/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
+++ b/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\papadoal\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damon\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB375D9-647B-4BB0-9F58-31BE6DB42B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEABD923-7315-4D64-8DA7-E2807B76D3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="201">
   <si>
     <t>Dialogue Enter</t>
   </si>
@@ -649,7 +649,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -728,41 +728,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="43">
     <dxf>
       <fill>
         <patternFill>
@@ -1250,50 +1216,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM132" totalsRowShown="0" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM132" totalsRowShown="0" dataDxfId="42">
   <autoFilter ref="B5:AM132" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:AM20">
     <sortCondition ref="B5:B20"/>
   </sortState>
   <tableColumns count="38">
-    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="45"/>
-    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="43"/>
-    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="42"/>
-    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="41"/>
-    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="36"/>
-    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="35"/>
-    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="34"/>
-    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="32"/>
-    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="31"/>
-    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="30"/>
-    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="29"/>
-    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="28"/>
-    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="27"/>
-    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="26"/>
-    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="25"/>
-    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="24"/>
-    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="23"/>
-    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="22"/>
-    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="21"/>
-    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="20"/>
-    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="19"/>
-    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="18"/>
-    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="17"/>
-    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="16"/>
-    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="15"/>
-    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="14"/>
-    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="13"/>
-    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="12"/>
-    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="11"/>
-    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="10"/>
-    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="9"/>
-    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="8"/>
+    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="39"/>
+    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="38"/>
+    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="32"/>
+    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="31"/>
+    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="30"/>
+    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="28"/>
+    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="27"/>
+    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="26"/>
+    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="25"/>
+    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="24"/>
+    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="23"/>
+    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="22"/>
+    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="21"/>
+    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="20"/>
+    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="19"/>
+    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="18"/>
+    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="17"/>
+    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="16"/>
+    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="15"/>
+    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="14"/>
+    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="13"/>
+    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="12"/>
+    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="11"/>
+    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="10"/>
+    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="9"/>
+    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="8"/>
+    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="7"/>
+    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="6"/>
+    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="5"/>
+    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1650,38 +1616,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AD6004-D6D5-49E8-98E5-3900A70D687C}">
   <dimension ref="B4:AM132"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.875" customWidth="1"/>
-    <col min="2" max="2" width="8.625" customWidth="1"/>
-    <col min="3" max="3" width="15.75" customWidth="1"/>
-    <col min="4" max="7" width="14.75" customWidth="1"/>
-    <col min="8" max="8" width="60.75" customWidth="1"/>
-    <col min="9" max="10" width="14.75" customWidth="1"/>
-    <col min="11" max="14" width="15.75" customWidth="1"/>
-    <col min="15" max="15" width="20.75" customWidth="1"/>
-    <col min="16" max="16" width="18.75" customWidth="1"/>
-    <col min="17" max="17" width="15.75" customWidth="1"/>
-    <col min="18" max="18" width="14.75" customWidth="1"/>
-    <col min="19" max="21" width="15.75" customWidth="1"/>
-    <col min="22" max="22" width="20.75" customWidth="1"/>
-    <col min="23" max="23" width="18.75" customWidth="1"/>
-    <col min="24" max="24" width="15.75" customWidth="1"/>
-    <col min="25" max="25" width="14.75" customWidth="1"/>
-    <col min="26" max="28" width="15.75" customWidth="1"/>
-    <col min="29" max="29" width="20.75" customWidth="1"/>
-    <col min="30" max="30" width="18.75" customWidth="1"/>
-    <col min="31" max="31" width="15.75" customWidth="1"/>
-    <col min="32" max="32" width="14.75" customWidth="1"/>
-    <col min="33" max="35" width="15.75" customWidth="1"/>
-    <col min="36" max="36" width="20.75" customWidth="1"/>
-    <col min="37" max="37" width="18.75" customWidth="1"/>
-    <col min="38" max="38" width="15.75" customWidth="1"/>
-    <col min="39" max="39" width="14.75" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" customWidth="1"/>
+    <col min="4" max="7" width="14.77734375" customWidth="1"/>
+    <col min="8" max="8" width="60.77734375" customWidth="1"/>
+    <col min="9" max="10" width="14.77734375" customWidth="1"/>
+    <col min="11" max="14" width="15.77734375" customWidth="1"/>
+    <col min="15" max="15" width="20.77734375" customWidth="1"/>
+    <col min="16" max="16" width="18.77734375" customWidth="1"/>
+    <col min="17" max="17" width="15.77734375" customWidth="1"/>
+    <col min="18" max="18" width="14.77734375" customWidth="1"/>
+    <col min="19" max="21" width="15.77734375" customWidth="1"/>
+    <col min="22" max="22" width="20.77734375" customWidth="1"/>
+    <col min="23" max="23" width="18.77734375" customWidth="1"/>
+    <col min="24" max="24" width="15.77734375" customWidth="1"/>
+    <col min="25" max="25" width="14.77734375" customWidth="1"/>
+    <col min="26" max="28" width="15.77734375" customWidth="1"/>
+    <col min="29" max="29" width="20.77734375" customWidth="1"/>
+    <col min="30" max="30" width="18.77734375" customWidth="1"/>
+    <col min="31" max="31" width="15.77734375" customWidth="1"/>
+    <col min="32" max="32" width="14.77734375" customWidth="1"/>
+    <col min="33" max="35" width="15.77734375" customWidth="1"/>
+    <col min="36" max="36" width="20.77734375" customWidth="1"/>
+    <col min="37" max="37" width="18.77734375" customWidth="1"/>
+    <col min="38" max="38" width="15.77734375" customWidth="1"/>
+    <col min="39" max="39" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:39" ht="88.9" customHeight="1"/>
-    <row r="5" spans="2:39">
+    <row r="4" spans="2:39" ht="88.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>22</v>
       </c>
@@ -1797,7 +1763,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:39" ht="28.5">
+    <row r="6" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>0</v>
       </c>
@@ -1851,7 +1817,7 @@
       <c r="AL6" s="7"/>
       <c r="AM6" s="7"/>
     </row>
-    <row r="7" spans="2:39" ht="28.5">
+    <row r="7" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <f t="shared" ref="B7:B70" si="0">1+B6</f>
         <v>1</v>
@@ -1906,7 +1872,7 @@
       <c r="AL7" s="7"/>
       <c r="AM7" s="7"/>
     </row>
-    <row r="8" spans="2:39" ht="28.5">
+    <row r="8" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1959,7 +1925,7 @@
       <c r="AL8" s="7"/>
       <c r="AM8" s="7"/>
     </row>
-    <row r="9" spans="2:39" ht="42.75">
+    <row r="9" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -2014,7 +1980,7 @@
       <c r="AL9" s="7"/>
       <c r="AM9" s="7"/>
     </row>
-    <row r="10" spans="2:39" ht="28.5">
+    <row r="10" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2073,7 +2039,7 @@
       <c r="AL10" s="7"/>
       <c r="AM10" s="7"/>
     </row>
-    <row r="11" spans="2:39">
+    <row r="11" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2130,7 +2096,7 @@
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
     </row>
-    <row r="12" spans="2:39" ht="42.75">
+    <row r="12" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2183,7 +2149,7 @@
       <c r="AL12" s="7"/>
       <c r="AM12" s="7"/>
     </row>
-    <row r="13" spans="2:39" ht="28.5">
+    <row r="13" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2236,7 +2202,7 @@
       <c r="AL13" s="7"/>
       <c r="AM13" s="7"/>
     </row>
-    <row r="14" spans="2:39">
+    <row r="14" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2291,7 +2257,7 @@
       <c r="AL14" s="7"/>
       <c r="AM14" s="7"/>
     </row>
-    <row r="15" spans="2:39" ht="28.5">
+    <row r="15" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2356,7 +2322,7 @@
       <c r="AL15" s="7"/>
       <c r="AM15" s="7"/>
     </row>
-    <row r="16" spans="2:39">
+    <row r="16" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2413,7 +2379,7 @@
       <c r="AL16" s="7"/>
       <c r="AM16" s="7"/>
     </row>
-    <row r="17" spans="2:39" ht="28.5">
+    <row r="17" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2468,7 +2434,7 @@
       <c r="AL17" s="7"/>
       <c r="AM17" s="7"/>
     </row>
-    <row r="18" spans="2:39">
+    <row r="18" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B18" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2525,7 +2491,7 @@
       <c r="AL18" s="7"/>
       <c r="AM18" s="7"/>
     </row>
-    <row r="19" spans="2:39" ht="28.5">
+    <row r="19" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B19" s="1">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2582,7 +2548,7 @@
       <c r="AL19" s="7"/>
       <c r="AM19" s="7"/>
     </row>
-    <row r="20" spans="2:39">
+    <row r="20" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2637,7 +2603,7 @@
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
     </row>
-    <row r="21" spans="2:39">
+    <row r="21" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B21" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2690,7 +2656,7 @@
       <c r="AL21" s="7"/>
       <c r="AM21" s="7"/>
     </row>
-    <row r="22" spans="2:39" ht="42.75">
+    <row r="22" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2743,7 +2709,7 @@
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
     </row>
-    <row r="23" spans="2:39" ht="28.5">
+    <row r="23" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2796,7 +2762,7 @@
       <c r="AL23" s="7"/>
       <c r="AM23" s="7"/>
     </row>
-    <row r="24" spans="2:39">
+    <row r="24" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B24" s="1">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2849,7 +2815,7 @@
       <c r="AL24" s="7"/>
       <c r="AM24" s="7"/>
     </row>
-    <row r="25" spans="2:39" ht="28.5">
+    <row r="25" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B25" s="1">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2926,7 +2892,7 @@
       <c r="AL25" s="7"/>
       <c r="AM25" s="7"/>
     </row>
-    <row r="26" spans="2:39">
+    <row r="26" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B26" s="1">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2983,7 +2949,7 @@
       <c r="AL26" s="7"/>
       <c r="AM26" s="7"/>
     </row>
-    <row r="27" spans="2:39" ht="28.5">
+    <row r="27" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B27" s="1">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3036,7 +3002,7 @@
       <c r="AL27" s="7"/>
       <c r="AM27" s="7"/>
     </row>
-    <row r="28" spans="2:39">
+    <row r="28" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B28" s="1">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3091,7 +3057,7 @@
       <c r="AL28" s="7"/>
       <c r="AM28" s="7"/>
     </row>
-    <row r="29" spans="2:39">
+    <row r="29" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B29" s="1">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3146,7 +3112,7 @@
       <c r="AL29" s="7"/>
       <c r="AM29" s="7"/>
     </row>
-    <row r="30" spans="2:39">
+    <row r="30" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B30" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3201,7 +3167,7 @@
       <c r="AL30" s="7"/>
       <c r="AM30" s="7"/>
     </row>
-    <row r="31" spans="2:39">
+    <row r="31" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B31" s="1">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3256,7 +3222,7 @@
       <c r="AL31" s="7"/>
       <c r="AM31" s="7"/>
     </row>
-    <row r="32" spans="2:39">
+    <row r="32" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3309,7 +3275,7 @@
       <c r="AL32" s="7"/>
       <c r="AM32" s="7"/>
     </row>
-    <row r="33" spans="2:39">
+    <row r="33" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3364,7 +3330,7 @@
       <c r="AL33" s="7"/>
       <c r="AM33" s="7"/>
     </row>
-    <row r="34" spans="2:39">
+    <row r="34" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B34" s="1">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3419,7 +3385,7 @@
       <c r="AL34" s="7"/>
       <c r="AM34" s="7"/>
     </row>
-    <row r="35" spans="2:39" ht="28.5">
+    <row r="35" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B35" s="1">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3474,7 +3440,7 @@
       <c r="AL35" s="7"/>
       <c r="AM35" s="7"/>
     </row>
-    <row r="36" spans="2:39">
+    <row r="36" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3527,7 +3493,7 @@
       <c r="AL36" s="7"/>
       <c r="AM36" s="7"/>
     </row>
-    <row r="37" spans="2:39">
+    <row r="37" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B37" s="1">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3582,7 +3548,7 @@
       <c r="AL37" s="7"/>
       <c r="AM37" s="7"/>
     </row>
-    <row r="38" spans="2:39">
+    <row r="38" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B38" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3635,7 +3601,7 @@
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
     </row>
-    <row r="39" spans="2:39">
+    <row r="39" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B39" s="1">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3690,7 +3656,7 @@
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
     </row>
-    <row r="40" spans="2:39" ht="28.5">
+    <row r="40" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B40" s="1">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3743,7 +3709,7 @@
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
     </row>
-    <row r="41" spans="2:39" ht="28.5">
+    <row r="41" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B41" s="1">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3796,7 +3762,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
     </row>
-    <row r="42" spans="2:39" ht="28.5">
+    <row r="42" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B42" s="1">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3851,7 +3817,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
     </row>
-    <row r="43" spans="2:39">
+    <row r="43" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B43" s="1">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3904,7 +3870,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
     </row>
-    <row r="44" spans="2:39">
+    <row r="44" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B44" s="1">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3973,7 +3939,7 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
     </row>
-    <row r="45" spans="2:39">
+    <row r="45" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B45" s="1">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -4030,7 +3996,7 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
     </row>
-    <row r="46" spans="2:39" ht="28.5">
+    <row r="46" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B46" s="1">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -4085,7 +4051,7 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
     </row>
-    <row r="47" spans="2:39" ht="42.75">
+    <row r="47" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B47" s="1">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -4140,7 +4106,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
     </row>
-    <row r="48" spans="2:39">
+    <row r="48" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B48" s="1">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -4195,7 +4161,7 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
     </row>
-    <row r="49" spans="2:39" ht="28.5">
+    <row r="49" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B49" s="1">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -4250,7 +4216,7 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
     </row>
-    <row r="50" spans="2:39" ht="42.75">
+    <row r="50" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B50" s="1">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -4305,7 +4271,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
     </row>
-    <row r="51" spans="2:39" ht="28.5">
+    <row r="51" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B51" s="1">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -4358,7 +4324,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
     </row>
-    <row r="52" spans="2:39">
+    <row r="52" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B52" s="1">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -4413,7 +4379,7 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
     </row>
-    <row r="53" spans="2:39" ht="28.5">
+    <row r="53" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B53" s="1">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -4466,7 +4432,7 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
     </row>
-    <row r="54" spans="2:39" ht="28.5">
+    <row r="54" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B54" s="1">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -4521,7 +4487,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
     </row>
-    <row r="55" spans="2:39" ht="42.75">
+    <row r="55" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B55" s="1">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -4574,7 +4540,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
     </row>
-    <row r="56" spans="2:39" ht="28.5">
+    <row r="56" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B56" s="1">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -4651,7 +4617,7 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
     </row>
-    <row r="57" spans="2:39" ht="28.5">
+    <row r="57" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B57" s="1">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -4706,7 +4672,7 @@
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
     </row>
-    <row r="58" spans="2:39">
+    <row r="58" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B58" s="1">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -4761,7 +4727,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
     </row>
-    <row r="59" spans="2:39">
+    <row r="59" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B59" s="1">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -4816,7 +4782,7 @@
       <c r="AL59" s="7"/>
       <c r="AM59" s="7"/>
     </row>
-    <row r="60" spans="2:39">
+    <row r="60" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B60" s="1">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -4871,7 +4837,7 @@
       <c r="AL60" s="7"/>
       <c r="AM60" s="7"/>
     </row>
-    <row r="61" spans="2:39">
+    <row r="61" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B61" s="1">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -4928,7 +4894,7 @@
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
     </row>
-    <row r="62" spans="2:39">
+    <row r="62" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B62" s="1">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -4985,7 +4951,7 @@
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
     </row>
-    <row r="63" spans="2:39">
+    <row r="63" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B63" s="1">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -5048,7 +5014,7 @@
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
     </row>
-    <row r="64" spans="2:39">
+    <row r="64" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B64" s="1">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -5099,7 +5065,7 @@
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
     </row>
-    <row r="65" spans="2:39" ht="42.75">
+    <row r="65" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B65" s="1">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -5154,7 +5120,7 @@
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
     </row>
-    <row r="66" spans="2:39" ht="42.75">
+    <row r="66" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B66" s="1">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -5207,7 +5173,7 @@
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
     </row>
-    <row r="67" spans="2:39" ht="28.5">
+    <row r="67" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B67" s="1">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -5260,7 +5226,7 @@
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
     </row>
-    <row r="68" spans="2:39" ht="28.5">
+    <row r="68" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B68" s="1">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -5313,7 +5279,7 @@
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
     </row>
-    <row r="69" spans="2:39" ht="42.75">
+    <row r="69" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B69" s="1">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -5366,7 +5332,7 @@
       <c r="AL69" s="7"/>
       <c r="AM69" s="7"/>
     </row>
-    <row r="70" spans="2:39" ht="28.5">
+    <row r="70" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B70" s="1">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -5419,7 +5385,7 @@
       <c r="AL70" s="7"/>
       <c r="AM70" s="7"/>
     </row>
-    <row r="71" spans="2:39" ht="28.5">
+    <row r="71" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B71" s="1">
         <f t="shared" ref="B71:B132" si="1">1+B70</f>
         <v>65</v>
@@ -5472,7 +5438,7 @@
       <c r="AL71" s="7"/>
       <c r="AM71" s="7"/>
     </row>
-    <row r="72" spans="2:39" ht="42.75">
+    <row r="72" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B72" s="1">
         <f t="shared" si="1"/>
         <v>66</v>
@@ -5525,7 +5491,7 @@
       <c r="AL72" s="7"/>
       <c r="AM72" s="7"/>
     </row>
-    <row r="73" spans="2:39" ht="28.5">
+    <row r="73" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B73" s="1">
         <f t="shared" si="1"/>
         <v>67</v>
@@ -5578,7 +5544,7 @@
       <c r="AL73" s="7"/>
       <c r="AM73" s="7"/>
     </row>
-    <row r="74" spans="2:39" ht="42.75">
+    <row r="74" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B74" s="1">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -5631,7 +5597,7 @@
       <c r="AL74" s="7"/>
       <c r="AM74" s="7"/>
     </row>
-    <row r="75" spans="2:39" ht="28.5">
+    <row r="75" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B75" s="1">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -5684,7 +5650,7 @@
       <c r="AL75" s="7"/>
       <c r="AM75" s="7"/>
     </row>
-    <row r="76" spans="2:39" ht="28.5">
+    <row r="76" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B76" s="1">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -5737,7 +5703,7 @@
       <c r="AL76" s="7"/>
       <c r="AM76" s="7"/>
     </row>
-    <row r="77" spans="2:39" ht="28.5">
+    <row r="77" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B77" s="1">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -5790,7 +5756,7 @@
       <c r="AL77" s="7"/>
       <c r="AM77" s="7"/>
     </row>
-    <row r="78" spans="2:39" ht="28.5">
+    <row r="78" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B78" s="1">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -5843,7 +5809,7 @@
       <c r="AL78" s="7"/>
       <c r="AM78" s="7"/>
     </row>
-    <row r="79" spans="2:39" ht="28.5">
+    <row r="79" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B79" s="1">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -5896,7 +5862,7 @@
       <c r="AL79" s="7"/>
       <c r="AM79" s="7"/>
     </row>
-    <row r="80" spans="2:39">
+    <row r="80" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B80" s="1">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -5949,7 +5915,7 @@
       <c r="AL80" s="7"/>
       <c r="AM80" s="7"/>
     </row>
-    <row r="81" spans="2:39">
+    <row r="81" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B81" s="1">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -6002,7 +5968,7 @@
       <c r="AL81" s="7"/>
       <c r="AM81" s="7"/>
     </row>
-    <row r="82" spans="2:39" ht="28.5">
+    <row r="82" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B82" s="1">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -6055,7 +6021,7 @@
       <c r="AL82" s="7"/>
       <c r="AM82" s="7"/>
     </row>
-    <row r="83" spans="2:39" ht="42.75">
+    <row r="83" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B83" s="1">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -6108,7 +6074,7 @@
       <c r="AL83" s="7"/>
       <c r="AM83" s="7"/>
     </row>
-    <row r="84" spans="2:39">
+    <row r="84" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B84" s="1">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -6161,7 +6127,7 @@
       <c r="AL84" s="7"/>
       <c r="AM84" s="7"/>
     </row>
-    <row r="85" spans="2:39" ht="28.5">
+    <row r="85" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B85" s="1">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -6214,7 +6180,7 @@
       <c r="AL85" s="7"/>
       <c r="AM85" s="7"/>
     </row>
-    <row r="86" spans="2:39">
+    <row r="86" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B86" s="1">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -6267,7 +6233,7 @@
       <c r="AL86" s="7"/>
       <c r="AM86" s="7"/>
     </row>
-    <row r="87" spans="2:39" ht="28.5">
+    <row r="87" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B87" s="1">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -6320,13 +6286,17 @@
       <c r="AL87" s="7"/>
       <c r="AM87" s="7"/>
     </row>
-    <row r="88" spans="2:39">
+    <row r="88" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B88" s="1">
         <f t="shared" si="1"/>
         <v>82</v>
       </c>
-      <c r="C88" s="1"/>
-      <c r="D88" s="1"/>
+      <c r="C88" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
@@ -6334,8 +6304,12 @@
         <v>175</v>
       </c>
       <c r="I88" s="1"/>
-      <c r="J88" s="1"/>
-      <c r="K88" s="1"/>
+      <c r="J88" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L88" s="1"/>
       <c r="M88" s="1"/>
       <c r="N88" s="1"/>
@@ -6365,13 +6339,17 @@
       <c r="AL88" s="7"/>
       <c r="AM88" s="7"/>
     </row>
-    <row r="89" spans="2:39" ht="42.75">
+    <row r="89" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B89" s="1">
         <f t="shared" si="1"/>
         <v>83</v>
       </c>
-      <c r="C89" s="1"/>
-      <c r="D89" s="1"/>
+      <c r="C89" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
@@ -6379,8 +6357,12 @@
         <v>174</v>
       </c>
       <c r="I89" s="1"/>
-      <c r="J89" s="1"/>
-      <c r="K89" s="1"/>
+      <c r="J89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L89" s="1"/>
       <c r="M89" s="1"/>
       <c r="N89" s="1"/>
@@ -6410,13 +6392,17 @@
       <c r="AL89" s="7"/>
       <c r="AM89" s="7"/>
     </row>
-    <row r="90" spans="2:39" ht="28.5">
+    <row r="90" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B90" s="1">
         <f t="shared" si="1"/>
         <v>84</v>
       </c>
-      <c r="C90" s="1"/>
-      <c r="D90" s="1"/>
+      <c r="C90" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
@@ -6424,8 +6410,12 @@
         <v>176</v>
       </c>
       <c r="I90" s="1"/>
-      <c r="J90" s="1"/>
-      <c r="K90" s="1"/>
+      <c r="J90" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L90" s="1"/>
       <c r="M90" s="1"/>
       <c r="N90" s="1"/>
@@ -6455,13 +6445,17 @@
       <c r="AL90" s="7"/>
       <c r="AM90" s="7"/>
     </row>
-    <row r="91" spans="2:39">
+    <row r="91" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B91" s="1">
         <f t="shared" si="1"/>
         <v>85</v>
       </c>
-      <c r="C91" s="1"/>
-      <c r="D91" s="1"/>
+      <c r="C91" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
@@ -6469,8 +6463,12 @@
         <v>177</v>
       </c>
       <c r="I91" s="1"/>
-      <c r="J91" s="1"/>
-      <c r="K91" s="1"/>
+      <c r="J91" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L91" s="1"/>
       <c r="M91" s="1"/>
       <c r="N91" s="1"/>
@@ -6500,13 +6498,17 @@
       <c r="AL91" s="7"/>
       <c r="AM91" s="7"/>
     </row>
-    <row r="92" spans="2:39">
+    <row r="92" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B92" s="1">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-      <c r="C92" s="1"/>
-      <c r="D92" s="1"/>
+      <c r="C92" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
@@ -6514,8 +6516,12 @@
         <v>178</v>
       </c>
       <c r="I92" s="1"/>
-      <c r="J92" s="1"/>
-      <c r="K92" s="1"/>
+      <c r="J92" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L92" s="1"/>
       <c r="M92" s="1"/>
       <c r="N92" s="1"/>
@@ -6545,13 +6551,17 @@
       <c r="AL92" s="7"/>
       <c r="AM92" s="7"/>
     </row>
-    <row r="93" spans="2:39" ht="28.5">
+    <row r="93" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B93" s="1">
         <f t="shared" si="1"/>
         <v>87</v>
       </c>
-      <c r="C93" s="1"/>
-      <c r="D93" s="1"/>
+      <c r="C93" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
@@ -6559,8 +6569,12 @@
         <v>179</v>
       </c>
       <c r="I93" s="1"/>
-      <c r="J93" s="1"/>
-      <c r="K93" s="1"/>
+      <c r="J93" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L93" s="1"/>
       <c r="M93" s="1"/>
       <c r="N93" s="1"/>
@@ -6590,13 +6604,17 @@
       <c r="AL93" s="7"/>
       <c r="AM93" s="7"/>
     </row>
-    <row r="94" spans="2:39" ht="28.5">
+    <row r="94" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B94" s="1">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="C94" s="1"/>
-      <c r="D94" s="1"/>
+      <c r="C94" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
@@ -6604,8 +6622,12 @@
         <v>180</v>
       </c>
       <c r="I94" s="1"/>
-      <c r="J94" s="1"/>
-      <c r="K94" s="1"/>
+      <c r="J94" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K94" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L94" s="1"/>
       <c r="M94" s="1"/>
       <c r="N94" s="1"/>
@@ -6635,13 +6657,17 @@
       <c r="AL94" s="7"/>
       <c r="AM94" s="7"/>
     </row>
-    <row r="95" spans="2:39" ht="42.75">
+    <row r="95" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B95" s="1">
         <f t="shared" si="1"/>
         <v>89</v>
       </c>
-      <c r="C95" s="1"/>
-      <c r="D95" s="1"/>
+      <c r="C95" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
@@ -6649,8 +6675,12 @@
         <v>181</v>
       </c>
       <c r="I95" s="1"/>
-      <c r="J95" s="1"/>
-      <c r="K95" s="1"/>
+      <c r="J95" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L95" s="1"/>
       <c r="M95" s="1"/>
       <c r="N95" s="1"/>
@@ -6680,13 +6710,17 @@
       <c r="AL95" s="7"/>
       <c r="AM95" s="7"/>
     </row>
-    <row r="96" spans="2:39" ht="28.5">
+    <row r="96" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B96" s="1">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="C96" s="1"/>
-      <c r="D96" s="1"/>
+      <c r="C96" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
       <c r="G96" s="1"/>
@@ -6694,8 +6728,12 @@
         <v>182</v>
       </c>
       <c r="I96" s="1"/>
-      <c r="J96" s="1"/>
-      <c r="K96" s="1"/>
+      <c r="J96" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L96" s="1"/>
       <c r="M96" s="1"/>
       <c r="N96" s="1"/>
@@ -6725,13 +6763,17 @@
       <c r="AL96" s="7"/>
       <c r="AM96" s="7"/>
     </row>
-    <row r="97" spans="2:39">
+    <row r="97" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B97" s="1">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
-      <c r="C97" s="1"/>
-      <c r="D97" s="1"/>
+      <c r="C97" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
       <c r="G97" s="1"/>
@@ -6739,8 +6781,12 @@
         <v>183</v>
       </c>
       <c r="I97" s="1"/>
-      <c r="J97" s="1"/>
-      <c r="K97" s="1"/>
+      <c r="J97" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L97" s="1"/>
       <c r="M97" s="1"/>
       <c r="N97" s="1"/>
@@ -6770,13 +6816,17 @@
       <c r="AL97" s="7"/>
       <c r="AM97" s="7"/>
     </row>
-    <row r="98" spans="2:39" ht="28.5">
+    <row r="98" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B98" s="1">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
-      <c r="C98" s="1"/>
-      <c r="D98" s="1"/>
+      <c r="C98" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
       <c r="G98" s="1"/>
@@ -6784,8 +6834,12 @@
         <v>184</v>
       </c>
       <c r="I98" s="1"/>
-      <c r="J98" s="1"/>
-      <c r="K98" s="1"/>
+      <c r="J98" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L98" s="1"/>
       <c r="M98" s="1"/>
       <c r="N98" s="1"/>
@@ -6815,13 +6869,17 @@
       <c r="AL98" s="7"/>
       <c r="AM98" s="7"/>
     </row>
-    <row r="99" spans="2:39" ht="28.5">
+    <row r="99" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B99" s="1">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
+      <c r="C99" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
       <c r="G99" s="1"/>
@@ -6829,8 +6887,12 @@
         <v>185</v>
       </c>
       <c r="I99" s="1"/>
-      <c r="J99" s="1"/>
-      <c r="K99" s="1"/>
+      <c r="J99" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L99" s="1"/>
       <c r="M99" s="1"/>
       <c r="N99" s="1"/>
@@ -6860,13 +6922,17 @@
       <c r="AL99" s="7"/>
       <c r="AM99" s="7"/>
     </row>
-    <row r="100" spans="2:39">
+    <row r="100" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B100" s="1">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1"/>
+      <c r="C100" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
@@ -6874,8 +6940,12 @@
         <v>186</v>
       </c>
       <c r="I100" s="1"/>
-      <c r="J100" s="1"/>
-      <c r="K100" s="1"/>
+      <c r="J100" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L100" s="1"/>
       <c r="M100" s="1"/>
       <c r="N100" s="1"/>
@@ -6905,13 +6975,17 @@
       <c r="AL100" s="7"/>
       <c r="AM100" s="7"/>
     </row>
-    <row r="101" spans="2:39" ht="28.5">
+    <row r="101" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B101" s="1">
         <f t="shared" si="1"/>
         <v>95</v>
       </c>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
+      <c r="C101" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
@@ -6919,8 +6993,12 @@
         <v>187</v>
       </c>
       <c r="I101" s="1"/>
-      <c r="J101" s="1"/>
-      <c r="K101" s="1"/>
+      <c r="J101" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L101" s="1"/>
       <c r="M101" s="1"/>
       <c r="N101" s="1"/>
@@ -6950,13 +7028,17 @@
       <c r="AL101" s="7"/>
       <c r="AM101" s="7"/>
     </row>
-    <row r="102" spans="2:39" ht="42.75">
+    <row r="102" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B102" s="1">
         <f t="shared" si="1"/>
         <v>96</v>
       </c>
-      <c r="C102" s="1"/>
-      <c r="D102" s="1"/>
+      <c r="C102" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
       <c r="G102" s="1"/>
@@ -6964,8 +7046,12 @@
         <v>188</v>
       </c>
       <c r="I102" s="1"/>
-      <c r="J102" s="1"/>
-      <c r="K102" s="1"/>
+      <c r="J102" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K102" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L102" s="1"/>
       <c r="M102" s="1"/>
       <c r="N102" s="1"/>
@@ -6995,13 +7081,17 @@
       <c r="AL102" s="7"/>
       <c r="AM102" s="7"/>
     </row>
-    <row r="103" spans="2:39" ht="28.5">
+    <row r="103" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B103" s="1">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="C103" s="1"/>
-      <c r="D103" s="1"/>
+      <c r="C103" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
@@ -7009,8 +7099,12 @@
         <v>189</v>
       </c>
       <c r="I103" s="1"/>
-      <c r="J103" s="1"/>
-      <c r="K103" s="1"/>
+      <c r="J103" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L103" s="1"/>
       <c r="M103" s="1"/>
       <c r="N103" s="1"/>
@@ -7040,13 +7134,17 @@
       <c r="AL103" s="7"/>
       <c r="AM103" s="7"/>
     </row>
-    <row r="104" spans="2:39" ht="42.75">
+    <row r="104" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B104" s="1">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-      <c r="C104" s="1"/>
-      <c r="D104" s="1"/>
+      <c r="C104" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E104" s="1"/>
       <c r="F104" s="1" t="s">
         <v>2</v>
@@ -7056,8 +7154,12 @@
         <v>190</v>
       </c>
       <c r="I104" s="1"/>
-      <c r="J104" s="1"/>
-      <c r="K104" s="1"/>
+      <c r="J104" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K104" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L104" s="1"/>
       <c r="M104" s="1"/>
       <c r="N104" s="1"/>
@@ -7087,20 +7189,28 @@
       <c r="AL104" s="7"/>
       <c r="AM104" s="7"/>
     </row>
-    <row r="105" spans="2:39">
+    <row r="105" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B105" s="1">
         <f t="shared" si="1"/>
         <v>99</v>
       </c>
-      <c r="C105" s="1"/>
-      <c r="D105" s="1"/>
+      <c r="C105" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
       <c r="G105" s="1"/>
       <c r="H105" s="8"/>
       <c r="I105" s="1"/>
-      <c r="J105" s="1"/>
-      <c r="K105" s="1"/>
+      <c r="J105" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K105" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L105" s="1"/>
       <c r="M105" s="1"/>
       <c r="N105" s="1"/>
@@ -7130,13 +7240,17 @@
       <c r="AL105" s="7"/>
       <c r="AM105" s="7"/>
     </row>
-    <row r="106" spans="2:39">
+    <row r="106" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B106" s="1">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="C106" s="1"/>
-      <c r="D106" s="1"/>
+      <c r="C106" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
       <c r="G106" s="1" t="s">
@@ -7146,8 +7260,12 @@
         <v>192</v>
       </c>
       <c r="I106" s="1"/>
-      <c r="J106" s="1"/>
-      <c r="K106" s="1"/>
+      <c r="J106" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K106" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L106" s="1"/>
       <c r="M106" s="1"/>
       <c r="N106" s="1"/>
@@ -7177,13 +7295,17 @@
       <c r="AL106" s="7"/>
       <c r="AM106" s="7"/>
     </row>
-    <row r="107" spans="2:39" ht="28.5">
+    <row r="107" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B107" s="1">
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
-      <c r="C107" s="1"/>
-      <c r="D107" s="1"/>
+      <c r="C107" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
@@ -7191,8 +7313,12 @@
         <v>193</v>
       </c>
       <c r="I107" s="1"/>
-      <c r="J107" s="1"/>
-      <c r="K107" s="1"/>
+      <c r="J107" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K107" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L107" s="1"/>
       <c r="M107" s="1"/>
       <c r="N107" s="1"/>
@@ -7222,13 +7348,17 @@
       <c r="AL107" s="7"/>
       <c r="AM107" s="7"/>
     </row>
-    <row r="108" spans="2:39">
+    <row r="108" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B108" s="1">
         <f t="shared" si="1"/>
         <v>102</v>
       </c>
-      <c r="C108" s="1"/>
-      <c r="D108" s="1"/>
+      <c r="C108" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
@@ -7236,8 +7366,12 @@
         <v>194</v>
       </c>
       <c r="I108" s="1"/>
-      <c r="J108" s="1"/>
-      <c r="K108" s="1"/>
+      <c r="J108" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K108" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L108" s="1"/>
       <c r="M108" s="1"/>
       <c r="N108" s="1"/>
@@ -7267,13 +7401,17 @@
       <c r="AL108" s="7"/>
       <c r="AM108" s="7"/>
     </row>
-    <row r="109" spans="2:39" ht="28.5">
+    <row r="109" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B109" s="1">
         <f t="shared" si="1"/>
         <v>103</v>
       </c>
-      <c r="C109" s="1"/>
-      <c r="D109" s="1"/>
+      <c r="C109" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
       <c r="G109" s="1"/>
@@ -7281,8 +7419,12 @@
         <v>195</v>
       </c>
       <c r="I109" s="1"/>
-      <c r="J109" s="1"/>
-      <c r="K109" s="1"/>
+      <c r="J109" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K109" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L109" s="1"/>
       <c r="M109" s="1"/>
       <c r="N109" s="1"/>
@@ -7312,13 +7454,17 @@
       <c r="AL109" s="7"/>
       <c r="AM109" s="7"/>
     </row>
-    <row r="110" spans="2:39" ht="28.5">
+    <row r="110" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B110" s="1">
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
-      <c r="C110" s="1"/>
-      <c r="D110" s="1"/>
+      <c r="C110" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
       <c r="G110" s="1"/>
@@ -7326,8 +7472,12 @@
         <v>195</v>
       </c>
       <c r="I110" s="1"/>
-      <c r="J110" s="1"/>
-      <c r="K110" s="1"/>
+      <c r="J110" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K110" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L110" s="1"/>
       <c r="M110" s="1"/>
       <c r="N110" s="1"/>
@@ -7357,13 +7507,17 @@
       <c r="AL110" s="7"/>
       <c r="AM110" s="7"/>
     </row>
-    <row r="111" spans="2:39">
+    <row r="111" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B111" s="1">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
-      <c r="C111" s="1"/>
-      <c r="D111" s="1"/>
+      <c r="C111" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
       <c r="G111" s="1"/>
@@ -7371,8 +7525,12 @@
         <v>197</v>
       </c>
       <c r="I111" s="1"/>
-      <c r="J111" s="1"/>
-      <c r="K111" s="1"/>
+      <c r="J111" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K111" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L111" s="1"/>
       <c r="M111" s="1"/>
       <c r="N111" s="1"/>
@@ -7402,13 +7560,17 @@
       <c r="AL111" s="7"/>
       <c r="AM111" s="7"/>
     </row>
-    <row r="112" spans="2:39" ht="57">
+    <row r="112" spans="2:39" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B112" s="1">
         <f t="shared" si="1"/>
         <v>106</v>
       </c>
-      <c r="C112" s="1"/>
-      <c r="D112" s="1"/>
+      <c r="C112" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
@@ -7416,8 +7578,12 @@
         <v>196</v>
       </c>
       <c r="I112" s="1"/>
-      <c r="J112" s="1"/>
-      <c r="K112" s="1"/>
+      <c r="J112" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K112" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L112" s="1"/>
       <c r="M112" s="1"/>
       <c r="N112" s="1"/>
@@ -7447,13 +7613,17 @@
       <c r="AL112" s="7"/>
       <c r="AM112" s="7"/>
     </row>
-    <row r="113" spans="2:39" ht="28.5">
+    <row r="113" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B113" s="1">
         <f t="shared" si="1"/>
         <v>107</v>
       </c>
-      <c r="C113" s="1"/>
-      <c r="D113" s="1"/>
+      <c r="C113" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
       <c r="G113" s="1"/>
@@ -7461,8 +7631,12 @@
         <v>198</v>
       </c>
       <c r="I113" s="1"/>
-      <c r="J113" s="1"/>
-      <c r="K113" s="1"/>
+      <c r="J113" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K113" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L113" s="1"/>
       <c r="M113" s="1"/>
       <c r="N113" s="1"/>
@@ -7492,13 +7666,17 @@
       <c r="AL113" s="7"/>
       <c r="AM113" s="7"/>
     </row>
-    <row r="114" spans="2:39" ht="42.75">
+    <row r="114" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B114" s="1">
         <f t="shared" si="1"/>
         <v>108</v>
       </c>
-      <c r="C114" s="1"/>
-      <c r="D114" s="1"/>
+      <c r="C114" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E114" s="1"/>
       <c r="F114" s="1"/>
       <c r="G114" s="1"/>
@@ -7506,8 +7684,12 @@
         <v>199</v>
       </c>
       <c r="I114" s="1"/>
-      <c r="J114" s="1"/>
-      <c r="K114" s="1"/>
+      <c r="J114" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K114" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L114" s="1"/>
       <c r="M114" s="1"/>
       <c r="N114" s="1"/>
@@ -7537,13 +7719,17 @@
       <c r="AL114" s="7"/>
       <c r="AM114" s="7"/>
     </row>
-    <row r="115" spans="2:39" ht="28.5">
+    <row r="115" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B115" s="1">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
-      <c r="C115" s="1"/>
-      <c r="D115" s="1"/>
+      <c r="C115" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E115" s="1"/>
       <c r="F115" s="1" t="s">
         <v>2</v>
@@ -7553,8 +7739,12 @@
         <v>200</v>
       </c>
       <c r="I115" s="1"/>
-      <c r="J115" s="1"/>
-      <c r="K115" s="1"/>
+      <c r="J115" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K115" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L115" s="1"/>
       <c r="M115" s="1"/>
       <c r="N115" s="1"/>
@@ -7584,20 +7774,28 @@
       <c r="AL115" s="7"/>
       <c r="AM115" s="7"/>
     </row>
-    <row r="116" spans="2:39">
+    <row r="116" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B116" s="1">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="C116" s="1"/>
-      <c r="D116" s="1"/>
+      <c r="C116" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
       <c r="G116" s="1"/>
       <c r="H116" s="8"/>
       <c r="I116" s="1"/>
-      <c r="J116" s="1"/>
-      <c r="K116" s="1"/>
+      <c r="J116" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K116" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L116" s="1"/>
       <c r="M116" s="1"/>
       <c r="N116" s="1"/>
@@ -7627,20 +7825,28 @@
       <c r="AL116" s="7"/>
       <c r="AM116" s="7"/>
     </row>
-    <row r="117" spans="2:39">
+    <row r="117" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B117" s="1">
         <f t="shared" si="1"/>
         <v>111</v>
       </c>
-      <c r="C117" s="1"/>
-      <c r="D117" s="1"/>
+      <c r="C117" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
       <c r="H117" s="8"/>
       <c r="I117" s="1"/>
-      <c r="J117" s="1"/>
-      <c r="K117" s="1"/>
+      <c r="J117" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K117" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L117" s="1"/>
       <c r="M117" s="1"/>
       <c r="N117" s="1"/>
@@ -7670,20 +7876,28 @@
       <c r="AL117" s="7"/>
       <c r="AM117" s="7"/>
     </row>
-    <row r="118" spans="2:39">
+    <row r="118" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B118" s="1">
         <f t="shared" si="1"/>
         <v>112</v>
       </c>
-      <c r="C118" s="1"/>
-      <c r="D118" s="1"/>
+      <c r="C118" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
       <c r="H118" s="8"/>
       <c r="I118" s="1"/>
-      <c r="J118" s="1"/>
-      <c r="K118" s="1"/>
+      <c r="J118" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K118" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L118" s="1"/>
       <c r="M118" s="1"/>
       <c r="N118" s="1"/>
@@ -7713,20 +7927,28 @@
       <c r="AL118" s="7"/>
       <c r="AM118" s="7"/>
     </row>
-    <row r="119" spans="2:39">
+    <row r="119" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B119" s="1">
         <f t="shared" si="1"/>
         <v>113</v>
       </c>
-      <c r="C119" s="1"/>
-      <c r="D119" s="1"/>
+      <c r="C119" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
       <c r="H119" s="8"/>
       <c r="I119" s="1"/>
-      <c r="J119" s="1"/>
-      <c r="K119" s="1"/>
+      <c r="J119" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K119" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L119" s="1"/>
       <c r="M119" s="1"/>
       <c r="N119" s="1"/>
@@ -7756,20 +7978,28 @@
       <c r="AL119" s="7"/>
       <c r="AM119" s="7"/>
     </row>
-    <row r="120" spans="2:39">
+    <row r="120" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B120" s="1">
         <f t="shared" si="1"/>
         <v>114</v>
       </c>
-      <c r="C120" s="1"/>
-      <c r="D120" s="1"/>
+      <c r="C120" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
       <c r="H120" s="8"/>
       <c r="I120" s="1"/>
-      <c r="J120" s="1"/>
-      <c r="K120" s="1"/>
+      <c r="J120" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K120" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L120" s="1"/>
       <c r="M120" s="1"/>
       <c r="N120" s="1"/>
@@ -7799,20 +8029,28 @@
       <c r="AL120" s="7"/>
       <c r="AM120" s="7"/>
     </row>
-    <row r="121" spans="2:39">
+    <row r="121" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B121" s="1">
         <f t="shared" si="1"/>
         <v>115</v>
       </c>
-      <c r="C121" s="1"/>
-      <c r="D121" s="1"/>
+      <c r="C121" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
       <c r="H121" s="8"/>
       <c r="I121" s="1"/>
-      <c r="J121" s="1"/>
-      <c r="K121" s="1"/>
+      <c r="J121" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K121" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L121" s="1"/>
       <c r="M121" s="1"/>
       <c r="N121" s="1"/>
@@ -7842,20 +8080,28 @@
       <c r="AL121" s="7"/>
       <c r="AM121" s="7"/>
     </row>
-    <row r="122" spans="2:39">
+    <row r="122" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B122" s="1">
         <f t="shared" si="1"/>
         <v>116</v>
       </c>
-      <c r="C122" s="1"/>
-      <c r="D122" s="1"/>
+      <c r="C122" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
       <c r="H122" s="8"/>
       <c r="I122" s="1"/>
-      <c r="J122" s="1"/>
-      <c r="K122" s="1"/>
+      <c r="J122" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K122" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L122" s="1"/>
       <c r="M122" s="1"/>
       <c r="N122" s="1"/>
@@ -7885,20 +8131,28 @@
       <c r="AL122" s="7"/>
       <c r="AM122" s="7"/>
     </row>
-    <row r="123" spans="2:39">
+    <row r="123" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B123" s="1">
         <f t="shared" si="1"/>
         <v>117</v>
       </c>
-      <c r="C123" s="1"/>
-      <c r="D123" s="1"/>
+      <c r="C123" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
       <c r="G123" s="1"/>
       <c r="H123" s="8"/>
       <c r="I123" s="1"/>
-      <c r="J123" s="1"/>
-      <c r="K123" s="1"/>
+      <c r="J123" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K123" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L123" s="1"/>
       <c r="M123" s="1"/>
       <c r="N123" s="1"/>
@@ -7928,20 +8182,28 @@
       <c r="AL123" s="7"/>
       <c r="AM123" s="7"/>
     </row>
-    <row r="124" spans="2:39">
+    <row r="124" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B124" s="1">
         <f t="shared" si="1"/>
         <v>118</v>
       </c>
-      <c r="C124" s="1"/>
-      <c r="D124" s="1"/>
+      <c r="C124" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
       <c r="G124" s="1"/>
       <c r="H124" s="8"/>
       <c r="I124" s="1"/>
-      <c r="J124" s="1"/>
-      <c r="K124" s="1"/>
+      <c r="J124" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K124" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L124" s="1"/>
       <c r="M124" s="1"/>
       <c r="N124" s="1"/>
@@ -7971,20 +8233,28 @@
       <c r="AL124" s="7"/>
       <c r="AM124" s="7"/>
     </row>
-    <row r="125" spans="2:39">
+    <row r="125" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B125" s="1">
         <f t="shared" si="1"/>
         <v>119</v>
       </c>
-      <c r="C125" s="1"/>
-      <c r="D125" s="1"/>
+      <c r="C125" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
       <c r="H125" s="8"/>
       <c r="I125" s="1"/>
-      <c r="J125" s="1"/>
-      <c r="K125" s="1"/>
+      <c r="J125" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K125" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L125" s="1"/>
       <c r="M125" s="1"/>
       <c r="N125" s="1"/>
@@ -8014,20 +8284,28 @@
       <c r="AL125" s="7"/>
       <c r="AM125" s="7"/>
     </row>
-    <row r="126" spans="2:39">
+    <row r="126" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B126" s="1">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="C126" s="1"/>
-      <c r="D126" s="1"/>
+      <c r="C126" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
       <c r="H126" s="8"/>
       <c r="I126" s="1"/>
-      <c r="J126" s="1"/>
-      <c r="K126" s="1"/>
+      <c r="J126" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K126" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L126" s="1"/>
       <c r="M126" s="1"/>
       <c r="N126" s="1"/>
@@ -8057,20 +8335,28 @@
       <c r="AL126" s="7"/>
       <c r="AM126" s="7"/>
     </row>
-    <row r="127" spans="2:39">
+    <row r="127" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B127" s="1">
         <f t="shared" si="1"/>
         <v>121</v>
       </c>
-      <c r="C127" s="1"/>
-      <c r="D127" s="1"/>
+      <c r="C127" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
       <c r="H127" s="8"/>
       <c r="I127" s="1"/>
-      <c r="J127" s="1"/>
-      <c r="K127" s="1"/>
+      <c r="J127" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K127" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L127" s="1"/>
       <c r="M127" s="1"/>
       <c r="N127" s="1"/>
@@ -8100,20 +8386,28 @@
       <c r="AL127" s="7"/>
       <c r="AM127" s="7"/>
     </row>
-    <row r="128" spans="2:39">
+    <row r="128" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B128" s="1">
         <f t="shared" si="1"/>
         <v>122</v>
       </c>
-      <c r="C128" s="1"/>
-      <c r="D128" s="1"/>
+      <c r="C128" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
       <c r="H128" s="8"/>
       <c r="I128" s="1"/>
-      <c r="J128" s="1"/>
-      <c r="K128" s="1"/>
+      <c r="J128" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K128" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L128" s="1"/>
       <c r="M128" s="1"/>
       <c r="N128" s="1"/>
@@ -8143,20 +8437,28 @@
       <c r="AL128" s="7"/>
       <c r="AM128" s="7"/>
     </row>
-    <row r="129" spans="2:39">
+    <row r="129" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B129" s="1">
         <f t="shared" si="1"/>
         <v>123</v>
       </c>
-      <c r="C129" s="1"/>
-      <c r="D129" s="1"/>
+      <c r="C129" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
       <c r="H129" s="8"/>
       <c r="I129" s="1"/>
-      <c r="J129" s="1"/>
-      <c r="K129" s="1"/>
+      <c r="J129" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K129" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L129" s="1"/>
       <c r="M129" s="1"/>
       <c r="N129" s="1"/>
@@ -8186,20 +8488,28 @@
       <c r="AL129" s="7"/>
       <c r="AM129" s="7"/>
     </row>
-    <row r="130" spans="2:39">
+    <row r="130" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B130" s="1">
         <f t="shared" si="1"/>
         <v>124</v>
       </c>
-      <c r="C130" s="1"/>
-      <c r="D130" s="1"/>
+      <c r="C130" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
       <c r="H130" s="8"/>
       <c r="I130" s="1"/>
-      <c r="J130" s="1"/>
-      <c r="K130" s="1"/>
+      <c r="J130" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K130" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L130" s="1"/>
       <c r="M130" s="1"/>
       <c r="N130" s="1"/>
@@ -8229,20 +8539,28 @@
       <c r="AL130" s="7"/>
       <c r="AM130" s="7"/>
     </row>
-    <row r="131" spans="2:39">
+    <row r="131" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B131" s="1">
         <f t="shared" si="1"/>
         <v>125</v>
       </c>
-      <c r="C131" s="1"/>
-      <c r="D131" s="1"/>
+      <c r="C131" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
       <c r="H131" s="8"/>
       <c r="I131" s="1"/>
-      <c r="J131" s="1"/>
-      <c r="K131" s="1"/>
+      <c r="J131" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K131" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L131" s="1"/>
       <c r="M131" s="1"/>
       <c r="N131" s="1"/>
@@ -8272,20 +8590,28 @@
       <c r="AL131" s="7"/>
       <c r="AM131" s="7"/>
     </row>
-    <row r="132" spans="2:39">
+    <row r="132" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B132" s="1">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="C132" s="1"/>
-      <c r="D132" s="1"/>
+      <c r="C132" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
       <c r="H132" s="8"/>
       <c r="I132" s="1"/>
-      <c r="J132" s="1"/>
-      <c r="K132" s="1"/>
+      <c r="J132" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K132" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="L132" s="1"/>
       <c r="M132" s="1"/>
       <c r="N132" s="1"/>
@@ -8356,14 +8682,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EDBD295-5C93-44DD-9985-3C1BB495EB4B}">
   <dimension ref="B2:F11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.25" customWidth="1"/>
-    <col min="4" max="4" width="14.125" customWidth="1"/>
-    <col min="6" max="6" width="16.875" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -8374,7 +8700,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="2:6">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>16</v>
       </c>
@@ -8385,7 +8711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:6">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -8396,7 +8722,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="2:6">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>41</v>
       </c>
@@ -8407,7 +8733,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>20</v>
       </c>
@@ -8415,7 +8741,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -8423,7 +8749,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:6">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>18</v>
       </c>
@@ -8431,7 +8757,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="2:6">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>19</v>
       </c>
@@ -8439,12 +8765,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:6">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
The script just needs to be carried over, then its ready for playtest (so late, I know, Im trying)
</commit_message>
<xml_diff>
--- a/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
+++ b/PADS/Assets/Editor/PoliticiaDialogueSpreadsheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damon\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\papadoal\source\repos\Political-Alien-Dating-Sim\PADS\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEABD923-7315-4D64-8DA7-E2807B76D3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2895F36-6A73-410A-8760-29AF53CF7C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3FB009F-9B8A-4212-A295-1ED52465BDAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="252">
   <si>
     <t>Dialogue Enter</t>
   </si>
@@ -643,13 +643,166 @@
   </si>
   <si>
     <t>Your commander’s face disappears from the bridge and your crew members wait on your word. You have your orders.</t>
+  </si>
+  <si>
+    <t>Wrong Exercise</t>
+  </si>
+  <si>
+    <t>Incorrect, please pick Judah and Shira to continue;</t>
+  </si>
+  <si>
+    <t>Body</t>
+  </si>
+  <si>
+    <t>Mind</t>
+  </si>
+  <si>
+    <t>Judah</t>
+  </si>
+  <si>
+    <t>Shira</t>
+  </si>
+  <si>
+    <t>The Amore charts its course to the first planet on your alliance-building mission. Ai opens the AstratechTM file on the main console.</t>
+  </si>
+  <si>
+    <t>Blorfengarl, a planet with an intense gravitational pull. Its dominant lifeform is a mucusoid species known as blorforms.</t>
+  </si>
+  <si>
+    <t>Initially hostile to earlier exploratory missions, they have since built and launched an orbital station named Membrane on which to receive guests.</t>
+  </si>
+  <si>
+    <t>You make your approach to this round, bubble-shaped spacestation. Docking into a large ship-bay, you are struck by a wave of hot air as the humidity seeps through your clothing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vents and spherical outcropping dot the hall, and despite its emptiness you can’t shake the feeling of being watched. </t>
+  </si>
+  <si>
+    <t>Hello</t>
+  </si>
+  <si>
+    <t>Have your crew forgotten to announce themselves beforehand? Your call echoes around the bay before the sound of gurgling at your feet draws your gaze downwards.</t>
+  </si>
+  <si>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>Investigate your Surroundings</t>
+  </si>
+  <si>
+    <t>The vents and spherical outcroppings have windows and holes. Strange for the purposes of ventilation but less so for the purpose of cautiously viewing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As mucusoids blorforms should easily be able to pass through grates and fit their bodies into tight spaces. As if on cue a gurgling at the grate beneath your feet proves your hypothesis. </t>
+  </si>
+  <si>
+    <t>Despite your best efforts you find yourself simply looking back and forth futilely. You still cannot shake the feeling of being watched. You jump as you are startled by a gurgling at your feet.</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>Out from a grate, green viscous fluid begins to pour forth. It arranges itself into the dumpy form, rolls on top of rolls cascaded down this standing puddle of a creature.</t>
+  </si>
+  <si>
+    <t>Its body a sickly green, a single lashed eyestalk peers forth as its other eye floats aimlessly through the main body.</t>
+  </si>
+  <si>
+    <t>Its mouth was more similar to a relief carved onto a sculpture or pastry, the slab-like teeth barely more defined than the indented “mouth” that helped them.</t>
+  </si>
+  <si>
+    <t>It altogether seems unnatural for a creature that can simply schlorp its body around anything it wishes to consume.</t>
+  </si>
+  <si>
+    <t>In a way it is almost cute, a gesture to elicit some goodwill from the foreigners it is greeting. A medal floats in its transparent body, on it a name inscribed. General Goumyster.</t>
+  </si>
+  <si>
+    <t>The general’s voice is strange and garbled, like someone trying to speak with a full mouth or underwater.</t>
+  </si>
+  <si>
+    <t>Through the distortion you can detect a note of discomfort, is the species unaccustomed to verbal conversation or are they somehow already displeased with you in some way.</t>
+  </si>
+  <si>
+    <t>No matter. As an AstraTechTM certified diplomacy captain and brand ambassador you are adept at navigating tricky situations to ensure an optimal outcome for all stakeholders.</t>
+  </si>
+  <si>
+    <t>A question, an opportunity. You can attempt to use your advanced negotiative techniques you’ve been perfecting all the way from Advertising Yourself 101, back in your cadet days.</t>
+  </si>
+  <si>
+    <t>Positivity. AstraInsiderTM has stated for years that people in positions of authority enjoy relentless enthusiasm, happiness, and satisfaction from their subordinates and those that they encounter elsewhere.</t>
+  </si>
+  <si>
+    <t>For the greater good of your corporation, nay your conglomerate, you will adopt the submissive position.</t>
+  </si>
+  <si>
+    <t>Lulling them into a sense of security and satisfaction can make future negotiations lean towards favorable outcomes for your party.</t>
+  </si>
+  <si>
+    <t>1M</t>
+  </si>
+  <si>
+    <t>Tension. Though verbalizing discomfort is not technically permitted under the AstraTechTM employee charter, in your role as captain you are permitted to bend the rules a bit in order to foster a greater sense of emotional proximity with your potential clients.</t>
+  </si>
+  <si>
+    <t>You have observed on occasion lower-level employees bonding over the shared commiseration of misfortunes and ills of all manners.</t>
+  </si>
+  <si>
+    <t>Additionally the discomfort posed by displeasure may momentarily disarm your opponent, affording you better leverage in future negotiations.</t>
+  </si>
+  <si>
+    <t>HA! Apologies Captain, we meant no harm! We're due for a new Fnozzle for the artificial gravity core!</t>
+  </si>
+  <si>
+    <t>The General’s form starts swaying aggressively as their transparent interior produces plumes of bubbles and froth. Anger? Fear? Embarrassment?</t>
+  </si>
+  <si>
+    <t>Now did you mean to accuse or cause offence with your words? It is of no importance, they have shown their belly and you are ready to pounce.</t>
+  </si>
+  <si>
+    <t>The General’s swaying has grown ever more frantic as if they can’t wait to move. SUCCESS? You have made this stranger uncomfortable.</t>
+  </si>
+  <si>
+    <t>Humour. A charming anecdote that would prove to be supremely relatable and well received. Humour is the basis of many an excellent advertisement.</t>
+  </si>
+  <si>
+    <t>It is memorable and can be repeated in the future to strengthen positive memories of the experience. Yes, the perfect approach to disarm your opponent for future investigations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The General unleashes a violent jiggle before composing themself. You see a flash of hunger in their eyes, the same ravenous hunger that binds all life forms and thrusts them forward. </t>
+  </si>
+  <si>
+    <t>The burning that can only be satisfied with a range of delicious, nutritious, and affordable foodstuffs purchasable in any friendly canteen.</t>
+  </si>
+  <si>
+    <t>hmm, well we have some Bleeding Grapes back at the Space Station you can have some of those.</t>
+  </si>
+  <si>
+    <t>The general turns away, a wet slurping sound fills the bay, as they drag their body on the floor, leaving a sticky green trail behind them.</t>
+  </si>
+  <si>
+    <t>President? The general has an attending superior? Have you wasted your excellent social skills on a mere underling?</t>
+  </si>
+  <si>
+    <t>Those are valuable billable hours you have spent suboptimally. Fortunately you yourself  don’t have a supervisor present, otherwise your wages may be garnished for such an offence.</t>
+  </si>
+  <si>
+    <t>Humanoid in shape, she’s a tall green skinned woman with big compound eyes. The lights of the space station reflect and shine off them like the hazy glow of a distant city at night.</t>
+  </si>
+  <si>
+    <t>While dressed far too scandalously for your expectations of a politician, you are more shocked by her species.</t>
+  </si>
+  <si>
+    <t>She is clearly not a blorform. Odd that such a traditionally reclusive and hostile species has elected a foreigner to oversee these negotiations.</t>
+  </si>
+  <si>
+    <t>The general shuffles off, but the strange feeling that you are being watched does not follow him out.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -728,7 +881,41 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="47">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1216,50 +1403,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM132" totalsRowShown="0" dataDxfId="42">
-  <autoFilter ref="B5:AM132" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}" name="Dialogue" displayName="Dialogue" ref="B5:AM177" totalsRowShown="0" dataDxfId="46">
+  <autoFilter ref="B5:AM177" xr:uid="{D2D5E833-C969-47F1-B36D-7A7FDD3BE4F8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:AM20">
     <sortCondition ref="B5:B20"/>
   </sortState>
   <tableColumns count="38">
-    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="41"/>
-    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="39"/>
-    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="38"/>
-    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="32"/>
-    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="31"/>
-    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="30"/>
-    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="28"/>
-    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="27"/>
-    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="26"/>
-    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="25"/>
-    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="24"/>
-    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="23"/>
-    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="22"/>
-    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="21"/>
-    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="20"/>
-    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="19"/>
-    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="18"/>
-    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="17"/>
-    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="16"/>
-    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="15"/>
-    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="14"/>
-    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="13"/>
-    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="12"/>
-    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="11"/>
-    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="10"/>
-    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="9"/>
-    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="8"/>
-    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="7"/>
-    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="6"/>
-    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="5"/>
-    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="4"/>
+    <tableColumn id="56" xr3:uid="{09125C0D-8B10-43E0-A5C7-83AA1C0438E4}" name="Index" dataDxfId="45"/>
+    <tableColumn id="1" xr3:uid="{C8641FE3-8417-4114-B6D8-F9904FB0CDDB}" name="Left Character" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{BCD9A495-8337-4E42-AF2D-09E789FAD79C}" name="Left Expression" dataDxfId="43"/>
+    <tableColumn id="13" xr3:uid="{DA1E4994-40CC-4128-B249-B0A5B473F5EF}" name="Is Left Speaking?" dataDxfId="42"/>
+    <tableColumn id="15" xr3:uid="{A9C394D3-880A-418B-A6C9-701F7CA7ABC5}" name="End Dialogue?" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{C70DAC7F-E424-46AE-BD9A-91F1E1632B9A}" name="Dialogue Enter" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{DCC897A1-70A3-4C28-B1B2-0FBC3CC4422B}" name="Dialogue Text" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{CBCADF4A-0140-441F-8A63-731F45641E14}" name="Dialogue Exit" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{D02CCC46-0E2B-4B42-A2F2-116D38B44296}" name="Right Expression" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{513F13A5-7A6C-4917-BC2A-42835B70275C}" name="Right Character" dataDxfId="36"/>
+    <tableColumn id="61" xr3:uid="{A3C99AFD-B985-43B8-9C55-625F8F254585}" name="Value Check A" dataDxfId="35"/>
+    <tableColumn id="64" xr3:uid="{40263D7D-ED81-4134-B9D8-20A5E5EDD5C0}" name="Conditional A" dataDxfId="34"/>
+    <tableColumn id="65" xr3:uid="{806DA262-150A-4905-8BC7-A837710A0467}" name="Requirement A" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{3258BD14-E46D-43FD-9353-006E4431D22E}" name="Dialogue Option A" dataDxfId="32"/>
+    <tableColumn id="62" xr3:uid="{BC21EF94-22C6-4B5E-ADCE-8DA1E19E2943}" name="Variable Change A" dataDxfId="31"/>
+    <tableColumn id="63" xr3:uid="{B9B0AC2C-34DF-403A-B90B-7859E7C20819}" name="Value Change A" dataDxfId="30"/>
+    <tableColumn id="57" xr3:uid="{37EE4195-EF48-41D9-9120-F37357150341}" name="Exit A" dataDxfId="29"/>
+    <tableColumn id="66" xr3:uid="{AB539150-2E1C-4D50-9DC9-2A985BD1EAD0}" name="Value Check B" dataDxfId="28"/>
+    <tableColumn id="67" xr3:uid="{E8F68698-DE27-4B18-BE85-07D0A70C4733}" name="Conditional B" dataDxfId="27"/>
+    <tableColumn id="68" xr3:uid="{AE027240-1467-43CB-9384-B927613F30A9}" name="Requirement B" dataDxfId="26"/>
+    <tableColumn id="69" xr3:uid="{8AED339C-B64B-4C8A-B979-32160D57BAB1}" name="Dialogue Option B" dataDxfId="25"/>
+    <tableColumn id="70" xr3:uid="{D271AED5-3061-484E-8C5C-7D1CFDD3EF1F}" name="Variable Change B" dataDxfId="24"/>
+    <tableColumn id="71" xr3:uid="{4829F23F-4EE7-45BA-8839-5063AFD38D28}" name="Value Change B" dataDxfId="23"/>
+    <tableColumn id="72" xr3:uid="{E242E34F-7964-4CDD-8774-0D6A2DF6D59A}" name="Exit B" dataDxfId="22"/>
+    <tableColumn id="73" xr3:uid="{972FBE7E-C2F9-4214-8217-012BD22A5913}" name="Value Check C" dataDxfId="21"/>
+    <tableColumn id="74" xr3:uid="{81DCE3B0-B0E1-452E-95EA-B10CE4370FF5}" name="Conditional C" dataDxfId="20"/>
+    <tableColumn id="75" xr3:uid="{110CBAC7-6FF1-4870-90E8-3923265382D3}" name="Requirement C" dataDxfId="19"/>
+    <tableColumn id="76" xr3:uid="{0E58C58F-E67A-4DDD-96A9-7A4552C04D7D}" name="Dialogue Option C" dataDxfId="18"/>
+    <tableColumn id="77" xr3:uid="{E1629C60-280F-4E07-B992-B0A9F238D15E}" name="Variable Change C" dataDxfId="17"/>
+    <tableColumn id="78" xr3:uid="{5B0F8594-A24C-41A6-9A9F-E1CFF3D64FAB}" name="Value Change C" dataDxfId="16"/>
+    <tableColumn id="79" xr3:uid="{44ADCDF8-A71E-46E7-A9A2-C4EF144DE36C}" name="Exit C" dataDxfId="15"/>
+    <tableColumn id="80" xr3:uid="{A1F71E74-5C22-4789-8E4F-E7085E320909}" name="Value Check D" dataDxfId="14"/>
+    <tableColumn id="81" xr3:uid="{B4B32F8C-6116-41E8-9326-7C0DDE6FB46B}" name="Conditional D" dataDxfId="13"/>
+    <tableColumn id="82" xr3:uid="{42622F75-9694-4772-BC74-D6656E27BF59}" name="Requirement D" dataDxfId="12"/>
+    <tableColumn id="83" xr3:uid="{20DB4193-321D-4EB5-9C23-40D767A62F90}" name="Dialogue Option D" dataDxfId="11"/>
+    <tableColumn id="84" xr3:uid="{3E23DFE2-C4D4-4E80-BBDE-01D49E11F2F0}" name="Variable Change D" dataDxfId="10"/>
+    <tableColumn id="85" xr3:uid="{B40A46D8-1E19-4B2F-B77E-160648B46BAA}" name="Value Change D" dataDxfId="9"/>
+    <tableColumn id="86" xr3:uid="{C1A3B19C-14D6-46BA-87CE-7F613358AA23}" name="Exit D" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1615,39 +1802,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AD6004-D6D5-49E8-98E5-3900A70D687C}">
-  <dimension ref="B4:AM132"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B4:AM177"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" customWidth="1"/>
-    <col min="4" max="7" width="14.77734375" customWidth="1"/>
-    <col min="8" max="8" width="60.77734375" customWidth="1"/>
-    <col min="9" max="10" width="14.77734375" customWidth="1"/>
-    <col min="11" max="14" width="15.77734375" customWidth="1"/>
-    <col min="15" max="15" width="20.77734375" customWidth="1"/>
-    <col min="16" max="16" width="18.77734375" customWidth="1"/>
-    <col min="17" max="17" width="15.77734375" customWidth="1"/>
-    <col min="18" max="18" width="14.77734375" customWidth="1"/>
-    <col min="19" max="21" width="15.77734375" customWidth="1"/>
-    <col min="22" max="22" width="20.77734375" customWidth="1"/>
-    <col min="23" max="23" width="18.77734375" customWidth="1"/>
-    <col min="24" max="24" width="15.77734375" customWidth="1"/>
-    <col min="25" max="25" width="14.77734375" customWidth="1"/>
-    <col min="26" max="28" width="15.77734375" customWidth="1"/>
-    <col min="29" max="29" width="20.77734375" customWidth="1"/>
-    <col min="30" max="30" width="18.77734375" customWidth="1"/>
-    <col min="31" max="31" width="15.77734375" customWidth="1"/>
-    <col min="32" max="32" width="14.77734375" customWidth="1"/>
-    <col min="33" max="35" width="15.77734375" customWidth="1"/>
-    <col min="36" max="36" width="20.77734375" customWidth="1"/>
-    <col min="37" max="37" width="18.77734375" customWidth="1"/>
-    <col min="38" max="38" width="15.77734375" customWidth="1"/>
-    <col min="39" max="39" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="8.875" customWidth="1"/>
+    <col min="2" max="2" width="8.625" customWidth="1"/>
+    <col min="3" max="3" width="15.75" customWidth="1"/>
+    <col min="4" max="7" width="14.75" customWidth="1"/>
+    <col min="8" max="8" width="60.75" customWidth="1"/>
+    <col min="9" max="10" width="14.75" customWidth="1"/>
+    <col min="11" max="14" width="15.75" customWidth="1"/>
+    <col min="15" max="15" width="20.75" customWidth="1"/>
+    <col min="16" max="16" width="18.75" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.75" customWidth="1"/>
+    <col min="19" max="21" width="15.75" customWidth="1"/>
+    <col min="22" max="22" width="20.75" customWidth="1"/>
+    <col min="23" max="23" width="18.75" customWidth="1"/>
+    <col min="24" max="24" width="15.75" customWidth="1"/>
+    <col min="25" max="25" width="14.75" customWidth="1"/>
+    <col min="26" max="28" width="15.75" customWidth="1"/>
+    <col min="29" max="29" width="20.75" customWidth="1"/>
+    <col min="30" max="30" width="18.75" customWidth="1"/>
+    <col min="31" max="31" width="15.75" customWidth="1"/>
+    <col min="32" max="32" width="14.75" customWidth="1"/>
+    <col min="33" max="35" width="15.75" customWidth="1"/>
+    <col min="36" max="36" width="20.75" customWidth="1"/>
+    <col min="37" max="37" width="18.75" customWidth="1"/>
+    <col min="38" max="38" width="15.75" customWidth="1"/>
+    <col min="39" max="39" width="14.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:39" ht="88.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:39" ht="88.9" customHeight="1"/>
+    <row r="5" spans="2:39">
       <c r="B5" t="s">
         <v>22</v>
       </c>
@@ -1763,7 +1950,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:39" ht="28.5">
       <c r="B6" s="1">
         <v>0</v>
       </c>
@@ -1817,7 +2004,7 @@
       <c r="AL6" s="7"/>
       <c r="AM6" s="7"/>
     </row>
-    <row r="7" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:39" ht="28.5">
       <c r="B7" s="1">
         <f t="shared" ref="B7:B70" si="0">1+B6</f>
         <v>1</v>
@@ -1872,7 +2059,7 @@
       <c r="AL7" s="7"/>
       <c r="AM7" s="7"/>
     </row>
-    <row r="8" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:39" ht="28.5">
       <c r="B8" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1925,7 +2112,7 @@
       <c r="AL8" s="7"/>
       <c r="AM8" s="7"/>
     </row>
-    <row r="9" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:39" ht="42.75">
       <c r="B9" s="1">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1980,7 +2167,7 @@
       <c r="AL9" s="7"/>
       <c r="AM9" s="7"/>
     </row>
-    <row r="10" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:39" ht="28.5">
       <c r="B10" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2039,7 +2226,7 @@
       <c r="AL10" s="7"/>
       <c r="AM10" s="7"/>
     </row>
-    <row r="11" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:39">
       <c r="B11" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2096,7 +2283,7 @@
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
     </row>
-    <row r="12" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:39" ht="42.75">
       <c r="B12" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2107,9 +2294,7 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="1" t="s">
-        <v>70</v>
-      </c>
+      <c r="G12" s="1"/>
       <c r="H12" s="8" t="s">
         <v>71</v>
       </c>
@@ -2149,7 +2334,7 @@
       <c r="AL12" s="7"/>
       <c r="AM12" s="7"/>
     </row>
-    <row r="13" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:39" ht="28.5">
       <c r="B13" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2202,7 +2387,7 @@
       <c r="AL13" s="7"/>
       <c r="AM13" s="7"/>
     </row>
-    <row r="14" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:39">
       <c r="B14" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2257,7 +2442,7 @@
       <c r="AL14" s="7"/>
       <c r="AM14" s="7"/>
     </row>
-    <row r="15" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:39" ht="28.5">
       <c r="B15" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2322,7 +2507,7 @@
       <c r="AL15" s="7"/>
       <c r="AM15" s="7"/>
     </row>
-    <row r="16" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:39">
       <c r="B16" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2335,9 +2520,7 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="1" t="s">
-        <v>75</v>
-      </c>
+      <c r="G16" s="1"/>
       <c r="H16" s="8" t="s">
         <v>76</v>
       </c>
@@ -2379,7 +2562,7 @@
       <c r="AL16" s="7"/>
       <c r="AM16" s="7"/>
     </row>
-    <row r="17" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:39" ht="28.5">
       <c r="B17" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2392,9 +2575,7 @@
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="1" t="s">
-        <v>78</v>
-      </c>
+      <c r="G17" s="1"/>
       <c r="H17" s="8" t="s">
         <v>77</v>
       </c>
@@ -2434,7 +2615,7 @@
       <c r="AL17" s="7"/>
       <c r="AM17" s="7"/>
     </row>
-    <row r="18" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:39">
       <c r="B18" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2491,7 +2672,7 @@
       <c r="AL18" s="7"/>
       <c r="AM18" s="7"/>
     </row>
-    <row r="19" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:39" ht="28.5">
       <c r="B19" s="1">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2504,9 +2685,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="G19" s="1"/>
       <c r="H19" s="8" t="s">
         <v>147</v>
       </c>
@@ -2548,7 +2727,7 @@
       <c r="AL19" s="7"/>
       <c r="AM19" s="7"/>
     </row>
-    <row r="20" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:39">
       <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2561,9 +2740,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="1"/>
-      <c r="G20" s="1" t="s">
-        <v>84</v>
-      </c>
+      <c r="G20" s="1"/>
       <c r="H20" s="8" t="s">
         <v>85</v>
       </c>
@@ -2603,7 +2780,7 @@
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
     </row>
-    <row r="21" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:39">
       <c r="B21" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2656,7 +2833,7 @@
       <c r="AL21" s="7"/>
       <c r="AM21" s="7"/>
     </row>
-    <row r="22" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:39" ht="42.75">
       <c r="B22" s="1">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2709,7 +2886,7 @@
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
     </row>
-    <row r="23" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:39" ht="28.5">
       <c r="B23" s="1">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2762,7 +2939,7 @@
       <c r="AL23" s="7"/>
       <c r="AM23" s="7"/>
     </row>
-    <row r="24" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:39">
       <c r="B24" s="1">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2815,7 +2992,7 @@
       <c r="AL24" s="7"/>
       <c r="AM24" s="7"/>
     </row>
-    <row r="25" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:39" ht="28.5">
       <c r="B25" s="1">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2892,7 +3069,7 @@
       <c r="AL25" s="7"/>
       <c r="AM25" s="7"/>
     </row>
-    <row r="26" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:39">
       <c r="B26" s="1">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2907,9 +3084,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="1"/>
-      <c r="G26" s="1" t="s">
-        <v>96</v>
-      </c>
+      <c r="G26" s="1"/>
       <c r="H26" s="8" t="s">
         <v>97</v>
       </c>
@@ -2949,7 +3124,7 @@
       <c r="AL26" s="7"/>
       <c r="AM26" s="7"/>
     </row>
-    <row r="27" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:39" ht="28.5">
       <c r="B27" s="1">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3002,7 +3177,7 @@
       <c r="AL27" s="7"/>
       <c r="AM27" s="7"/>
     </row>
-    <row r="28" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:39">
       <c r="B28" s="1">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3057,7 +3232,7 @@
       <c r="AL28" s="7"/>
       <c r="AM28" s="7"/>
     </row>
-    <row r="29" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:39">
       <c r="B29" s="1">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3112,7 +3287,7 @@
       <c r="AL29" s="7"/>
       <c r="AM29" s="7"/>
     </row>
-    <row r="30" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:39">
       <c r="B30" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3125,9 +3300,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="1"/>
-      <c r="G30" s="1" t="s">
-        <v>95</v>
-      </c>
+      <c r="G30" s="1"/>
       <c r="H30" s="8" t="s">
         <v>101</v>
       </c>
@@ -3167,7 +3340,7 @@
       <c r="AL30" s="7"/>
       <c r="AM30" s="7"/>
     </row>
-    <row r="31" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:39">
       <c r="B31" s="1">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3222,7 +3395,7 @@
       <c r="AL31" s="7"/>
       <c r="AM31" s="7"/>
     </row>
-    <row r="32" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:39">
       <c r="B32" s="1">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3275,7 +3448,7 @@
       <c r="AL32" s="7"/>
       <c r="AM32" s="7"/>
     </row>
-    <row r="33" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:39">
       <c r="B33" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3330,7 +3503,7 @@
       <c r="AL33" s="7"/>
       <c r="AM33" s="7"/>
     </row>
-    <row r="34" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:39">
       <c r="B34" s="1">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3385,7 +3558,7 @@
       <c r="AL34" s="7"/>
       <c r="AM34" s="7"/>
     </row>
-    <row r="35" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:39" ht="28.5">
       <c r="B35" s="1">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3398,9 +3571,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="1"/>
-      <c r="G35" s="1" t="s">
-        <v>94</v>
-      </c>
+      <c r="G35" s="1"/>
       <c r="H35" s="8" t="s">
         <v>108</v>
       </c>
@@ -3440,7 +3611,7 @@
       <c r="AL35" s="7"/>
       <c r="AM35" s="7"/>
     </row>
-    <row r="36" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:39">
       <c r="B36" s="1">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3493,7 +3664,7 @@
       <c r="AL36" s="7"/>
       <c r="AM36" s="7"/>
     </row>
-    <row r="37" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:39">
       <c r="B37" s="1">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3548,7 +3719,7 @@
       <c r="AL37" s="7"/>
       <c r="AM37" s="7"/>
     </row>
-    <row r="38" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:39">
       <c r="B38" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3601,7 +3772,7 @@
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
     </row>
-    <row r="39" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:39">
       <c r="B39" s="1">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3656,7 +3827,7 @@
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
     </row>
-    <row r="40" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:39" ht="28.5">
       <c r="B40" s="1">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3709,7 +3880,7 @@
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
     </row>
-    <row r="41" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:39" ht="28.5">
       <c r="B41" s="1">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3762,7 +3933,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
     </row>
-    <row r="42" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:39" ht="28.5">
       <c r="B42" s="1">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3817,7 +3988,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
     </row>
-    <row r="43" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:39">
       <c r="B43" s="1">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3870,7 +4041,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
     </row>
-    <row r="44" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:39">
       <c r="B44" s="1">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3939,7 +4110,7 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
     </row>
-    <row r="45" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:39">
       <c r="B45" s="1">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3954,9 +4125,7 @@
         <v>2</v>
       </c>
       <c r="F45" s="1"/>
-      <c r="G45" s="1" t="s">
-        <v>119</v>
-      </c>
+      <c r="G45" s="1"/>
       <c r="H45" s="8" t="s">
         <v>122</v>
       </c>
@@ -3996,7 +4165,7 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
     </row>
-    <row r="46" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:39" ht="28.5">
       <c r="B46" s="1">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -4051,7 +4220,7 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
     </row>
-    <row r="47" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:39" ht="42.75">
       <c r="B47" s="1">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -4064,9 +4233,7 @@
         <v>2</v>
       </c>
       <c r="F47" s="1"/>
-      <c r="G47" s="1" t="s">
-        <v>121</v>
-      </c>
+      <c r="G47" s="1"/>
       <c r="H47" s="8" t="s">
         <v>124</v>
       </c>
@@ -4106,7 +4273,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
     </row>
-    <row r="48" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:39">
       <c r="B48" s="1">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -4161,7 +4328,7 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
     </row>
-    <row r="49" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:39" ht="28.5">
       <c r="B49" s="1">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -4174,9 +4341,7 @@
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
-      <c r="G49" s="1" t="s">
-        <v>106</v>
-      </c>
+      <c r="G49" s="1"/>
       <c r="H49" s="8" t="s">
         <v>126</v>
       </c>
@@ -4216,7 +4381,7 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
     </row>
-    <row r="50" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:39" ht="42.75">
       <c r="B50" s="1">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -4271,7 +4436,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
     </row>
-    <row r="51" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:39" ht="28.5">
       <c r="B51" s="1">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -4324,7 +4489,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
     </row>
-    <row r="52" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:39">
       <c r="B52" s="1">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -4379,7 +4544,7 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
     </row>
-    <row r="53" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:39" ht="28.5">
       <c r="B53" s="1">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -4432,7 +4597,7 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
     </row>
-    <row r="54" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:39" ht="28.5">
       <c r="B54" s="1">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -4487,7 +4652,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
     </row>
-    <row r="55" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:39" ht="42.75">
       <c r="B55" s="1">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -4540,7 +4705,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
     </row>
-    <row r="56" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:39" ht="28.5">
       <c r="B56" s="1">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -4617,7 +4782,7 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
     </row>
-    <row r="57" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:39" ht="28.5">
       <c r="B57" s="1">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -4630,9 +4795,7 @@
         <v>2</v>
       </c>
       <c r="F57" s="1"/>
-      <c r="G57" s="1" t="s">
-        <v>135</v>
-      </c>
+      <c r="G57" s="1"/>
       <c r="H57" s="8" t="s">
         <v>139</v>
       </c>
@@ -4672,7 +4835,7 @@
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
     </row>
-    <row r="58" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:39">
       <c r="B58" s="1">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -4727,7 +4890,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
     </row>
-    <row r="59" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:39">
       <c r="B59" s="1">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -4782,7 +4945,7 @@
       <c r="AL59" s="7"/>
       <c r="AM59" s="7"/>
     </row>
-    <row r="60" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:39">
       <c r="B60" s="1">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -4795,9 +4958,7 @@
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
-      <c r="G60" s="1" t="s">
-        <v>138</v>
-      </c>
+      <c r="G60" s="1"/>
       <c r="H60" s="8" t="s">
         <v>142</v>
       </c>
@@ -4837,7 +4998,7 @@
       <c r="AL60" s="7"/>
       <c r="AM60" s="7"/>
     </row>
-    <row r="61" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:39">
       <c r="B61" s="1">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -4894,7 +5055,7 @@
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
     </row>
-    <row r="62" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:39">
       <c r="B62" s="1">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -4907,9 +5068,7 @@
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
-      <c r="G62" s="1" t="s">
-        <v>107</v>
-      </c>
+      <c r="G62" s="1"/>
       <c r="H62" s="8" t="s">
         <v>144</v>
       </c>
@@ -4951,7 +5110,7 @@
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
     </row>
-    <row r="63" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:39">
       <c r="B63" s="1">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -4964,9 +5123,7 @@
         <v>2</v>
       </c>
       <c r="F63" s="1"/>
-      <c r="G63" s="1" t="s">
-        <v>145</v>
-      </c>
+      <c r="G63" s="1"/>
       <c r="H63" s="8" t="s">
         <v>146</v>
       </c>
@@ -5014,7 +5171,7 @@
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
     </row>
-    <row r="64" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:39">
       <c r="B64" s="1">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -5065,7 +5222,7 @@
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
     </row>
-    <row r="65" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:39" ht="42.75">
       <c r="B65" s="1">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -5078,9 +5235,7 @@
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
-      <c r="G65" s="1" t="s">
-        <v>150</v>
-      </c>
+      <c r="G65" s="1"/>
       <c r="H65" s="8" t="s">
         <v>151</v>
       </c>
@@ -5120,7 +5275,7 @@
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
     </row>
-    <row r="66" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:39" ht="42.75">
       <c r="B66" s="1">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -5173,7 +5328,7 @@
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
     </row>
-    <row r="67" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:39" ht="28.5">
       <c r="B67" s="1">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -5226,7 +5381,7 @@
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
     </row>
-    <row r="68" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:39" ht="28.5">
       <c r="B68" s="1">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -5279,7 +5434,7 @@
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
     </row>
-    <row r="69" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:39" ht="42.75">
       <c r="B69" s="1">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -5332,7 +5487,7 @@
       <c r="AL69" s="7"/>
       <c r="AM69" s="7"/>
     </row>
-    <row r="70" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:39" ht="28.5">
       <c r="B70" s="1">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -5385,9 +5540,9 @@
       <c r="AL70" s="7"/>
       <c r="AM70" s="7"/>
     </row>
-    <row r="71" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:39" ht="28.5">
       <c r="B71" s="1">
-        <f t="shared" ref="B71:B132" si="1">1+B70</f>
+        <f t="shared" ref="B71:B131" si="1">1+B70</f>
         <v>65</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -5438,7 +5593,7 @@
       <c r="AL71" s="7"/>
       <c r="AM71" s="7"/>
     </row>
-    <row r="72" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:39" ht="42.75">
       <c r="B72" s="1">
         <f t="shared" si="1"/>
         <v>66</v>
@@ -5491,7 +5646,7 @@
       <c r="AL72" s="7"/>
       <c r="AM72" s="7"/>
     </row>
-    <row r="73" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:39" ht="28.5">
       <c r="B73" s="1">
         <f t="shared" si="1"/>
         <v>67</v>
@@ -5544,7 +5699,7 @@
       <c r="AL73" s="7"/>
       <c r="AM73" s="7"/>
     </row>
-    <row r="74" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:39" ht="42.75">
       <c r="B74" s="1">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -5597,7 +5752,7 @@
       <c r="AL74" s="7"/>
       <c r="AM74" s="7"/>
     </row>
-    <row r="75" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:39" ht="28.5">
       <c r="B75" s="1">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -5650,7 +5805,7 @@
       <c r="AL75" s="7"/>
       <c r="AM75" s="7"/>
     </row>
-    <row r="76" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:39" ht="28.5">
       <c r="B76" s="1">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -5703,7 +5858,7 @@
       <c r="AL76" s="7"/>
       <c r="AM76" s="7"/>
     </row>
-    <row r="77" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:39" ht="28.5">
       <c r="B77" s="1">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -5756,7 +5911,7 @@
       <c r="AL77" s="7"/>
       <c r="AM77" s="7"/>
     </row>
-    <row r="78" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:39" ht="28.5">
       <c r="B78" s="1">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -5809,7 +5964,7 @@
       <c r="AL78" s="7"/>
       <c r="AM78" s="7"/>
     </row>
-    <row r="79" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:39" ht="28.5">
       <c r="B79" s="1">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -5862,7 +6017,7 @@
       <c r="AL79" s="7"/>
       <c r="AM79" s="7"/>
     </row>
-    <row r="80" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:39">
       <c r="B80" s="1">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -5915,7 +6070,7 @@
       <c r="AL80" s="7"/>
       <c r="AM80" s="7"/>
     </row>
-    <row r="81" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:39">
       <c r="B81" s="1">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -5968,7 +6123,7 @@
       <c r="AL81" s="7"/>
       <c r="AM81" s="7"/>
     </row>
-    <row r="82" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:39" ht="28.5">
       <c r="B82" s="1">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -6021,7 +6176,7 @@
       <c r="AL82" s="7"/>
       <c r="AM82" s="7"/>
     </row>
-    <row r="83" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:39" ht="42.75">
       <c r="B83" s="1">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -6074,7 +6229,7 @@
       <c r="AL83" s="7"/>
       <c r="AM83" s="7"/>
     </row>
-    <row r="84" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:39">
       <c r="B84" s="1">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -6127,7 +6282,7 @@
       <c r="AL84" s="7"/>
       <c r="AM84" s="7"/>
     </row>
-    <row r="85" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:39" ht="28.5">
       <c r="B85" s="1">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -6180,7 +6335,7 @@
       <c r="AL85" s="7"/>
       <c r="AM85" s="7"/>
     </row>
-    <row r="86" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:39">
       <c r="B86" s="1">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -6233,7 +6388,7 @@
       <c r="AL86" s="7"/>
       <c r="AM86" s="7"/>
     </row>
-    <row r="87" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:39" ht="28.5">
       <c r="B87" s="1">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -6286,7 +6441,7 @@
       <c r="AL87" s="7"/>
       <c r="AM87" s="7"/>
     </row>
-    <row r="88" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:39">
       <c r="B88" s="1">
         <f t="shared" si="1"/>
         <v>82</v>
@@ -6339,7 +6494,7 @@
       <c r="AL88" s="7"/>
       <c r="AM88" s="7"/>
     </row>
-    <row r="89" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:39" ht="42.75">
       <c r="B89" s="1">
         <f t="shared" si="1"/>
         <v>83</v>
@@ -6392,7 +6547,7 @@
       <c r="AL89" s="7"/>
       <c r="AM89" s="7"/>
     </row>
-    <row r="90" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:39" ht="28.5">
       <c r="B90" s="1">
         <f t="shared" si="1"/>
         <v>84</v>
@@ -6445,7 +6600,7 @@
       <c r="AL90" s="7"/>
       <c r="AM90" s="7"/>
     </row>
-    <row r="91" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:39">
       <c r="B91" s="1">
         <f t="shared" si="1"/>
         <v>85</v>
@@ -6498,7 +6653,7 @@
       <c r="AL91" s="7"/>
       <c r="AM91" s="7"/>
     </row>
-    <row r="92" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:39">
       <c r="B92" s="1">
         <f t="shared" si="1"/>
         <v>86</v>
@@ -6551,7 +6706,7 @@
       <c r="AL92" s="7"/>
       <c r="AM92" s="7"/>
     </row>
-    <row r="93" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:39" ht="28.5">
       <c r="B93" s="1">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -6604,7 +6759,7 @@
       <c r="AL93" s="7"/>
       <c r="AM93" s="7"/>
     </row>
-    <row r="94" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:39" ht="28.5">
       <c r="B94" s="1">
         <f t="shared" si="1"/>
         <v>88</v>
@@ -6657,7 +6812,7 @@
       <c r="AL94" s="7"/>
       <c r="AM94" s="7"/>
     </row>
-    <row r="95" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:39" ht="42.75">
       <c r="B95" s="1">
         <f t="shared" si="1"/>
         <v>89</v>
@@ -6710,7 +6865,7 @@
       <c r="AL95" s="7"/>
       <c r="AM95" s="7"/>
     </row>
-    <row r="96" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:39" ht="28.5">
       <c r="B96" s="1">
         <f t="shared" si="1"/>
         <v>90</v>
@@ -6763,7 +6918,7 @@
       <c r="AL96" s="7"/>
       <c r="AM96" s="7"/>
     </row>
-    <row r="97" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:39">
       <c r="B97" s="1">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -6816,7 +6971,7 @@
       <c r="AL97" s="7"/>
       <c r="AM97" s="7"/>
     </row>
-    <row r="98" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:39" ht="28.5">
       <c r="B98" s="1">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -6869,7 +7024,7 @@
       <c r="AL98" s="7"/>
       <c r="AM98" s="7"/>
     </row>
-    <row r="99" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:39" ht="28.5">
       <c r="B99" s="1">
         <f t="shared" si="1"/>
         <v>93</v>
@@ -6922,7 +7077,7 @@
       <c r="AL99" s="7"/>
       <c r="AM99" s="7"/>
     </row>
-    <row r="100" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:39">
       <c r="B100" s="1">
         <f t="shared" si="1"/>
         <v>94</v>
@@ -6975,7 +7130,7 @@
       <c r="AL100" s="7"/>
       <c r="AM100" s="7"/>
     </row>
-    <row r="101" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:39" ht="28.5">
       <c r="B101" s="1">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -7028,7 +7183,7 @@
       <c r="AL101" s="7"/>
       <c r="AM101" s="7"/>
     </row>
-    <row r="102" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:39" ht="42.75">
       <c r="B102" s="1">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -7081,7 +7236,7 @@
       <c r="AL102" s="7"/>
       <c r="AM102" s="7"/>
     </row>
-    <row r="103" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:39" ht="28.5">
       <c r="B103" s="1">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -7094,7 +7249,9 @@
       </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
-      <c r="G103" s="1"/>
+      <c r="G103" s="1" t="s">
+        <v>150</v>
+      </c>
       <c r="H103" s="8" t="s">
         <v>189</v>
       </c>
@@ -7134,7 +7291,7 @@
       <c r="AL103" s="7"/>
       <c r="AM103" s="7"/>
     </row>
-    <row r="104" spans="2:39" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:39" ht="42.75">
       <c r="B104" s="1">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -7189,7 +7346,7 @@
       <c r="AL104" s="7"/>
       <c r="AM104" s="7"/>
     </row>
-    <row r="105" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:39">
       <c r="B105" s="1">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -7240,7 +7397,7 @@
       <c r="AL105" s="7"/>
       <c r="AM105" s="7"/>
     </row>
-    <row r="106" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:39">
       <c r="B106" s="1">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -7295,7 +7452,7 @@
       <c r="AL106" s="7"/>
       <c r="AM106" s="7"/>
     </row>
-    <row r="107" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:39" ht="28.5">
       <c r="B107" s="1">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -7348,7 +7505,7 @@
       <c r="AL107" s="7"/>
       <c r="AM107" s="7"/>
     </row>
-    <row r="108" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:39">
       <c r="B108" s="1">
         <f t="shared" si="1"/>
         <v>102</v>
@@ -7372,17 +7529,33 @@
       <c r="K108" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L108" s="1"/>
-      <c r="M108" s="1"/>
-      <c r="N108" s="1"/>
-      <c r="O108" s="7"/>
+      <c r="L108" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="M108" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="N108" s="1">
+        <v>100</v>
+      </c>
+      <c r="O108" s="7" t="s">
+        <v>203</v>
+      </c>
       <c r="P108" s="7"/>
       <c r="Q108" s="7"/>
       <c r="R108" s="7"/>
-      <c r="S108" s="7"/>
-      <c r="T108" s="7"/>
-      <c r="U108" s="7"/>
-      <c r="V108" s="7"/>
+      <c r="S108" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="T108" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="U108" s="7">
+        <v>1</v>
+      </c>
+      <c r="V108" s="7" t="s">
+        <v>204</v>
+      </c>
       <c r="W108" s="7"/>
       <c r="X108" s="7"/>
       <c r="Y108" s="7"/>
@@ -7401,7 +7574,7 @@
       <c r="AL108" s="7"/>
       <c r="AM108" s="7"/>
     </row>
-    <row r="109" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:39" ht="28.5">
       <c r="B109" s="1">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -7425,17 +7598,33 @@
       <c r="K109" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L109" s="1"/>
-      <c r="M109" s="1"/>
-      <c r="N109" s="1"/>
-      <c r="O109" s="7"/>
+      <c r="L109" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="M109" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="N109" s="1">
+        <v>100</v>
+      </c>
+      <c r="O109" s="7" t="s">
+        <v>205</v>
+      </c>
       <c r="P109" s="7"/>
       <c r="Q109" s="7"/>
       <c r="R109" s="7"/>
-      <c r="S109" s="7"/>
-      <c r="T109" s="7"/>
-      <c r="U109" s="7"/>
-      <c r="V109" s="7"/>
+      <c r="S109" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="T109" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="U109" s="7">
+        <v>1</v>
+      </c>
+      <c r="V109" s="7" t="s">
+        <v>206</v>
+      </c>
       <c r="W109" s="7"/>
       <c r="X109" s="7"/>
       <c r="Y109" s="7"/>
@@ -7454,7 +7643,7 @@
       <c r="AL109" s="7"/>
       <c r="AM109" s="7"/>
     </row>
-    <row r="110" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:39" ht="28.5">
       <c r="B110" s="1">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -7469,7 +7658,7 @@
       <c r="F110" s="1"/>
       <c r="G110" s="1"/>
       <c r="H110" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I110" s="1"/>
       <c r="J110" s="1" t="s">
@@ -7507,7 +7696,7 @@
       <c r="AL110" s="7"/>
       <c r="AM110" s="7"/>
     </row>
-    <row r="111" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:39" ht="57">
       <c r="B111" s="1">
         <f t="shared" si="1"/>
         <v>105</v>
@@ -7522,7 +7711,7 @@
       <c r="F111" s="1"/>
       <c r="G111" s="1"/>
       <c r="H111" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I111" s="1"/>
       <c r="J111" s="1" t="s">
@@ -7560,7 +7749,7 @@
       <c r="AL111" s="7"/>
       <c r="AM111" s="7"/>
     </row>
-    <row r="112" spans="2:39" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:39" ht="28.5">
       <c r="B112" s="1">
         <f t="shared" si="1"/>
         <v>106</v>
@@ -7575,7 +7764,7 @@
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
       <c r="H112" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="I112" s="1"/>
       <c r="J112" s="1" t="s">
@@ -7613,7 +7802,7 @@
       <c r="AL112" s="7"/>
       <c r="AM112" s="7"/>
     </row>
-    <row r="113" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:39" ht="42.75">
       <c r="B113" s="1">
         <f t="shared" si="1"/>
         <v>107</v>
@@ -7628,7 +7817,7 @@
       <c r="F113" s="1"/>
       <c r="G113" s="1"/>
       <c r="H113" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I113" s="1"/>
       <c r="J113" s="1" t="s">
@@ -7666,7 +7855,7 @@
       <c r="AL113" s="7"/>
       <c r="AM113" s="7"/>
     </row>
-    <row r="114" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:39" ht="28.5">
       <c r="B114" s="1">
         <f t="shared" si="1"/>
         <v>108</v>
@@ -7678,10 +7867,12 @@
         <v>13</v>
       </c>
       <c r="E114" s="1"/>
-      <c r="F114" s="1"/>
+      <c r="F114" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="G114" s="1"/>
       <c r="H114" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I114" s="1"/>
       <c r="J114" s="1" t="s">
@@ -7719,7 +7910,7 @@
       <c r="AL114" s="7"/>
       <c r="AM114" s="7"/>
     </row>
-    <row r="115" spans="2:39" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:39">
       <c r="B115" s="1">
         <f t="shared" si="1"/>
         <v>109</v>
@@ -7731,13 +7922,9 @@
         <v>13</v>
       </c>
       <c r="E115" s="1"/>
-      <c r="F115" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="F115" s="1"/>
       <c r="G115" s="1"/>
-      <c r="H115" s="8" t="s">
-        <v>200</v>
-      </c>
+      <c r="H115" s="8"/>
       <c r="I115" s="1"/>
       <c r="J115" s="1" t="s">
         <v>13</v>
@@ -7774,7 +7961,7 @@
       <c r="AL115" s="7"/>
       <c r="AM115" s="7"/>
     </row>
-    <row r="116" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:39">
       <c r="B116" s="1">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -7786,9 +7973,15 @@
         <v>13</v>
       </c>
       <c r="E116" s="1"/>
-      <c r="F116" s="1"/>
-      <c r="G116" s="1"/>
-      <c r="H116" s="8"/>
+      <c r="F116" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H116" s="8" t="s">
+        <v>202</v>
+      </c>
       <c r="I116" s="1"/>
       <c r="J116" s="1" t="s">
         <v>13</v>
@@ -7825,7 +8018,7 @@
       <c r="AL116" s="7"/>
       <c r="AM116" s="7"/>
     </row>
-    <row r="117" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:39">
       <c r="B117" s="1">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -7876,7 +8069,7 @@
       <c r="AL117" s="7"/>
       <c r="AM117" s="7"/>
     </row>
-    <row r="118" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:39" ht="28.5">
       <c r="B118" s="1">
         <f t="shared" si="1"/>
         <v>112</v>
@@ -7889,8 +8082,12 @@
       </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
-      <c r="G118" s="1"/>
-      <c r="H118" s="8"/>
+      <c r="G118" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H118" s="8" t="s">
+        <v>207</v>
+      </c>
       <c r="I118" s="1"/>
       <c r="J118" s="1" t="s">
         <v>13</v>
@@ -7927,7 +8124,7 @@
       <c r="AL118" s="7"/>
       <c r="AM118" s="7"/>
     </row>
-    <row r="119" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:39" ht="28.5">
       <c r="B119" s="1">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -7941,7 +8138,9 @@
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
-      <c r="H119" s="8"/>
+      <c r="H119" s="8" t="s">
+        <v>208</v>
+      </c>
       <c r="I119" s="1"/>
       <c r="J119" s="1" t="s">
         <v>13</v>
@@ -7978,7 +8177,7 @@
       <c r="AL119" s="7"/>
       <c r="AM119" s="7"/>
     </row>
-    <row r="120" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:39" ht="42.75">
       <c r="B120" s="1">
         <f t="shared" si="1"/>
         <v>114</v>
@@ -7992,7 +8191,9 @@
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
-      <c r="H120" s="8"/>
+      <c r="H120" s="8" t="s">
+        <v>209</v>
+      </c>
       <c r="I120" s="1"/>
       <c r="J120" s="1" t="s">
         <v>13</v>
@@ -8029,7 +8230,7 @@
       <c r="AL120" s="7"/>
       <c r="AM120" s="7"/>
     </row>
-    <row r="121" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:39" ht="42.75">
       <c r="B121" s="1">
         <f t="shared" si="1"/>
         <v>115</v>
@@ -8043,7 +8244,9 @@
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
-      <c r="H121" s="8"/>
+      <c r="H121" s="8" t="s">
+        <v>210</v>
+      </c>
       <c r="I121" s="1"/>
       <c r="J121" s="1" t="s">
         <v>13</v>
@@ -8080,7 +8283,7 @@
       <c r="AL121" s="7"/>
       <c r="AM121" s="7"/>
     </row>
-    <row r="122" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:39" ht="28.5">
       <c r="B122" s="1">
         <f t="shared" si="1"/>
         <v>116</v>
@@ -8094,7 +8297,9 @@
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
-      <c r="H122" s="8"/>
+      <c r="H122" s="8" t="s">
+        <v>211</v>
+      </c>
       <c r="I122" s="1"/>
       <c r="J122" s="1" t="s">
         <v>13</v>
@@ -8105,17 +8310,31 @@
       <c r="L122" s="1"/>
       <c r="M122" s="1"/>
       <c r="N122" s="1"/>
-      <c r="O122" s="7"/>
+      <c r="O122" s="7" t="s">
+        <v>214</v>
+      </c>
       <c r="P122" s="7"/>
       <c r="Q122" s="7"/>
-      <c r="R122" s="7"/>
-      <c r="S122" s="7"/>
-      <c r="T122" s="7"/>
-      <c r="U122" s="7"/>
-      <c r="V122" s="7"/>
+      <c r="R122" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="S122" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="T122" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="U122" s="7">
+        <v>9</v>
+      </c>
+      <c r="V122" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="W122" s="7"/>
       <c r="X122" s="7"/>
-      <c r="Y122" s="7"/>
+      <c r="Y122" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="Z122" s="7"/>
       <c r="AA122" s="7"/>
       <c r="AB122" s="7"/>
@@ -8131,7 +8350,7 @@
       <c r="AL122" s="7"/>
       <c r="AM122" s="7"/>
     </row>
-    <row r="123" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:39" ht="42.75">
       <c r="B123" s="1">
         <f t="shared" si="1"/>
         <v>117</v>
@@ -8144,8 +8363,12 @@
       </c>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
-      <c r="G123" s="1"/>
-      <c r="H123" s="8"/>
+      <c r="G123" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H123" s="8" t="s">
+        <v>213</v>
+      </c>
       <c r="I123" s="1"/>
       <c r="J123" s="1" t="s">
         <v>13</v>
@@ -8182,7 +8405,7 @@
       <c r="AL123" s="7"/>
       <c r="AM123" s="7"/>
     </row>
-    <row r="124" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:39" ht="42.75">
       <c r="B124" s="1">
         <f t="shared" si="1"/>
         <v>118</v>
@@ -8195,8 +8418,12 @@
       </c>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="1"/>
-      <c r="H124" s="8"/>
+      <c r="G124" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H124" s="8" t="s">
+        <v>216</v>
+      </c>
       <c r="I124" s="1"/>
       <c r="J124" s="1" t="s">
         <v>13</v>
@@ -8233,7 +8460,7 @@
       <c r="AL124" s="7"/>
       <c r="AM124" s="7"/>
     </row>
-    <row r="125" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:39" ht="42.75">
       <c r="B125" s="1">
         <f t="shared" si="1"/>
         <v>119</v>
@@ -8247,8 +8474,12 @@
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
-      <c r="H125" s="8"/>
-      <c r="I125" s="1"/>
+      <c r="H125" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="I125" s="1" t="s">
+        <v>219</v>
+      </c>
       <c r="J125" s="1" t="s">
         <v>13</v>
       </c>
@@ -8284,7 +8515,7 @@
       <c r="AL125" s="7"/>
       <c r="AM125" s="7"/>
     </row>
-    <row r="126" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:39" ht="42.75">
       <c r="B126" s="1">
         <f t="shared" si="1"/>
         <v>120</v>
@@ -8297,9 +8528,15 @@
       </c>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-      <c r="G126" s="1"/>
-      <c r="H126" s="8"/>
-      <c r="I126" s="1"/>
+      <c r="G126" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H126" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="I126" s="1" t="s">
+        <v>219</v>
+      </c>
       <c r="J126" s="1" t="s">
         <v>13</v>
       </c>
@@ -8335,7 +8572,7 @@
       <c r="AL126" s="7"/>
       <c r="AM126" s="7"/>
     </row>
-    <row r="127" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:39" ht="42.75">
       <c r="B127" s="1">
         <f t="shared" si="1"/>
         <v>121</v>
@@ -8348,8 +8585,12 @@
       </c>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
-      <c r="G127" s="1"/>
-      <c r="H127" s="8"/>
+      <c r="G127" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H127" s="8" t="s">
+        <v>220</v>
+      </c>
       <c r="I127" s="1"/>
       <c r="J127" s="1" t="s">
         <v>13</v>
@@ -8386,7 +8627,7 @@
       <c r="AL127" s="7"/>
       <c r="AM127" s="7"/>
     </row>
-    <row r="128" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:39" ht="28.5">
       <c r="B128" s="1">
         <f t="shared" si="1"/>
         <v>122</v>
@@ -8400,7 +8641,9 @@
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
-      <c r="H128" s="8"/>
+      <c r="H128" s="8" t="s">
+        <v>221</v>
+      </c>
       <c r="I128" s="1"/>
       <c r="J128" s="1" t="s">
         <v>13</v>
@@ -8437,7 +8680,7 @@
       <c r="AL128" s="7"/>
       <c r="AM128" s="7"/>
     </row>
-    <row r="129" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:39" ht="42.75">
       <c r="B129" s="1">
         <f t="shared" si="1"/>
         <v>123</v>
@@ -8451,7 +8694,9 @@
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
-      <c r="H129" s="8"/>
+      <c r="H129" s="8" t="s">
+        <v>222</v>
+      </c>
       <c r="I129" s="1"/>
       <c r="J129" s="1" t="s">
         <v>13</v>
@@ -8488,7 +8733,7 @@
       <c r="AL129" s="7"/>
       <c r="AM129" s="7"/>
     </row>
-    <row r="130" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:39" ht="28.5">
       <c r="B130" s="1">
         <f t="shared" si="1"/>
         <v>124</v>
@@ -8502,7 +8747,9 @@
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
-      <c r="H130" s="8"/>
+      <c r="H130" s="8" t="s">
+        <v>223</v>
+      </c>
       <c r="I130" s="1"/>
       <c r="J130" s="1" t="s">
         <v>13</v>
@@ -8539,7 +8786,7 @@
       <c r="AL130" s="7"/>
       <c r="AM130" s="7"/>
     </row>
-    <row r="131" spans="2:39" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:39" ht="42.75">
       <c r="B131" s="1">
         <f t="shared" si="1"/>
         <v>125</v>
@@ -8553,7 +8800,9 @@
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
-      <c r="H131" s="8"/>
+      <c r="H131" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="I131" s="1"/>
       <c r="J131" s="1" t="s">
         <v>13</v>
@@ -8590,27 +8839,22 @@
       <c r="AL131" s="7"/>
       <c r="AM131" s="7"/>
     </row>
-    <row r="132" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="B132" s="1">
-        <f t="shared" si="1"/>
-        <v>126</v>
-      </c>
+    <row r="132" spans="2:39" ht="28.5">
+      <c r="B132" s="1"/>
       <c r="C132" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D132" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="D132" s="1"/>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
-      <c r="H132" s="8"/>
+      <c r="H132" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="I132" s="1"/>
-      <c r="J132" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="J132" s="1"/>
       <c r="K132" s="1" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="L132" s="1"/>
       <c r="M132" s="1"/>
@@ -8641,32 +8885,2058 @@
       <c r="AL132" s="7"/>
       <c r="AM132" s="7"/>
     </row>
+    <row r="133" spans="2:39" ht="28.5">
+      <c r="B133" s="1"/>
+      <c r="C133" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D133" s="1"/>
+      <c r="E133" s="1"/>
+      <c r="F133" s="1"/>
+      <c r="G133" s="1"/>
+      <c r="H133" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="I133" s="1"/>
+      <c r="J133" s="1"/>
+      <c r="K133" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L133" s="1"/>
+      <c r="M133" s="1"/>
+      <c r="N133" s="1"/>
+      <c r="O133" s="7"/>
+      <c r="P133" s="7"/>
+      <c r="Q133" s="7"/>
+      <c r="R133" s="7"/>
+      <c r="S133" s="7"/>
+      <c r="T133" s="7"/>
+      <c r="U133" s="7"/>
+      <c r="V133" s="7"/>
+      <c r="W133" s="7"/>
+      <c r="X133" s="7"/>
+      <c r="Y133" s="7"/>
+      <c r="Z133" s="7"/>
+      <c r="AA133" s="7"/>
+      <c r="AB133" s="7"/>
+      <c r="AC133" s="7"/>
+      <c r="AD133" s="7"/>
+      <c r="AE133" s="7"/>
+      <c r="AF133" s="7"/>
+      <c r="AG133" s="7"/>
+      <c r="AH133" s="7"/>
+      <c r="AI133" s="7"/>
+      <c r="AJ133" s="7"/>
+      <c r="AK133" s="7"/>
+      <c r="AL133" s="7"/>
+      <c r="AM133" s="7"/>
+    </row>
+    <row r="134" spans="2:39" ht="42.75">
+      <c r="B134" s="1"/>
+      <c r="C134" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D134" s="1"/>
+      <c r="E134" s="1"/>
+      <c r="F134" s="1"/>
+      <c r="G134" s="1"/>
+      <c r="H134" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="I134" s="1"/>
+      <c r="J134" s="1"/>
+      <c r="K134" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L134" s="1"/>
+      <c r="M134" s="1"/>
+      <c r="N134" s="1"/>
+      <c r="O134" s="7"/>
+      <c r="P134" s="7"/>
+      <c r="Q134" s="7"/>
+      <c r="R134" s="7"/>
+      <c r="S134" s="7"/>
+      <c r="T134" s="7"/>
+      <c r="U134" s="7"/>
+      <c r="V134" s="7"/>
+      <c r="W134" s="7"/>
+      <c r="X134" s="7"/>
+      <c r="Y134" s="7"/>
+      <c r="Z134" s="7"/>
+      <c r="AA134" s="7"/>
+      <c r="AB134" s="7"/>
+      <c r="AC134" s="7"/>
+      <c r="AD134" s="7"/>
+      <c r="AE134" s="7"/>
+      <c r="AF134" s="7"/>
+      <c r="AG134" s="7"/>
+      <c r="AH134" s="7"/>
+      <c r="AI134" s="7"/>
+      <c r="AJ134" s="7"/>
+      <c r="AK134" s="7"/>
+      <c r="AL134" s="7"/>
+      <c r="AM134" s="7"/>
+    </row>
+    <row r="135" spans="2:39">
+      <c r="B135" s="1"/>
+      <c r="C135" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D135" s="1"/>
+      <c r="E135" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F135" s="1"/>
+      <c r="G135" s="1"/>
+      <c r="H135" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I135" s="1"/>
+      <c r="J135" s="1"/>
+      <c r="K135" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L135" s="1"/>
+      <c r="M135" s="1"/>
+      <c r="N135" s="1"/>
+      <c r="O135" s="7"/>
+      <c r="P135" s="7"/>
+      <c r="Q135" s="7"/>
+      <c r="R135" s="7"/>
+      <c r="S135" s="7"/>
+      <c r="T135" s="7"/>
+      <c r="U135" s="7"/>
+      <c r="V135" s="7"/>
+      <c r="W135" s="7"/>
+      <c r="X135" s="7"/>
+      <c r="Y135" s="7"/>
+      <c r="Z135" s="7"/>
+      <c r="AA135" s="7"/>
+      <c r="AB135" s="7"/>
+      <c r="AC135" s="7"/>
+      <c r="AD135" s="7"/>
+      <c r="AE135" s="7"/>
+      <c r="AF135" s="7"/>
+      <c r="AG135" s="7"/>
+      <c r="AH135" s="7"/>
+      <c r="AI135" s="7"/>
+      <c r="AJ135" s="7"/>
+      <c r="AK135" s="7"/>
+      <c r="AL135" s="7"/>
+      <c r="AM135" s="7"/>
+    </row>
+    <row r="136" spans="2:39" ht="42.75">
+      <c r="B136" s="1"/>
+      <c r="C136" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D136" s="1"/>
+      <c r="E136" s="1"/>
+      <c r="F136" s="1"/>
+      <c r="G136" s="1"/>
+      <c r="H136" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="I136" s="1"/>
+      <c r="J136" s="1"/>
+      <c r="K136" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L136" s="1"/>
+      <c r="M136" s="1"/>
+      <c r="N136" s="1"/>
+      <c r="O136" s="7"/>
+      <c r="P136" s="7"/>
+      <c r="Q136" s="7"/>
+      <c r="R136" s="7"/>
+      <c r="S136" s="7"/>
+      <c r="T136" s="7"/>
+      <c r="U136" s="7"/>
+      <c r="V136" s="7"/>
+      <c r="W136" s="7"/>
+      <c r="X136" s="7"/>
+      <c r="Y136" s="7"/>
+      <c r="Z136" s="7"/>
+      <c r="AA136" s="7"/>
+      <c r="AB136" s="7"/>
+      <c r="AC136" s="7"/>
+      <c r="AD136" s="7"/>
+      <c r="AE136" s="7"/>
+      <c r="AF136" s="7"/>
+      <c r="AG136" s="7"/>
+      <c r="AH136" s="7"/>
+      <c r="AI136" s="7"/>
+      <c r="AJ136" s="7"/>
+      <c r="AK136" s="7"/>
+      <c r="AL136" s="7"/>
+      <c r="AM136" s="7"/>
+    </row>
+    <row r="137" spans="2:39">
+      <c r="B137" s="1"/>
+      <c r="C137" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D137" s="1"/>
+      <c r="E137" s="1"/>
+      <c r="F137" s="1"/>
+      <c r="G137" s="1"/>
+      <c r="H137" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I137" s="1"/>
+      <c r="J137" s="1"/>
+      <c r="K137" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L137" s="1"/>
+      <c r="M137" s="1"/>
+      <c r="N137" s="1"/>
+      <c r="O137" s="7"/>
+      <c r="P137" s="7"/>
+      <c r="Q137" s="7"/>
+      <c r="R137" s="7"/>
+      <c r="S137" s="7"/>
+      <c r="T137" s="7"/>
+      <c r="U137" s="7"/>
+      <c r="V137" s="7"/>
+      <c r="W137" s="7"/>
+      <c r="X137" s="7"/>
+      <c r="Y137" s="7"/>
+      <c r="Z137" s="7"/>
+      <c r="AA137" s="7"/>
+      <c r="AB137" s="7"/>
+      <c r="AC137" s="7"/>
+      <c r="AD137" s="7"/>
+      <c r="AE137" s="7"/>
+      <c r="AF137" s="7"/>
+      <c r="AG137" s="7"/>
+      <c r="AH137" s="7"/>
+      <c r="AI137" s="7"/>
+      <c r="AJ137" s="7"/>
+      <c r="AK137" s="7"/>
+      <c r="AL137" s="7"/>
+      <c r="AM137" s="7"/>
+    </row>
+    <row r="138" spans="2:39" ht="42.75">
+      <c r="B138" s="1"/>
+      <c r="C138" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D138" s="1"/>
+      <c r="E138" s="1"/>
+      <c r="F138" s="1"/>
+      <c r="G138" s="1"/>
+      <c r="H138" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="I138" s="1"/>
+      <c r="J138" s="1"/>
+      <c r="K138" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L138" s="1"/>
+      <c r="M138" s="1"/>
+      <c r="N138" s="1"/>
+      <c r="O138" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="P138" s="7"/>
+      <c r="Q138" s="7"/>
+      <c r="R138" s="7"/>
+      <c r="S138" s="7"/>
+      <c r="T138" s="7"/>
+      <c r="U138" s="7"/>
+      <c r="V138" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="W138" s="7"/>
+      <c r="X138" s="7"/>
+      <c r="Y138" s="7"/>
+      <c r="Z138" s="7"/>
+      <c r="AA138" s="7"/>
+      <c r="AB138" s="7"/>
+      <c r="AC138" s="7"/>
+      <c r="AD138" s="7"/>
+      <c r="AE138" s="7"/>
+      <c r="AF138" s="7"/>
+      <c r="AG138" s="7"/>
+      <c r="AH138" s="7"/>
+      <c r="AI138" s="7"/>
+      <c r="AJ138" s="7"/>
+      <c r="AK138" s="7"/>
+      <c r="AL138" s="7"/>
+      <c r="AM138" s="7"/>
+    </row>
+    <row r="139" spans="2:39" ht="42.75">
+      <c r="B139" s="1"/>
+      <c r="C139" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D139" s="1"/>
+      <c r="E139" s="1"/>
+      <c r="F139" s="1"/>
+      <c r="G139" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H139" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="I139" s="1"/>
+      <c r="J139" s="1"/>
+      <c r="K139" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L139" s="1"/>
+      <c r="M139" s="1"/>
+      <c r="N139" s="1"/>
+      <c r="O139" s="7"/>
+      <c r="P139" s="7"/>
+      <c r="Q139" s="7"/>
+      <c r="R139" s="7"/>
+      <c r="S139" s="7"/>
+      <c r="T139" s="7"/>
+      <c r="U139" s="7"/>
+      <c r="V139" s="7"/>
+      <c r="W139" s="7"/>
+      <c r="X139" s="7"/>
+      <c r="Y139" s="7"/>
+      <c r="Z139" s="7"/>
+      <c r="AA139" s="7"/>
+      <c r="AB139" s="7"/>
+      <c r="AC139" s="7"/>
+      <c r="AD139" s="7"/>
+      <c r="AE139" s="7"/>
+      <c r="AF139" s="7"/>
+      <c r="AG139" s="7"/>
+      <c r="AH139" s="7"/>
+      <c r="AI139" s="7"/>
+      <c r="AJ139" s="7"/>
+      <c r="AK139" s="7"/>
+      <c r="AL139" s="7"/>
+      <c r="AM139" s="7"/>
+    </row>
+    <row r="140" spans="2:39" ht="28.5">
+      <c r="B140" s="1"/>
+      <c r="C140" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D140" s="1"/>
+      <c r="E140" s="1"/>
+      <c r="F140" s="1"/>
+      <c r="G140" s="1"/>
+      <c r="H140" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="I140" s="1"/>
+      <c r="J140" s="1"/>
+      <c r="K140" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L140" s="1"/>
+      <c r="M140" s="1"/>
+      <c r="N140" s="1"/>
+      <c r="O140" s="7"/>
+      <c r="P140" s="7"/>
+      <c r="Q140" s="7"/>
+      <c r="R140" s="7"/>
+      <c r="S140" s="7"/>
+      <c r="T140" s="7"/>
+      <c r="U140" s="7"/>
+      <c r="V140" s="7"/>
+      <c r="W140" s="7"/>
+      <c r="X140" s="7"/>
+      <c r="Y140" s="7"/>
+      <c r="Z140" s="7"/>
+      <c r="AA140" s="7"/>
+      <c r="AB140" s="7"/>
+      <c r="AC140" s="7"/>
+      <c r="AD140" s="7"/>
+      <c r="AE140" s="7"/>
+      <c r="AF140" s="7"/>
+      <c r="AG140" s="7"/>
+      <c r="AH140" s="7"/>
+      <c r="AI140" s="7"/>
+      <c r="AJ140" s="7"/>
+      <c r="AK140" s="7"/>
+      <c r="AL140" s="7"/>
+      <c r="AM140" s="7"/>
+    </row>
+    <row r="141" spans="2:39" ht="28.5">
+      <c r="B141" s="1"/>
+      <c r="C141" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D141" s="1"/>
+      <c r="E141" s="1"/>
+      <c r="F141" s="1"/>
+      <c r="G141" s="1"/>
+      <c r="H141" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="I141" s="1"/>
+      <c r="J141" s="1"/>
+      <c r="K141" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L141" s="1"/>
+      <c r="M141" s="1"/>
+      <c r="N141" s="1"/>
+      <c r="O141" s="7"/>
+      <c r="P141" s="7"/>
+      <c r="Q141" s="7"/>
+      <c r="R141" s="7"/>
+      <c r="S141" s="7"/>
+      <c r="T141" s="7"/>
+      <c r="U141" s="7"/>
+      <c r="V141" s="7"/>
+      <c r="W141" s="7"/>
+      <c r="X141" s="7"/>
+      <c r="Y141" s="7"/>
+      <c r="Z141" s="7"/>
+      <c r="AA141" s="7"/>
+      <c r="AB141" s="7"/>
+      <c r="AC141" s="7"/>
+      <c r="AD141" s="7"/>
+      <c r="AE141" s="7"/>
+      <c r="AF141" s="7"/>
+      <c r="AG141" s="7"/>
+      <c r="AH141" s="7"/>
+      <c r="AI141" s="7"/>
+      <c r="AJ141" s="7"/>
+      <c r="AK141" s="7"/>
+      <c r="AL141" s="7"/>
+      <c r="AM141" s="7"/>
+    </row>
+    <row r="142" spans="2:39">
+      <c r="B142" s="1"/>
+      <c r="C142" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D142" s="1"/>
+      <c r="E142" s="1"/>
+      <c r="F142" s="1"/>
+      <c r="G142" s="1"/>
+      <c r="H142" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="I142" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="J142" s="1"/>
+      <c r="K142" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L142" s="1"/>
+      <c r="M142" s="1"/>
+      <c r="N142" s="1"/>
+      <c r="O142" s="7"/>
+      <c r="P142" s="7"/>
+      <c r="Q142" s="7"/>
+      <c r="R142" s="7"/>
+      <c r="S142" s="7"/>
+      <c r="T142" s="7"/>
+      <c r="U142" s="7"/>
+      <c r="V142" s="7"/>
+      <c r="W142" s="7"/>
+      <c r="X142" s="7"/>
+      <c r="Y142" s="7"/>
+      <c r="Z142" s="7"/>
+      <c r="AA142" s="7"/>
+      <c r="AB142" s="7"/>
+      <c r="AC142" s="7"/>
+      <c r="AD142" s="7"/>
+      <c r="AE142" s="7"/>
+      <c r="AF142" s="7"/>
+      <c r="AG142" s="7"/>
+      <c r="AH142" s="7"/>
+      <c r="AI142" s="7"/>
+      <c r="AJ142" s="7"/>
+      <c r="AK142" s="7"/>
+      <c r="AL142" s="7"/>
+      <c r="AM142" s="7"/>
+    </row>
+    <row r="143" spans="2:39" ht="57">
+      <c r="B143" s="1"/>
+      <c r="C143" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D143" s="1"/>
+      <c r="E143" s="1"/>
+      <c r="F143" s="1"/>
+      <c r="G143" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H143" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="I143" s="1"/>
+      <c r="J143" s="1"/>
+      <c r="K143" s="1"/>
+      <c r="L143" s="1"/>
+      <c r="M143" s="1"/>
+      <c r="N143" s="1"/>
+      <c r="O143" s="7"/>
+      <c r="P143" s="7"/>
+      <c r="Q143" s="7"/>
+      <c r="R143" s="7"/>
+      <c r="S143" s="7"/>
+      <c r="T143" s="7"/>
+      <c r="U143" s="7"/>
+      <c r="V143" s="7"/>
+      <c r="W143" s="7"/>
+      <c r="X143" s="7"/>
+      <c r="Y143" s="7"/>
+      <c r="Z143" s="7"/>
+      <c r="AA143" s="7"/>
+      <c r="AB143" s="7"/>
+      <c r="AC143" s="7"/>
+      <c r="AD143" s="7"/>
+      <c r="AE143" s="7"/>
+      <c r="AF143" s="7"/>
+      <c r="AG143" s="7"/>
+      <c r="AH143" s="7"/>
+      <c r="AI143" s="7"/>
+      <c r="AJ143" s="7"/>
+      <c r="AK143" s="7"/>
+      <c r="AL143" s="7"/>
+      <c r="AM143" s="7"/>
+    </row>
+    <row r="144" spans="2:39" ht="28.5">
+      <c r="B144" s="1"/>
+      <c r="C144" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D144" s="1"/>
+      <c r="E144" s="1"/>
+      <c r="F144" s="1"/>
+      <c r="G144" s="1"/>
+      <c r="H144" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="I144" s="1"/>
+      <c r="J144" s="1"/>
+      <c r="K144" s="1"/>
+      <c r="L144" s="1"/>
+      <c r="M144" s="1"/>
+      <c r="N144" s="1"/>
+      <c r="O144" s="7"/>
+      <c r="P144" s="7"/>
+      <c r="Q144" s="7"/>
+      <c r="R144" s="7"/>
+      <c r="S144" s="7"/>
+      <c r="T144" s="7"/>
+      <c r="U144" s="7"/>
+      <c r="V144" s="7"/>
+      <c r="W144" s="7"/>
+      <c r="X144" s="7"/>
+      <c r="Y144" s="7"/>
+      <c r="Z144" s="7"/>
+      <c r="AA144" s="7"/>
+      <c r="AB144" s="7"/>
+      <c r="AC144" s="7"/>
+      <c r="AD144" s="7"/>
+      <c r="AE144" s="7"/>
+      <c r="AF144" s="7"/>
+      <c r="AG144" s="7"/>
+      <c r="AH144" s="7"/>
+      <c r="AI144" s="7"/>
+      <c r="AJ144" s="7"/>
+      <c r="AK144" s="7"/>
+      <c r="AL144" s="7"/>
+      <c r="AM144" s="7"/>
+    </row>
+    <row r="145" spans="2:39" ht="42.75">
+      <c r="B145" s="1"/>
+      <c r="C145" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D145" s="1"/>
+      <c r="E145" s="1"/>
+      <c r="F145" s="1"/>
+      <c r="G145" s="1"/>
+      <c r="H145" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="I145" s="1"/>
+      <c r="J145" s="1"/>
+      <c r="K145" s="1"/>
+      <c r="L145" s="1"/>
+      <c r="M145" s="1"/>
+      <c r="N145" s="1"/>
+      <c r="O145" s="7"/>
+      <c r="P145" s="7"/>
+      <c r="Q145" s="7"/>
+      <c r="R145" s="7"/>
+      <c r="S145" s="7"/>
+      <c r="T145" s="7"/>
+      <c r="U145" s="7"/>
+      <c r="V145" s="7"/>
+      <c r="W145" s="7"/>
+      <c r="X145" s="7"/>
+      <c r="Y145" s="7"/>
+      <c r="Z145" s="7"/>
+      <c r="AA145" s="7"/>
+      <c r="AB145" s="7"/>
+      <c r="AC145" s="7"/>
+      <c r="AD145" s="7"/>
+      <c r="AE145" s="7"/>
+      <c r="AF145" s="7"/>
+      <c r="AG145" s="7"/>
+      <c r="AH145" s="7"/>
+      <c r="AI145" s="7"/>
+      <c r="AJ145" s="7"/>
+      <c r="AK145" s="7"/>
+      <c r="AL145" s="7"/>
+      <c r="AM145" s="7"/>
+    </row>
+    <row r="146" spans="2:39" ht="28.5">
+      <c r="B146" s="1"/>
+      <c r="C146" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D146" s="1"/>
+      <c r="E146" s="1"/>
+      <c r="F146" s="1"/>
+      <c r="G146" s="1"/>
+      <c r="H146" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="I146" s="1"/>
+      <c r="J146" s="1"/>
+      <c r="K146" s="1"/>
+      <c r="L146" s="1"/>
+      <c r="M146" s="1"/>
+      <c r="N146" s="1"/>
+      <c r="O146" s="7"/>
+      <c r="P146" s="7"/>
+      <c r="Q146" s="7"/>
+      <c r="R146" s="7"/>
+      <c r="S146" s="7"/>
+      <c r="T146" s="7"/>
+      <c r="U146" s="7"/>
+      <c r="V146" s="7"/>
+      <c r="W146" s="7"/>
+      <c r="X146" s="7"/>
+      <c r="Y146" s="7"/>
+      <c r="Z146" s="7"/>
+      <c r="AA146" s="7"/>
+      <c r="AB146" s="7"/>
+      <c r="AC146" s="7"/>
+      <c r="AD146" s="7"/>
+      <c r="AE146" s="7"/>
+      <c r="AF146" s="7"/>
+      <c r="AG146" s="7"/>
+      <c r="AH146" s="7"/>
+      <c r="AI146" s="7"/>
+      <c r="AJ146" s="7"/>
+      <c r="AK146" s="7"/>
+      <c r="AL146" s="7"/>
+      <c r="AM146" s="7"/>
+    </row>
+    <row r="147" spans="2:39" ht="42.75">
+      <c r="B147" s="1"/>
+      <c r="C147" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D147" s="1"/>
+      <c r="E147" s="1"/>
+      <c r="F147" s="1"/>
+      <c r="G147" s="1"/>
+      <c r="H147" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="I147" s="1"/>
+      <c r="J147" s="1"/>
+      <c r="K147" s="1"/>
+      <c r="L147" s="1"/>
+      <c r="M147" s="1"/>
+      <c r="N147" s="1"/>
+      <c r="O147" s="7"/>
+      <c r="P147" s="7"/>
+      <c r="Q147" s="7"/>
+      <c r="R147" s="7"/>
+      <c r="S147" s="7"/>
+      <c r="T147" s="7"/>
+      <c r="U147" s="7"/>
+      <c r="V147" s="7"/>
+      <c r="W147" s="7"/>
+      <c r="X147" s="7"/>
+      <c r="Y147" s="7"/>
+      <c r="Z147" s="7"/>
+      <c r="AA147" s="7"/>
+      <c r="AB147" s="7"/>
+      <c r="AC147" s="7"/>
+      <c r="AD147" s="7"/>
+      <c r="AE147" s="7"/>
+      <c r="AF147" s="7"/>
+      <c r="AG147" s="7"/>
+      <c r="AH147" s="7"/>
+      <c r="AI147" s="7"/>
+      <c r="AJ147" s="7"/>
+      <c r="AK147" s="7"/>
+      <c r="AL147" s="7"/>
+      <c r="AM147" s="7"/>
+    </row>
+    <row r="148" spans="2:39" ht="28.5">
+      <c r="B148" s="1"/>
+      <c r="C148" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D148" s="1"/>
+      <c r="E148" s="1"/>
+      <c r="F148" s="1"/>
+      <c r="G148" s="1"/>
+      <c r="H148" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="I148" s="1"/>
+      <c r="J148" s="1"/>
+      <c r="K148" s="1"/>
+      <c r="L148" s="1"/>
+      <c r="M148" s="1"/>
+      <c r="N148" s="1"/>
+      <c r="O148" s="7"/>
+      <c r="P148" s="7"/>
+      <c r="Q148" s="7"/>
+      <c r="R148" s="7"/>
+      <c r="S148" s="7"/>
+      <c r="T148" s="7"/>
+      <c r="U148" s="7"/>
+      <c r="V148" s="7"/>
+      <c r="W148" s="7"/>
+      <c r="X148" s="7"/>
+      <c r="Y148" s="7"/>
+      <c r="Z148" s="7"/>
+      <c r="AA148" s="7"/>
+      <c r="AB148" s="7"/>
+      <c r="AC148" s="7"/>
+      <c r="AD148" s="7"/>
+      <c r="AE148" s="7"/>
+      <c r="AF148" s="7"/>
+      <c r="AG148" s="7"/>
+      <c r="AH148" s="7"/>
+      <c r="AI148" s="7"/>
+      <c r="AJ148" s="7"/>
+      <c r="AK148" s="7"/>
+      <c r="AL148" s="7"/>
+      <c r="AM148" s="7"/>
+    </row>
+    <row r="149" spans="2:39">
+      <c r="B149" s="1"/>
+      <c r="C149" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D149" s="1"/>
+      <c r="E149" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F149" s="1"/>
+      <c r="G149" s="1"/>
+      <c r="H149" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I149" s="1"/>
+      <c r="J149" s="1"/>
+      <c r="K149" s="1"/>
+      <c r="L149" s="1"/>
+      <c r="M149" s="1"/>
+      <c r="N149" s="1"/>
+      <c r="O149" s="7"/>
+      <c r="P149" s="7"/>
+      <c r="Q149" s="7"/>
+      <c r="R149" s="7"/>
+      <c r="S149" s="7"/>
+      <c r="T149" s="7"/>
+      <c r="U149" s="7"/>
+      <c r="V149" s="7"/>
+      <c r="W149" s="7"/>
+      <c r="X149" s="7"/>
+      <c r="Y149" s="7"/>
+      <c r="Z149" s="7"/>
+      <c r="AA149" s="7"/>
+      <c r="AB149" s="7"/>
+      <c r="AC149" s="7"/>
+      <c r="AD149" s="7"/>
+      <c r="AE149" s="7"/>
+      <c r="AF149" s="7"/>
+      <c r="AG149" s="7"/>
+      <c r="AH149" s="7"/>
+      <c r="AI149" s="7"/>
+      <c r="AJ149" s="7"/>
+      <c r="AK149" s="7"/>
+      <c r="AL149" s="7"/>
+      <c r="AM149" s="7"/>
+    </row>
+    <row r="150" spans="2:39" ht="28.5">
+      <c r="B150" s="1"/>
+      <c r="C150" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D150" s="1"/>
+      <c r="E150" s="1"/>
+      <c r="F150" s="1"/>
+      <c r="G150" s="1"/>
+      <c r="H150" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="I150" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="J150" s="1"/>
+      <c r="K150" s="1"/>
+      <c r="L150" s="1"/>
+      <c r="M150" s="1"/>
+      <c r="N150" s="1"/>
+      <c r="O150" s="7"/>
+      <c r="P150" s="7"/>
+      <c r="Q150" s="7"/>
+      <c r="R150" s="7"/>
+      <c r="S150" s="7"/>
+      <c r="T150" s="7"/>
+      <c r="U150" s="7"/>
+      <c r="V150" s="7"/>
+      <c r="W150" s="7"/>
+      <c r="X150" s="7"/>
+      <c r="Y150" s="7"/>
+      <c r="Z150" s="7"/>
+      <c r="AA150" s="7"/>
+      <c r="AB150" s="7"/>
+      <c r="AC150" s="7"/>
+      <c r="AD150" s="7"/>
+      <c r="AE150" s="7"/>
+      <c r="AF150" s="7"/>
+      <c r="AG150" s="7"/>
+      <c r="AH150" s="7"/>
+      <c r="AI150" s="7"/>
+      <c r="AJ150" s="7"/>
+      <c r="AK150" s="7"/>
+      <c r="AL150" s="7"/>
+      <c r="AM150" s="7"/>
+    </row>
+    <row r="151" spans="2:39" ht="42.75">
+      <c r="B151" s="1"/>
+      <c r="C151" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D151" s="1"/>
+      <c r="E151" s="1"/>
+      <c r="F151" s="1"/>
+      <c r="G151" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H151" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="I151" s="1"/>
+      <c r="J151" s="1"/>
+      <c r="K151" s="1"/>
+      <c r="L151" s="1"/>
+      <c r="M151" s="1"/>
+      <c r="N151" s="1"/>
+      <c r="O151" s="7"/>
+      <c r="P151" s="7"/>
+      <c r="Q151" s="7"/>
+      <c r="R151" s="7"/>
+      <c r="S151" s="7"/>
+      <c r="T151" s="7"/>
+      <c r="U151" s="7"/>
+      <c r="V151" s="7"/>
+      <c r="W151" s="7"/>
+      <c r="X151" s="7"/>
+      <c r="Y151" s="7"/>
+      <c r="Z151" s="7"/>
+      <c r="AA151" s="7"/>
+      <c r="AB151" s="7"/>
+      <c r="AC151" s="7"/>
+      <c r="AD151" s="7"/>
+      <c r="AE151" s="7"/>
+      <c r="AF151" s="7"/>
+      <c r="AG151" s="7"/>
+      <c r="AH151" s="7"/>
+      <c r="AI151" s="7"/>
+      <c r="AJ151" s="7"/>
+      <c r="AK151" s="7"/>
+      <c r="AL151" s="7"/>
+      <c r="AM151" s="7"/>
+    </row>
+    <row r="152" spans="2:39" ht="42.75">
+      <c r="B152" s="1"/>
+      <c r="C152" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D152" s="1"/>
+      <c r="E152" s="1"/>
+      <c r="F152" s="1"/>
+      <c r="G152" s="1"/>
+      <c r="H152" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="I152" s="1"/>
+      <c r="J152" s="1"/>
+      <c r="K152" s="1"/>
+      <c r="L152" s="1"/>
+      <c r="M152" s="1"/>
+      <c r="N152" s="1"/>
+      <c r="O152" s="7"/>
+      <c r="P152" s="7"/>
+      <c r="Q152" s="7"/>
+      <c r="R152" s="7"/>
+      <c r="S152" s="7"/>
+      <c r="T152" s="7"/>
+      <c r="U152" s="7"/>
+      <c r="V152" s="7"/>
+      <c r="W152" s="7"/>
+      <c r="X152" s="7"/>
+      <c r="Y152" s="7"/>
+      <c r="Z152" s="7"/>
+      <c r="AA152" s="7"/>
+      <c r="AB152" s="7"/>
+      <c r="AC152" s="7"/>
+      <c r="AD152" s="7"/>
+      <c r="AE152" s="7"/>
+      <c r="AF152" s="7"/>
+      <c r="AG152" s="7"/>
+      <c r="AH152" s="7"/>
+      <c r="AI152" s="7"/>
+      <c r="AJ152" s="7"/>
+      <c r="AK152" s="7"/>
+      <c r="AL152" s="7"/>
+      <c r="AM152" s="7"/>
+    </row>
+    <row r="153" spans="2:39" ht="42.75">
+      <c r="B153" s="1"/>
+      <c r="C153" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D153" s="1"/>
+      <c r="E153" s="1"/>
+      <c r="F153" s="1"/>
+      <c r="G153" s="1"/>
+      <c r="H153" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="I153" s="1"/>
+      <c r="J153" s="1"/>
+      <c r="K153" s="1"/>
+      <c r="L153" s="1"/>
+      <c r="M153" s="1"/>
+      <c r="N153" s="1"/>
+      <c r="O153" s="7"/>
+      <c r="P153" s="7"/>
+      <c r="Q153" s="7"/>
+      <c r="R153" s="7"/>
+      <c r="S153" s="7"/>
+      <c r="T153" s="7"/>
+      <c r="U153" s="7"/>
+      <c r="V153" s="7"/>
+      <c r="W153" s="7"/>
+      <c r="X153" s="7"/>
+      <c r="Y153" s="7"/>
+      <c r="Z153" s="7"/>
+      <c r="AA153" s="7"/>
+      <c r="AB153" s="7"/>
+      <c r="AC153" s="7"/>
+      <c r="AD153" s="7"/>
+      <c r="AE153" s="7"/>
+      <c r="AF153" s="7"/>
+      <c r="AG153" s="7"/>
+      <c r="AH153" s="7"/>
+      <c r="AI153" s="7"/>
+      <c r="AJ153" s="7"/>
+      <c r="AK153" s="7"/>
+      <c r="AL153" s="7"/>
+      <c r="AM153" s="7"/>
+    </row>
+    <row r="154" spans="2:39" ht="28.5">
+      <c r="B154" s="1"/>
+      <c r="C154" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D154" s="1"/>
+      <c r="E154" s="1"/>
+      <c r="F154" s="1"/>
+      <c r="G154" s="1"/>
+      <c r="H154" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="I154" s="1"/>
+      <c r="J154" s="1"/>
+      <c r="K154" s="1"/>
+      <c r="L154" s="1"/>
+      <c r="M154" s="1"/>
+      <c r="N154" s="1"/>
+      <c r="O154" s="7"/>
+      <c r="P154" s="7"/>
+      <c r="Q154" s="7"/>
+      <c r="R154" s="7"/>
+      <c r="S154" s="7"/>
+      <c r="T154" s="7"/>
+      <c r="U154" s="7"/>
+      <c r="V154" s="7"/>
+      <c r="W154" s="7"/>
+      <c r="X154" s="7"/>
+      <c r="Y154" s="7"/>
+      <c r="Z154" s="7"/>
+      <c r="AA154" s="7"/>
+      <c r="AB154" s="7"/>
+      <c r="AC154" s="7"/>
+      <c r="AD154" s="7"/>
+      <c r="AE154" s="7"/>
+      <c r="AF154" s="7"/>
+      <c r="AG154" s="7"/>
+      <c r="AH154" s="7"/>
+      <c r="AI154" s="7"/>
+      <c r="AJ154" s="7"/>
+      <c r="AK154" s="7"/>
+      <c r="AL154" s="7"/>
+      <c r="AM154" s="7"/>
+    </row>
+    <row r="155" spans="2:39" ht="28.5">
+      <c r="B155" s="1"/>
+      <c r="C155" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D155" s="1"/>
+      <c r="E155" s="1"/>
+      <c r="F155" s="1"/>
+      <c r="G155" s="1"/>
+      <c r="H155" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="I155" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="J155" s="1"/>
+      <c r="K155" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L155" s="1"/>
+      <c r="M155" s="1"/>
+      <c r="N155" s="1"/>
+      <c r="O155" s="7"/>
+      <c r="P155" s="7"/>
+      <c r="Q155" s="7"/>
+      <c r="R155" s="7"/>
+      <c r="S155" s="7"/>
+      <c r="T155" s="7"/>
+      <c r="U155" s="7"/>
+      <c r="V155" s="7"/>
+      <c r="W155" s="7"/>
+      <c r="X155" s="7"/>
+      <c r="Y155" s="7"/>
+      <c r="Z155" s="7"/>
+      <c r="AA155" s="7"/>
+      <c r="AB155" s="7"/>
+      <c r="AC155" s="7"/>
+      <c r="AD155" s="7"/>
+      <c r="AE155" s="7"/>
+      <c r="AF155" s="7"/>
+      <c r="AG155" s="7"/>
+      <c r="AH155" s="7"/>
+      <c r="AI155" s="7"/>
+      <c r="AJ155" s="7"/>
+      <c r="AK155" s="7"/>
+      <c r="AL155" s="7"/>
+      <c r="AM155" s="7"/>
+    </row>
+    <row r="156" spans="2:39" ht="28.5">
+      <c r="B156" s="1"/>
+      <c r="C156" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D156" s="1"/>
+      <c r="E156" s="1"/>
+      <c r="F156" s="1"/>
+      <c r="G156" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H156" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="I156" s="1"/>
+      <c r="J156" s="1"/>
+      <c r="K156" s="1"/>
+      <c r="L156" s="1"/>
+      <c r="M156" s="1"/>
+      <c r="N156" s="1"/>
+      <c r="O156" s="7"/>
+      <c r="P156" s="7"/>
+      <c r="Q156" s="7"/>
+      <c r="R156" s="7"/>
+      <c r="S156" s="7"/>
+      <c r="T156" s="7"/>
+      <c r="U156" s="7"/>
+      <c r="V156" s="7"/>
+      <c r="W156" s="7"/>
+      <c r="X156" s="7"/>
+      <c r="Y156" s="7"/>
+      <c r="Z156" s="7"/>
+      <c r="AA156" s="7"/>
+      <c r="AB156" s="7"/>
+      <c r="AC156" s="7"/>
+      <c r="AD156" s="7"/>
+      <c r="AE156" s="7"/>
+      <c r="AF156" s="7"/>
+      <c r="AG156" s="7"/>
+      <c r="AH156" s="7"/>
+      <c r="AI156" s="7"/>
+      <c r="AJ156" s="7"/>
+      <c r="AK156" s="7"/>
+      <c r="AL156" s="7"/>
+      <c r="AM156" s="7"/>
+    </row>
+    <row r="157" spans="2:39">
+      <c r="B157" s="1"/>
+      <c r="C157" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D157" s="1"/>
+      <c r="E157" s="1"/>
+      <c r="F157" s="1"/>
+      <c r="G157" s="1"/>
+      <c r="H157" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="I157" s="1"/>
+      <c r="J157" s="1"/>
+      <c r="K157" s="1"/>
+      <c r="L157" s="1"/>
+      <c r="M157" s="1"/>
+      <c r="N157" s="1"/>
+      <c r="O157" s="7"/>
+      <c r="P157" s="7"/>
+      <c r="Q157" s="7"/>
+      <c r="R157" s="7"/>
+      <c r="S157" s="7"/>
+      <c r="T157" s="7"/>
+      <c r="U157" s="7"/>
+      <c r="V157" s="7"/>
+      <c r="W157" s="7"/>
+      <c r="X157" s="7"/>
+      <c r="Y157" s="7"/>
+      <c r="Z157" s="7"/>
+      <c r="AA157" s="7"/>
+      <c r="AB157" s="7"/>
+      <c r="AC157" s="7"/>
+      <c r="AD157" s="7"/>
+      <c r="AE157" s="7"/>
+      <c r="AF157" s="7"/>
+      <c r="AG157" s="7"/>
+      <c r="AH157" s="7"/>
+      <c r="AI157" s="7"/>
+      <c r="AJ157" s="7"/>
+      <c r="AK157" s="7"/>
+      <c r="AL157" s="7"/>
+      <c r="AM157" s="7"/>
+    </row>
+    <row r="158" spans="2:39" ht="28.5">
+      <c r="B158" s="1"/>
+      <c r="C158" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D158" s="1"/>
+      <c r="E158" s="1"/>
+      <c r="F158" s="1"/>
+      <c r="G158" s="1"/>
+      <c r="H158" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="I158" s="1"/>
+      <c r="J158" s="1"/>
+      <c r="K158" s="1"/>
+      <c r="L158" s="1"/>
+      <c r="M158" s="1"/>
+      <c r="N158" s="1"/>
+      <c r="O158" s="7"/>
+      <c r="P158" s="7"/>
+      <c r="Q158" s="7"/>
+      <c r="R158" s="7"/>
+      <c r="S158" s="7"/>
+      <c r="T158" s="7"/>
+      <c r="U158" s="7"/>
+      <c r="V158" s="7"/>
+      <c r="W158" s="7"/>
+      <c r="X158" s="7"/>
+      <c r="Y158" s="7"/>
+      <c r="Z158" s="7"/>
+      <c r="AA158" s="7"/>
+      <c r="AB158" s="7"/>
+      <c r="AC158" s="7"/>
+      <c r="AD158" s="7"/>
+      <c r="AE158" s="7"/>
+      <c r="AF158" s="7"/>
+      <c r="AG158" s="7"/>
+      <c r="AH158" s="7"/>
+      <c r="AI158" s="7"/>
+      <c r="AJ158" s="7"/>
+      <c r="AK158" s="7"/>
+      <c r="AL158" s="7"/>
+      <c r="AM158" s="7"/>
+    </row>
+    <row r="159" spans="2:39" ht="42.75">
+      <c r="B159" s="1"/>
+      <c r="C159" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D159" s="1"/>
+      <c r="E159" s="1"/>
+      <c r="F159" s="1"/>
+      <c r="G159" s="1"/>
+      <c r="H159" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="I159" s="1"/>
+      <c r="J159" s="1"/>
+      <c r="K159" s="1"/>
+      <c r="L159" s="1"/>
+      <c r="M159" s="1"/>
+      <c r="N159" s="1"/>
+      <c r="O159" s="7"/>
+      <c r="P159" s="7"/>
+      <c r="Q159" s="7"/>
+      <c r="R159" s="7"/>
+      <c r="S159" s="7"/>
+      <c r="T159" s="7"/>
+      <c r="U159" s="7"/>
+      <c r="V159" s="7"/>
+      <c r="W159" s="7"/>
+      <c r="X159" s="7"/>
+      <c r="Y159" s="7"/>
+      <c r="Z159" s="7"/>
+      <c r="AA159" s="7"/>
+      <c r="AB159" s="7"/>
+      <c r="AC159" s="7"/>
+      <c r="AD159" s="7"/>
+      <c r="AE159" s="7"/>
+      <c r="AF159" s="7"/>
+      <c r="AG159" s="7"/>
+      <c r="AH159" s="7"/>
+      <c r="AI159" s="7"/>
+      <c r="AJ159" s="7"/>
+      <c r="AK159" s="7"/>
+      <c r="AL159" s="7"/>
+      <c r="AM159" s="7"/>
+    </row>
+    <row r="160" spans="2:39" ht="42.75">
+      <c r="B160" s="1"/>
+      <c r="C160" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D160" s="1"/>
+      <c r="E160" s="1"/>
+      <c r="F160" s="1"/>
+      <c r="G160" s="1"/>
+      <c r="H160" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I160" s="1"/>
+      <c r="J160" s="1"/>
+      <c r="K160" s="1"/>
+      <c r="L160" s="1"/>
+      <c r="M160" s="1"/>
+      <c r="N160" s="1"/>
+      <c r="O160" s="7"/>
+      <c r="P160" s="7"/>
+      <c r="Q160" s="7"/>
+      <c r="R160" s="7"/>
+      <c r="S160" s="7"/>
+      <c r="T160" s="7"/>
+      <c r="U160" s="7"/>
+      <c r="V160" s="7"/>
+      <c r="W160" s="7"/>
+      <c r="X160" s="7"/>
+      <c r="Y160" s="7"/>
+      <c r="Z160" s="7"/>
+      <c r="AA160" s="7"/>
+      <c r="AB160" s="7"/>
+      <c r="AC160" s="7"/>
+      <c r="AD160" s="7"/>
+      <c r="AE160" s="7"/>
+      <c r="AF160" s="7"/>
+      <c r="AG160" s="7"/>
+      <c r="AH160" s="7"/>
+      <c r="AI160" s="7"/>
+      <c r="AJ160" s="7"/>
+      <c r="AK160" s="7"/>
+      <c r="AL160" s="7"/>
+      <c r="AM160" s="7"/>
+    </row>
+    <row r="161" spans="2:39" ht="42.75">
+      <c r="B161" s="1"/>
+      <c r="C161" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D161" s="1"/>
+      <c r="E161" s="1"/>
+      <c r="F161" s="1"/>
+      <c r="G161" s="1"/>
+      <c r="H161" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="I161" s="1"/>
+      <c r="J161" s="1"/>
+      <c r="K161" s="1"/>
+      <c r="L161" s="1"/>
+      <c r="M161" s="1"/>
+      <c r="N161" s="1"/>
+      <c r="O161" s="7"/>
+      <c r="P161" s="7"/>
+      <c r="Q161" s="7"/>
+      <c r="R161" s="7"/>
+      <c r="S161" s="7"/>
+      <c r="T161" s="7"/>
+      <c r="U161" s="7"/>
+      <c r="V161" s="7"/>
+      <c r="W161" s="7"/>
+      <c r="X161" s="7"/>
+      <c r="Y161" s="7"/>
+      <c r="Z161" s="7"/>
+      <c r="AA161" s="7"/>
+      <c r="AB161" s="7"/>
+      <c r="AC161" s="7"/>
+      <c r="AD161" s="7"/>
+      <c r="AE161" s="7"/>
+      <c r="AF161" s="7"/>
+      <c r="AG161" s="7"/>
+      <c r="AH161" s="7"/>
+      <c r="AI161" s="7"/>
+      <c r="AJ161" s="7"/>
+      <c r="AK161" s="7"/>
+      <c r="AL161" s="7"/>
+      <c r="AM161" s="7"/>
+    </row>
+    <row r="162" spans="2:39" ht="28.5">
+      <c r="B162" s="1"/>
+      <c r="C162" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D162" s="1"/>
+      <c r="E162" s="1"/>
+      <c r="F162" s="1"/>
+      <c r="G162" s="1"/>
+      <c r="H162" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="I162" s="1"/>
+      <c r="J162" s="1"/>
+      <c r="K162" s="1"/>
+      <c r="L162" s="1"/>
+      <c r="M162" s="1"/>
+      <c r="N162" s="1"/>
+      <c r="O162" s="7"/>
+      <c r="P162" s="7"/>
+      <c r="Q162" s="7"/>
+      <c r="R162" s="7"/>
+      <c r="S162" s="7"/>
+      <c r="T162" s="7"/>
+      <c r="U162" s="7"/>
+      <c r="V162" s="7"/>
+      <c r="W162" s="7"/>
+      <c r="X162" s="7"/>
+      <c r="Y162" s="7"/>
+      <c r="Z162" s="7"/>
+      <c r="AA162" s="7"/>
+      <c r="AB162" s="7"/>
+      <c r="AC162" s="7"/>
+      <c r="AD162" s="7"/>
+      <c r="AE162" s="7"/>
+      <c r="AF162" s="7"/>
+      <c r="AG162" s="7"/>
+      <c r="AH162" s="7"/>
+      <c r="AI162" s="7"/>
+      <c r="AJ162" s="7"/>
+      <c r="AK162" s="7"/>
+      <c r="AL162" s="7"/>
+      <c r="AM162" s="7"/>
+    </row>
+    <row r="163" spans="2:39" ht="28.5">
+      <c r="B163" s="1"/>
+      <c r="C163" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D163" s="1"/>
+      <c r="E163" s="1"/>
+      <c r="F163" s="1"/>
+      <c r="G163" s="1"/>
+      <c r="H163" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="I163" s="1"/>
+      <c r="J163" s="1"/>
+      <c r="K163" s="1"/>
+      <c r="L163" s="1"/>
+      <c r="M163" s="1"/>
+      <c r="N163" s="1"/>
+      <c r="O163" s="7"/>
+      <c r="P163" s="7"/>
+      <c r="Q163" s="7"/>
+      <c r="R163" s="7"/>
+      <c r="S163" s="7"/>
+      <c r="T163" s="7"/>
+      <c r="U163" s="7"/>
+      <c r="V163" s="7"/>
+      <c r="W163" s="7"/>
+      <c r="X163" s="7"/>
+      <c r="Y163" s="7"/>
+      <c r="Z163" s="7"/>
+      <c r="AA163" s="7"/>
+      <c r="AB163" s="7"/>
+      <c r="AC163" s="7"/>
+      <c r="AD163" s="7"/>
+      <c r="AE163" s="7"/>
+      <c r="AF163" s="7"/>
+      <c r="AG163" s="7"/>
+      <c r="AH163" s="7"/>
+      <c r="AI163" s="7"/>
+      <c r="AJ163" s="7"/>
+      <c r="AK163" s="7"/>
+      <c r="AL163" s="7"/>
+      <c r="AM163" s="7"/>
+    </row>
+    <row r="164" spans="2:39" ht="28.5">
+      <c r="B164" s="1"/>
+      <c r="C164" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D164" s="1"/>
+      <c r="E164" s="1"/>
+      <c r="F164" s="1"/>
+      <c r="G164" s="1"/>
+      <c r="H164" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="I164" s="1"/>
+      <c r="J164" s="1"/>
+      <c r="K164" s="1"/>
+      <c r="L164" s="1"/>
+      <c r="M164" s="1"/>
+      <c r="N164" s="1"/>
+      <c r="O164" s="7"/>
+      <c r="P164" s="7"/>
+      <c r="Q164" s="7"/>
+      <c r="R164" s="7"/>
+      <c r="S164" s="7"/>
+      <c r="T164" s="7"/>
+      <c r="U164" s="7"/>
+      <c r="V164" s="7"/>
+      <c r="W164" s="7"/>
+      <c r="X164" s="7"/>
+      <c r="Y164" s="7"/>
+      <c r="Z164" s="7"/>
+      <c r="AA164" s="7"/>
+      <c r="AB164" s="7"/>
+      <c r="AC164" s="7"/>
+      <c r="AD164" s="7"/>
+      <c r="AE164" s="7"/>
+      <c r="AF164" s="7"/>
+      <c r="AG164" s="7"/>
+      <c r="AH164" s="7"/>
+      <c r="AI164" s="7"/>
+      <c r="AJ164" s="7"/>
+      <c r="AK164" s="7"/>
+      <c r="AL164" s="7"/>
+      <c r="AM164" s="7"/>
+    </row>
+    <row r="165" spans="2:39">
+      <c r="B165" s="1"/>
+      <c r="C165" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D165" s="1"/>
+      <c r="E165" s="1"/>
+      <c r="F165" s="1"/>
+      <c r="G165" s="1"/>
+      <c r="H165" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="I165" s="1"/>
+      <c r="J165" s="1"/>
+      <c r="K165" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L165" s="1"/>
+      <c r="M165" s="1"/>
+      <c r="N165" s="1"/>
+      <c r="O165" s="7"/>
+      <c r="P165" s="7"/>
+      <c r="Q165" s="7"/>
+      <c r="R165" s="7"/>
+      <c r="S165" s="7"/>
+      <c r="T165" s="7"/>
+      <c r="U165" s="7"/>
+      <c r="V165" s="7"/>
+      <c r="W165" s="7"/>
+      <c r="X165" s="7"/>
+      <c r="Y165" s="7"/>
+      <c r="Z165" s="7"/>
+      <c r="AA165" s="7"/>
+      <c r="AB165" s="7"/>
+      <c r="AC165" s="7"/>
+      <c r="AD165" s="7"/>
+      <c r="AE165" s="7"/>
+      <c r="AF165" s="7"/>
+      <c r="AG165" s="7"/>
+      <c r="AH165" s="7"/>
+      <c r="AI165" s="7"/>
+      <c r="AJ165" s="7"/>
+      <c r="AK165" s="7"/>
+      <c r="AL165" s="7"/>
+      <c r="AM165" s="7"/>
+    </row>
+    <row r="166" spans="2:39">
+      <c r="B166" s="1"/>
+      <c r="C166" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D166" s="1"/>
+      <c r="E166" s="1"/>
+      <c r="F166" s="1"/>
+      <c r="G166" s="1"/>
+      <c r="H166" s="8"/>
+      <c r="I166" s="1"/>
+      <c r="J166" s="1"/>
+      <c r="K166" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L166" s="1"/>
+      <c r="M166" s="1"/>
+      <c r="N166" s="1"/>
+      <c r="O166" s="7"/>
+      <c r="P166" s="7"/>
+      <c r="Q166" s="7"/>
+      <c r="R166" s="7"/>
+      <c r="S166" s="7"/>
+      <c r="T166" s="7"/>
+      <c r="U166" s="7"/>
+      <c r="V166" s="7"/>
+      <c r="W166" s="7"/>
+      <c r="X166" s="7"/>
+      <c r="Y166" s="7"/>
+      <c r="Z166" s="7"/>
+      <c r="AA166" s="7"/>
+      <c r="AB166" s="7"/>
+      <c r="AC166" s="7"/>
+      <c r="AD166" s="7"/>
+      <c r="AE166" s="7"/>
+      <c r="AF166" s="7"/>
+      <c r="AG166" s="7"/>
+      <c r="AH166" s="7"/>
+      <c r="AI166" s="7"/>
+      <c r="AJ166" s="7"/>
+      <c r="AK166" s="7"/>
+      <c r="AL166" s="7"/>
+      <c r="AM166" s="7"/>
+    </row>
+    <row r="167" spans="2:39">
+      <c r="B167" s="1"/>
+      <c r="C167" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D167" s="1"/>
+      <c r="E167" s="1"/>
+      <c r="F167" s="1"/>
+      <c r="G167" s="1"/>
+      <c r="H167" s="8"/>
+      <c r="I167" s="1"/>
+      <c r="J167" s="1"/>
+      <c r="K167" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L167" s="1"/>
+      <c r="M167" s="1"/>
+      <c r="N167" s="1"/>
+      <c r="O167" s="7"/>
+      <c r="P167" s="7"/>
+      <c r="Q167" s="7"/>
+      <c r="R167" s="7"/>
+      <c r="S167" s="7"/>
+      <c r="T167" s="7"/>
+      <c r="U167" s="7"/>
+      <c r="V167" s="7"/>
+      <c r="W167" s="7"/>
+      <c r="X167" s="7"/>
+      <c r="Y167" s="7"/>
+      <c r="Z167" s="7"/>
+      <c r="AA167" s="7"/>
+      <c r="AB167" s="7"/>
+      <c r="AC167" s="7"/>
+      <c r="AD167" s="7"/>
+      <c r="AE167" s="7"/>
+      <c r="AF167" s="7"/>
+      <c r="AG167" s="7"/>
+      <c r="AH167" s="7"/>
+      <c r="AI167" s="7"/>
+      <c r="AJ167" s="7"/>
+      <c r="AK167" s="7"/>
+      <c r="AL167" s="7"/>
+      <c r="AM167" s="7"/>
+    </row>
+    <row r="168" spans="2:39">
+      <c r="B168" s="1"/>
+      <c r="C168" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D168" s="1"/>
+      <c r="E168" s="1"/>
+      <c r="F168" s="1"/>
+      <c r="G168" s="1"/>
+      <c r="H168" s="8"/>
+      <c r="I168" s="1"/>
+      <c r="J168" s="1"/>
+      <c r="K168" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L168" s="1"/>
+      <c r="M168" s="1"/>
+      <c r="N168" s="1"/>
+      <c r="O168" s="7"/>
+      <c r="P168" s="7"/>
+      <c r="Q168" s="7"/>
+      <c r="R168" s="7"/>
+      <c r="S168" s="7"/>
+      <c r="T168" s="7"/>
+      <c r="U168" s="7"/>
+      <c r="V168" s="7"/>
+      <c r="W168" s="7"/>
+      <c r="X168" s="7"/>
+      <c r="Y168" s="7"/>
+      <c r="Z168" s="7"/>
+      <c r="AA168" s="7"/>
+      <c r="AB168" s="7"/>
+      <c r="AC168" s="7"/>
+      <c r="AD168" s="7"/>
+      <c r="AE168" s="7"/>
+      <c r="AF168" s="7"/>
+      <c r="AG168" s="7"/>
+      <c r="AH168" s="7"/>
+      <c r="AI168" s="7"/>
+      <c r="AJ168" s="7"/>
+      <c r="AK168" s="7"/>
+      <c r="AL168" s="7"/>
+      <c r="AM168" s="7"/>
+    </row>
+    <row r="169" spans="2:39">
+      <c r="B169" s="1"/>
+      <c r="C169" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D169" s="1"/>
+      <c r="E169" s="1"/>
+      <c r="F169" s="1"/>
+      <c r="G169" s="1"/>
+      <c r="H169" s="8"/>
+      <c r="I169" s="1"/>
+      <c r="J169" s="1"/>
+      <c r="K169" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L169" s="1"/>
+      <c r="M169" s="1"/>
+      <c r="N169" s="1"/>
+      <c r="O169" s="7"/>
+      <c r="P169" s="7"/>
+      <c r="Q169" s="7"/>
+      <c r="R169" s="7"/>
+      <c r="S169" s="7"/>
+      <c r="T169" s="7"/>
+      <c r="U169" s="7"/>
+      <c r="V169" s="7"/>
+      <c r="W169" s="7"/>
+      <c r="X169" s="7"/>
+      <c r="Y169" s="7"/>
+      <c r="Z169" s="7"/>
+      <c r="AA169" s="7"/>
+      <c r="AB169" s="7"/>
+      <c r="AC169" s="7"/>
+      <c r="AD169" s="7"/>
+      <c r="AE169" s="7"/>
+      <c r="AF169" s="7"/>
+      <c r="AG169" s="7"/>
+      <c r="AH169" s="7"/>
+      <c r="AI169" s="7"/>
+      <c r="AJ169" s="7"/>
+      <c r="AK169" s="7"/>
+      <c r="AL169" s="7"/>
+      <c r="AM169" s="7"/>
+    </row>
+    <row r="170" spans="2:39">
+      <c r="B170" s="1"/>
+      <c r="C170" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D170" s="1"/>
+      <c r="E170" s="1"/>
+      <c r="F170" s="1"/>
+      <c r="G170" s="1"/>
+      <c r="H170" s="8"/>
+      <c r="I170" s="1"/>
+      <c r="J170" s="1"/>
+      <c r="K170" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L170" s="1"/>
+      <c r="M170" s="1"/>
+      <c r="N170" s="1"/>
+      <c r="O170" s="7"/>
+      <c r="P170" s="7"/>
+      <c r="Q170" s="7"/>
+      <c r="R170" s="7"/>
+      <c r="S170" s="7"/>
+      <c r="T170" s="7"/>
+      <c r="U170" s="7"/>
+      <c r="V170" s="7"/>
+      <c r="W170" s="7"/>
+      <c r="X170" s="7"/>
+      <c r="Y170" s="7"/>
+      <c r="Z170" s="7"/>
+      <c r="AA170" s="7"/>
+      <c r="AB170" s="7"/>
+      <c r="AC170" s="7"/>
+      <c r="AD170" s="7"/>
+      <c r="AE170" s="7"/>
+      <c r="AF170" s="7"/>
+      <c r="AG170" s="7"/>
+      <c r="AH170" s="7"/>
+      <c r="AI170" s="7"/>
+      <c r="AJ170" s="7"/>
+      <c r="AK170" s="7"/>
+      <c r="AL170" s="7"/>
+      <c r="AM170" s="7"/>
+    </row>
+    <row r="171" spans="2:39">
+      <c r="B171" s="1"/>
+      <c r="C171" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D171" s="1"/>
+      <c r="E171" s="1"/>
+      <c r="F171" s="1"/>
+      <c r="G171" s="1"/>
+      <c r="H171" s="8"/>
+      <c r="I171" s="1"/>
+      <c r="J171" s="1"/>
+      <c r="K171" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L171" s="1"/>
+      <c r="M171" s="1"/>
+      <c r="N171" s="1"/>
+      <c r="O171" s="7"/>
+      <c r="P171" s="7"/>
+      <c r="Q171" s="7"/>
+      <c r="R171" s="7"/>
+      <c r="S171" s="7"/>
+      <c r="T171" s="7"/>
+      <c r="U171" s="7"/>
+      <c r="V171" s="7"/>
+      <c r="W171" s="7"/>
+      <c r="X171" s="7"/>
+      <c r="Y171" s="7"/>
+      <c r="Z171" s="7"/>
+      <c r="AA171" s="7"/>
+      <c r="AB171" s="7"/>
+      <c r="AC171" s="7"/>
+      <c r="AD171" s="7"/>
+      <c r="AE171" s="7"/>
+      <c r="AF171" s="7"/>
+      <c r="AG171" s="7"/>
+      <c r="AH171" s="7"/>
+      <c r="AI171" s="7"/>
+      <c r="AJ171" s="7"/>
+      <c r="AK171" s="7"/>
+      <c r="AL171" s="7"/>
+      <c r="AM171" s="7"/>
+    </row>
+    <row r="172" spans="2:39">
+      <c r="B172" s="1"/>
+      <c r="C172" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D172" s="1"/>
+      <c r="E172" s="1"/>
+      <c r="F172" s="1"/>
+      <c r="G172" s="1"/>
+      <c r="H172" s="8"/>
+      <c r="I172" s="1"/>
+      <c r="J172" s="1"/>
+      <c r="K172" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L172" s="1"/>
+      <c r="M172" s="1"/>
+      <c r="N172" s="1"/>
+      <c r="O172" s="7"/>
+      <c r="P172" s="7"/>
+      <c r="Q172" s="7"/>
+      <c r="R172" s="7"/>
+      <c r="S172" s="7"/>
+      <c r="T172" s="7"/>
+      <c r="U172" s="7"/>
+      <c r="V172" s="7"/>
+      <c r="W172" s="7"/>
+      <c r="X172" s="7"/>
+      <c r="Y172" s="7"/>
+      <c r="Z172" s="7"/>
+      <c r="AA172" s="7"/>
+      <c r="AB172" s="7"/>
+      <c r="AC172" s="7"/>
+      <c r="AD172" s="7"/>
+      <c r="AE172" s="7"/>
+      <c r="AF172" s="7"/>
+      <c r="AG172" s="7"/>
+      <c r="AH172" s="7"/>
+      <c r="AI172" s="7"/>
+      <c r="AJ172" s="7"/>
+      <c r="AK172" s="7"/>
+      <c r="AL172" s="7"/>
+      <c r="AM172" s="7"/>
+    </row>
+    <row r="173" spans="2:39">
+      <c r="B173" s="1"/>
+      <c r="C173" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D173" s="1"/>
+      <c r="E173" s="1"/>
+      <c r="F173" s="1"/>
+      <c r="G173" s="1"/>
+      <c r="H173" s="8"/>
+      <c r="I173" s="1"/>
+      <c r="J173" s="1"/>
+      <c r="K173" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L173" s="1"/>
+      <c r="M173" s="1"/>
+      <c r="N173" s="1"/>
+      <c r="O173" s="7"/>
+      <c r="P173" s="7"/>
+      <c r="Q173" s="7"/>
+      <c r="R173" s="7"/>
+      <c r="S173" s="7"/>
+      <c r="T173" s="7"/>
+      <c r="U173" s="7"/>
+      <c r="V173" s="7"/>
+      <c r="W173" s="7"/>
+      <c r="X173" s="7"/>
+      <c r="Y173" s="7"/>
+      <c r="Z173" s="7"/>
+      <c r="AA173" s="7"/>
+      <c r="AB173" s="7"/>
+      <c r="AC173" s="7"/>
+      <c r="AD173" s="7"/>
+      <c r="AE173" s="7"/>
+      <c r="AF173" s="7"/>
+      <c r="AG173" s="7"/>
+      <c r="AH173" s="7"/>
+      <c r="AI173" s="7"/>
+      <c r="AJ173" s="7"/>
+      <c r="AK173" s="7"/>
+      <c r="AL173" s="7"/>
+      <c r="AM173" s="7"/>
+    </row>
+    <row r="174" spans="2:39">
+      <c r="B174" s="1"/>
+      <c r="C174" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D174" s="1"/>
+      <c r="E174" s="1"/>
+      <c r="F174" s="1"/>
+      <c r="G174" s="1"/>
+      <c r="H174" s="8"/>
+      <c r="I174" s="1"/>
+      <c r="J174" s="1"/>
+      <c r="K174" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L174" s="1"/>
+      <c r="M174" s="1"/>
+      <c r="N174" s="1"/>
+      <c r="O174" s="7"/>
+      <c r="P174" s="7"/>
+      <c r="Q174" s="7"/>
+      <c r="R174" s="7"/>
+      <c r="S174" s="7"/>
+      <c r="T174" s="7"/>
+      <c r="U174" s="7"/>
+      <c r="V174" s="7"/>
+      <c r="W174" s="7"/>
+      <c r="X174" s="7"/>
+      <c r="Y174" s="7"/>
+      <c r="Z174" s="7"/>
+      <c r="AA174" s="7"/>
+      <c r="AB174" s="7"/>
+      <c r="AC174" s="7"/>
+      <c r="AD174" s="7"/>
+      <c r="AE174" s="7"/>
+      <c r="AF174" s="7"/>
+      <c r="AG174" s="7"/>
+      <c r="AH174" s="7"/>
+      <c r="AI174" s="7"/>
+      <c r="AJ174" s="7"/>
+      <c r="AK174" s="7"/>
+      <c r="AL174" s="7"/>
+      <c r="AM174" s="7"/>
+    </row>
+    <row r="175" spans="2:39">
+      <c r="B175" s="1"/>
+      <c r="C175" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D175" s="1"/>
+      <c r="E175" s="1"/>
+      <c r="F175" s="1"/>
+      <c r="G175" s="1"/>
+      <c r="H175" s="8"/>
+      <c r="I175" s="1"/>
+      <c r="J175" s="1"/>
+      <c r="K175" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L175" s="1"/>
+      <c r="M175" s="1"/>
+      <c r="N175" s="1"/>
+      <c r="O175" s="7"/>
+      <c r="P175" s="7"/>
+      <c r="Q175" s="7"/>
+      <c r="R175" s="7"/>
+      <c r="S175" s="7"/>
+      <c r="T175" s="7"/>
+      <c r="U175" s="7"/>
+      <c r="V175" s="7"/>
+      <c r="W175" s="7"/>
+      <c r="X175" s="7"/>
+      <c r="Y175" s="7"/>
+      <c r="Z175" s="7"/>
+      <c r="AA175" s="7"/>
+      <c r="AB175" s="7"/>
+      <c r="AC175" s="7"/>
+      <c r="AD175" s="7"/>
+      <c r="AE175" s="7"/>
+      <c r="AF175" s="7"/>
+      <c r="AG175" s="7"/>
+      <c r="AH175" s="7"/>
+      <c r="AI175" s="7"/>
+      <c r="AJ175" s="7"/>
+      <c r="AK175" s="7"/>
+      <c r="AL175" s="7"/>
+      <c r="AM175" s="7"/>
+    </row>
+    <row r="176" spans="2:39">
+      <c r="B176" s="1"/>
+      <c r="C176" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D176" s="1"/>
+      <c r="E176" s="1"/>
+      <c r="F176" s="1"/>
+      <c r="G176" s="1"/>
+      <c r="H176" s="8"/>
+      <c r="I176" s="1"/>
+      <c r="J176" s="1"/>
+      <c r="K176" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L176" s="1"/>
+      <c r="M176" s="1"/>
+      <c r="N176" s="1"/>
+      <c r="O176" s="7"/>
+      <c r="P176" s="7"/>
+      <c r="Q176" s="7"/>
+      <c r="R176" s="7"/>
+      <c r="S176" s="7"/>
+      <c r="T176" s="7"/>
+      <c r="U176" s="7"/>
+      <c r="V176" s="7"/>
+      <c r="W176" s="7"/>
+      <c r="X176" s="7"/>
+      <c r="Y176" s="7"/>
+      <c r="Z176" s="7"/>
+      <c r="AA176" s="7"/>
+      <c r="AB176" s="7"/>
+      <c r="AC176" s="7"/>
+      <c r="AD176" s="7"/>
+      <c r="AE176" s="7"/>
+      <c r="AF176" s="7"/>
+      <c r="AG176" s="7"/>
+      <c r="AH176" s="7"/>
+      <c r="AI176" s="7"/>
+      <c r="AJ176" s="7"/>
+      <c r="AK176" s="7"/>
+      <c r="AL176" s="7"/>
+      <c r="AM176" s="7"/>
+    </row>
+    <row r="177" spans="2:39">
+      <c r="B177" s="1"/>
+      <c r="C177" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D177" s="1"/>
+      <c r="E177" s="1"/>
+      <c r="F177" s="1"/>
+      <c r="G177" s="1"/>
+      <c r="H177" s="8"/>
+      <c r="I177" s="1"/>
+      <c r="J177" s="1"/>
+      <c r="K177" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L177" s="1"/>
+      <c r="M177" s="1"/>
+      <c r="N177" s="1"/>
+      <c r="O177" s="7"/>
+      <c r="P177" s="7"/>
+      <c r="Q177" s="7"/>
+      <c r="R177" s="7"/>
+      <c r="S177" s="7"/>
+      <c r="T177" s="7"/>
+      <c r="U177" s="7"/>
+      <c r="V177" s="7"/>
+      <c r="W177" s="7"/>
+      <c r="X177" s="7"/>
+      <c r="Y177" s="7"/>
+      <c r="Z177" s="7"/>
+      <c r="AA177" s="7"/>
+      <c r="AB177" s="7"/>
+      <c r="AC177" s="7"/>
+      <c r="AD177" s="7"/>
+      <c r="AE177" s="7"/>
+      <c r="AF177" s="7"/>
+      <c r="AG177" s="7"/>
+      <c r="AH177" s="7"/>
+      <c r="AI177" s="7"/>
+      <c r="AJ177" s="7"/>
+      <c r="AK177" s="7"/>
+      <c r="AL177" s="7"/>
+      <c r="AM177" s="7"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="E6:E132">
-    <cfRule type="containsBlanks" dxfId="3" priority="1">
+  <conditionalFormatting sqref="E6:E177">
+    <cfRule type="containsBlanks" dxfId="7" priority="1">
       <formula>LEN(TRIM(E6))=0</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="x">
+    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",E6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F132">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+  <conditionalFormatting sqref="F6:F177">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>"ISBLANK"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D132 J6:J132" xr:uid="{CD5956F3-4E0A-44DB-A8DC-925168F89EE9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6 M8:M131 AH6:AH177 AA6:AA177 T6:T177" xr:uid="{F01B3C1A-78E2-4F4D-B484-DA9ABA464973}">
+      <formula1>INDIRECT("ConditionalsList[Conditionals]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J6:J177 D6:D177" xr:uid="{CD5956F3-4E0A-44DB-A8DC-925168F89EE9}">
       <formula1>INDIRECT("ExpressionsList[Expressions]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T132 AA6:AA132 AH6:AH132 M6 M8:M20" xr:uid="{F01B3C1A-78E2-4F4D-B484-DA9ABA464973}">
-      <formula1>INDIRECT("ConditionalsList[Conditionals]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C132 K6:K132" xr:uid="{3FFEAF7F-218C-4ED0-9224-5256A4750AA6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C177 K6:K177" xr:uid="{3FFEAF7F-218C-4ED0-9224-5256A4750AA6}">
       <formula1>INDIRECT("CharactersList[Characters]")</formula1>
     </dataValidation>
   </dataValidations>
@@ -8682,14 +10952,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EDBD295-5C93-44DD-9985-3C1BB495EB4B}">
   <dimension ref="B2:F11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.25" customWidth="1"/>
+    <col min="4" max="4" width="14.125" customWidth="1"/>
+    <col min="6" max="6" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -8700,7 +10970,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6">
       <c r="B3" t="s">
         <v>16</v>
       </c>
@@ -8711,7 +10981,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -8722,7 +10992,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6">
       <c r="B5" t="s">
         <v>41</v>
       </c>
@@ -8733,7 +11003,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6">
       <c r="B6" t="s">
         <v>20</v>
       </c>
@@ -8741,7 +11011,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6">
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -8749,7 +11019,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6">
       <c r="B8" t="s">
         <v>18</v>
       </c>
@@ -8757,7 +11027,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6">
       <c r="B9" t="s">
         <v>19</v>
       </c>
@@ -8765,12 +11035,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6">
       <c r="B10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6">
       <c r="B11" t="s">
         <v>17</v>
       </c>

</xml_diff>